<commit_message>
Reduced by 127 bytes IL code for linked matrix solving
</commit_message>
<xml_diff>
--- a/ILSIze.xlsx
+++ b/ILSIze.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7284AE1E-FD30-B542-A046-A6639A12F59E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC38C4D5-DD3C-214B-9F7B-D5861CD11201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35280" yWindow="-860" windowWidth="25440" windowHeight="14400" activeTab="4" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
+    <workbookView xWindow="10220" yWindow="4440" windowWidth="25600" windowHeight="16000" activeTab="5" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
   </bookViews>
   <sheets>
     <sheet name="Chemistry.cs" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="void OutputEnzymeKinematic" sheetId="3" r:id="rId3"/>
     <sheet name="LinearRegression.cs" sheetId="4" r:id="rId4"/>
     <sheet name="Student" sheetId="5" r:id="rId5"/>
+    <sheet name="Matrix.cs" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="76">
   <si>
     <t>Méthode</t>
   </si>
@@ -235,6 +236,39 @@
   </si>
   <si>
     <t>TryMultiply</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Stack</t>
+  </si>
+  <si>
+    <t>Locals</t>
+  </si>
+  <si>
+    <t>Methods</t>
+  </si>
+  <si>
+    <t>Iteration 1</t>
+  </si>
+  <si>
+    <t>SolveDiagonally</t>
+  </si>
+  <si>
+    <t>SolveLinkedLine</t>
+  </si>
+  <si>
+    <t>Iteration 2</t>
+  </si>
+  <si>
+    <t>Iteration 3</t>
+  </si>
+  <si>
+    <t>Iteration 4</t>
+  </si>
+  <si>
+    <t>Iteration 5</t>
   </si>
 </sst>
 </file>
@@ -298,10 +332,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -650,16 +684,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3" t="s">
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -1214,31 +1248,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3" t="s">
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3" t="s">
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3" t="s">
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3" t="s">
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="3"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -1621,16 +1655,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3" t="s">
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -1952,7 +1986,7 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E20" s="4">
+      <c r="E20" s="3">
         <f>E19/B18</f>
         <v>-0.47355163727959698</v>
       </c>
@@ -1964,4 +1998,290 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3446A6D4-E7A1-DE4F-AF79-3C1286851385}">
+  <dimension ref="A1:P7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B1" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I2" t="s">
+        <v>66</v>
+      </c>
+      <c r="J2" t="s">
+        <v>67</v>
+      </c>
+      <c r="K2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L2" t="s">
+        <v>66</v>
+      </c>
+      <c r="M2" t="s">
+        <v>67</v>
+      </c>
+      <c r="N2" t="s">
+        <v>65</v>
+      </c>
+      <c r="O2" t="s">
+        <v>66</v>
+      </c>
+      <c r="P2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3">
+        <v>700</v>
+      </c>
+      <c r="C3">
+        <v>7</v>
+      </c>
+      <c r="D3">
+        <v>16</v>
+      </c>
+      <c r="E3">
+        <v>675</v>
+      </c>
+      <c r="F3">
+        <v>7</v>
+      </c>
+      <c r="G3">
+        <v>13</v>
+      </c>
+      <c r="H3">
+        <v>665</v>
+      </c>
+      <c r="I3">
+        <v>7</v>
+      </c>
+      <c r="J3">
+        <v>11</v>
+      </c>
+      <c r="K3">
+        <v>628</v>
+      </c>
+      <c r="L3">
+        <v>7</v>
+      </c>
+      <c r="M3">
+        <v>10</v>
+      </c>
+      <c r="N3">
+        <v>620</v>
+      </c>
+      <c r="O3">
+        <v>7</v>
+      </c>
+      <c r="P3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4">
+        <v>291</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4">
+        <v>10</v>
+      </c>
+      <c r="E4">
+        <v>288</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>9</v>
+      </c>
+      <c r="H4">
+        <v>252</v>
+      </c>
+      <c r="I4">
+        <v>4</v>
+      </c>
+      <c r="J4">
+        <v>7</v>
+      </c>
+      <c r="K4">
+        <v>244</v>
+      </c>
+      <c r="L4">
+        <v>4</v>
+      </c>
+      <c r="M4">
+        <v>7</v>
+      </c>
+      <c r="N4">
+        <v>244</v>
+      </c>
+      <c r="O4">
+        <v>4</v>
+      </c>
+      <c r="P4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B5" s="1">
+        <f>SUM(B3:B4)</f>
+        <v>991</v>
+      </c>
+      <c r="C5" s="1">
+        <f>SUM(C3:C4)</f>
+        <v>11</v>
+      </c>
+      <c r="D5" s="1">
+        <f>SUM(D3:D4)</f>
+        <v>26</v>
+      </c>
+      <c r="E5" s="1">
+        <f>SUM(E3:E4)</f>
+        <v>963</v>
+      </c>
+      <c r="F5" s="1">
+        <f>SUM(F3:F4)</f>
+        <v>11</v>
+      </c>
+      <c r="G5" s="1">
+        <f>SUM(G3:G4)</f>
+        <v>22</v>
+      </c>
+      <c r="H5" s="1">
+        <f t="shared" ref="H5:J5" si="0">SUM(H3:H4)</f>
+        <v>917</v>
+      </c>
+      <c r="I5" s="1">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="J5" s="1">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="K5" s="1">
+        <f t="shared" ref="K5" si="1">SUM(K3:K4)</f>
+        <v>872</v>
+      </c>
+      <c r="L5" s="1">
+        <f t="shared" ref="L5" si="2">SUM(L3:L4)</f>
+        <v>11</v>
+      </c>
+      <c r="M5" s="1">
+        <f t="shared" ref="M5" si="3">SUM(M3:M4)</f>
+        <v>17</v>
+      </c>
+      <c r="N5" s="1">
+        <f t="shared" ref="N5" si="4">SUM(N3:N4)</f>
+        <v>864</v>
+      </c>
+      <c r="O5" s="1">
+        <f t="shared" ref="O5" si="5">SUM(O3:O4)</f>
+        <v>11</v>
+      </c>
+      <c r="P5" s="1">
+        <f t="shared" ref="P5" si="6">SUM(P3:P4)</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="N6">
+        <f>N5-B5</f>
+        <v>-127</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="N7" s="3">
+        <f>N6/B5</f>
+        <v>-0.12815338042381433</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="E1:G1"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="N1:P1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added mathematical functions operating on Decimal
But most of them are woefully inaccurate
</commit_message>
<xml_diff>
--- a/ILSIze.xlsx
+++ b/ILSIze.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC38C4D5-DD3C-214B-9F7B-D5861CD11201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87274557-5504-4948-B40A-52E010EFEB22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10220" yWindow="4440" windowWidth="25600" windowHeight="16000" activeTab="5" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
+    <workbookView xWindow="35000" yWindow="-2540" windowWidth="24960" windowHeight="15900" activeTab="6" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
   </bookViews>
   <sheets>
     <sheet name="Chemistry.cs" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="LinearRegression.cs" sheetId="4" r:id="rId4"/>
     <sheet name="Student" sheetId="5" r:id="rId5"/>
     <sheet name="Matrix.cs" sheetId="6" r:id="rId6"/>
+    <sheet name="ExtraMath_decimal.cs" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="97">
   <si>
     <t>Méthode</t>
   </si>
@@ -269,6 +270,69 @@
   </si>
   <si>
     <t>Iteration 5</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Iteration 0</t>
+  </si>
+  <si>
+    <t>Exp</t>
+  </si>
+  <si>
+    <t>Pow(decimal, decimal)</t>
+  </si>
+  <si>
+    <t>Pow(decimal, int)</t>
+  </si>
+  <si>
+    <t>IsInteger</t>
+  </si>
+  <si>
+    <t>Log</t>
+  </si>
+  <si>
+    <t>Log10</t>
+  </si>
+  <si>
+    <t>Cos</t>
+  </si>
+  <si>
+    <t>Tan</t>
+  </si>
+  <si>
+    <t>CalculateSinFromCos</t>
+  </si>
+  <si>
+    <t>Sin</t>
+  </si>
+  <si>
+    <t>TruncateToPeriodicInterval</t>
+  </si>
+  <si>
+    <t>IsSignOfSinePositive</t>
+  </si>
+  <si>
+    <t>Sinh</t>
+  </si>
+  <si>
+    <t>Cosh</t>
+  </si>
+  <si>
+    <t>Tanh</t>
+  </si>
+  <si>
+    <t>Asin</t>
+  </si>
+  <si>
+    <t>Atan</t>
+  </si>
+  <si>
+    <t>Acos</t>
+  </si>
+  <si>
+    <t>Atan2</t>
   </si>
 </sst>
 </file>
@@ -328,7 +392,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -336,6 +400,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2202,63 +2270,63 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B5" s="1">
-        <f>SUM(B3:B4)</f>
+        <f t="shared" ref="B5:G5" si="0">SUM(B3:B4)</f>
         <v>991</v>
       </c>
       <c r="C5" s="1">
-        <f>SUM(C3:C4)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="D5" s="1">
-        <f>SUM(D3:D4)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="E5" s="1">
-        <f>SUM(E3:E4)</f>
+        <f t="shared" si="0"/>
         <v>963</v>
       </c>
       <c r="F5" s="1">
-        <f>SUM(F3:F4)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="G5" s="1">
-        <f>SUM(G3:G4)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="H5" s="1">
-        <f t="shared" ref="H5:J5" si="0">SUM(H3:H4)</f>
+        <f t="shared" ref="H5:J5" si="1">SUM(H3:H4)</f>
         <v>917</v>
       </c>
       <c r="I5" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="J5" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="K5" s="1">
-        <f t="shared" ref="K5" si="1">SUM(K3:K4)</f>
+        <f t="shared" ref="K5" si="2">SUM(K3:K4)</f>
         <v>872</v>
       </c>
       <c r="L5" s="1">
-        <f t="shared" ref="L5" si="2">SUM(L3:L4)</f>
+        <f t="shared" ref="L5" si="3">SUM(L3:L4)</f>
         <v>11</v>
       </c>
       <c r="M5" s="1">
-        <f t="shared" ref="M5" si="3">SUM(M3:M4)</f>
+        <f t="shared" ref="M5" si="4">SUM(M3:M4)</f>
         <v>17</v>
       </c>
       <c r="N5" s="1">
-        <f t="shared" ref="N5" si="4">SUM(N3:N4)</f>
+        <f t="shared" ref="N5" si="5">SUM(N3:N4)</f>
         <v>864</v>
       </c>
       <c r="O5" s="1">
-        <f t="shared" ref="O5" si="5">SUM(O3:O4)</f>
+        <f t="shared" ref="O5" si="6">SUM(O3:O4)</f>
         <v>11</v>
       </c>
       <c r="P5" s="1">
-        <f t="shared" ref="P5" si="6">SUM(P3:P4)</f>
+        <f t="shared" ref="P5" si="7">SUM(P3:P4)</f>
         <v>18</v>
       </c>
     </row>
@@ -2284,4 +2352,793 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2043A2D3-B79F-994A-8E5F-6CAF0A113206}">
+  <dimension ref="A1:M22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A1" s="1"/>
+      <c r="B1" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3">
+        <v>199</v>
+      </c>
+      <c r="C3">
+        <v>6</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3">
+        <v>188</v>
+      </c>
+      <c r="F3">
+        <v>6</v>
+      </c>
+      <c r="G3">
+        <v>6</v>
+      </c>
+      <c r="H3">
+        <v>188</v>
+      </c>
+      <c r="I3">
+        <v>6</v>
+      </c>
+      <c r="J3">
+        <v>6</v>
+      </c>
+      <c r="K3">
+        <v>188</v>
+      </c>
+      <c r="L3">
+        <v>6</v>
+      </c>
+      <c r="M3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4">
+        <v>292</v>
+      </c>
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>243</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
+      <c r="H4">
+        <v>265</v>
+      </c>
+      <c r="I4">
+        <v>3</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <v>265</v>
+      </c>
+      <c r="L4">
+        <v>3</v>
+      </c>
+      <c r="M4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5">
+        <v>31</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>29</v>
+      </c>
+      <c r="F5">
+        <v>8</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6">
+        <v>109</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6">
+        <v>103</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>103</v>
+      </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B7">
+        <v>35</v>
+      </c>
+      <c r="C7">
+        <v>8</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>35</v>
+      </c>
+      <c r="F7">
+        <v>8</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>35</v>
+      </c>
+      <c r="I7">
+        <v>8</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A8" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8">
+        <v>270</v>
+      </c>
+      <c r="C8">
+        <v>6</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>257</v>
+      </c>
+      <c r="F8">
+        <v>6</v>
+      </c>
+      <c r="G8">
+        <v>8</v>
+      </c>
+      <c r="H8">
+        <v>257</v>
+      </c>
+      <c r="I8">
+        <v>6</v>
+      </c>
+      <c r="J8">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9">
+        <v>350</v>
+      </c>
+      <c r="C9">
+        <v>6</v>
+      </c>
+      <c r="D9">
+        <v>5</v>
+      </c>
+      <c r="E9">
+        <v>308</v>
+      </c>
+      <c r="F9">
+        <v>6</v>
+      </c>
+      <c r="G9">
+        <v>6</v>
+      </c>
+      <c r="H9">
+        <v>308</v>
+      </c>
+      <c r="I9">
+        <v>6</v>
+      </c>
+      <c r="J9">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10">
+        <v>45</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>56</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>56</v>
+      </c>
+      <c r="I10">
+        <v>3</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11">
+        <v>40</v>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>40</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>145</v>
+      </c>
+      <c r="I11">
+        <v>6</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B12">
+        <v>15</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>13</v>
+      </c>
+      <c r="F12">
+        <v>8</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>13</v>
+      </c>
+      <c r="I12">
+        <v>8</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A13" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B13">
+        <v>275</v>
+      </c>
+      <c r="C13">
+        <v>8</v>
+      </c>
+      <c r="D13">
+        <v>2</v>
+      </c>
+      <c r="E13">
+        <v>184</v>
+      </c>
+      <c r="F13">
+        <v>6</v>
+      </c>
+      <c r="G13">
+        <v>2</v>
+      </c>
+      <c r="H13">
+        <v>184</v>
+      </c>
+      <c r="I13">
+        <v>6</v>
+      </c>
+      <c r="J13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>89</v>
+      </c>
+      <c r="B14">
+        <v>238</v>
+      </c>
+      <c r="C14">
+        <v>6</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>116</v>
+      </c>
+      <c r="F14">
+        <v>6</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15">
+        <v>42</v>
+      </c>
+      <c r="C15">
+        <v>6</v>
+      </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
+      <c r="E15">
+        <v>40</v>
+      </c>
+      <c r="F15">
+        <v>6</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>40</v>
+      </c>
+      <c r="I15">
+        <v>6</v>
+      </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>91</v>
+      </c>
+      <c r="B16">
+        <v>42</v>
+      </c>
+      <c r="C16">
+        <v>6</v>
+      </c>
+      <c r="D16">
+        <v>2</v>
+      </c>
+      <c r="E16">
+        <v>40</v>
+      </c>
+      <c r="F16">
+        <v>6</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>40</v>
+      </c>
+      <c r="I16">
+        <v>6</v>
+      </c>
+      <c r="J16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>92</v>
+      </c>
+      <c r="B17">
+        <v>39</v>
+      </c>
+      <c r="C17">
+        <v>3</v>
+      </c>
+      <c r="D17">
+        <v>2</v>
+      </c>
+      <c r="E17">
+        <v>39</v>
+      </c>
+      <c r="F17">
+        <v>3</v>
+      </c>
+      <c r="G17">
+        <v>2</v>
+      </c>
+      <c r="H17">
+        <v>39</v>
+      </c>
+      <c r="I17">
+        <v>3</v>
+      </c>
+      <c r="J17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18">
+        <v>344</v>
+      </c>
+      <c r="C18">
+        <v>8</v>
+      </c>
+      <c r="D18">
+        <v>7</v>
+      </c>
+      <c r="E18">
+        <v>314</v>
+      </c>
+      <c r="F18">
+        <v>6</v>
+      </c>
+      <c r="G18">
+        <v>10</v>
+      </c>
+      <c r="H18">
+        <v>314</v>
+      </c>
+      <c r="I18">
+        <v>6</v>
+      </c>
+      <c r="J18">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>94</v>
+      </c>
+      <c r="B19">
+        <v>90</v>
+      </c>
+      <c r="C19">
+        <v>5</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>88</v>
+      </c>
+      <c r="F19">
+        <v>5</v>
+      </c>
+      <c r="G19">
+        <v>2</v>
+      </c>
+      <c r="H19">
+        <v>88</v>
+      </c>
+      <c r="I19">
+        <v>5</v>
+      </c>
+      <c r="J19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>95</v>
+      </c>
+      <c r="B20">
+        <v>144</v>
+      </c>
+      <c r="C20">
+        <v>5</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>123</v>
+      </c>
+      <c r="F20">
+        <v>6</v>
+      </c>
+      <c r="G20">
+        <v>3</v>
+      </c>
+      <c r="H20">
+        <v>123</v>
+      </c>
+      <c r="I20">
+        <v>6</v>
+      </c>
+      <c r="J20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>96</v>
+      </c>
+      <c r="B21">
+        <v>271</v>
+      </c>
+      <c r="C21">
+        <v>6</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>170</v>
+      </c>
+      <c r="F21">
+        <v>6</v>
+      </c>
+      <c r="G21">
+        <v>2</v>
+      </c>
+      <c r="H21">
+        <v>170</v>
+      </c>
+      <c r="I21">
+        <v>6</v>
+      </c>
+      <c r="J21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B22" s="1">
+        <f>SUM(B3:B21)</f>
+        <v>2871</v>
+      </c>
+      <c r="C22" s="1">
+        <f t="shared" ref="C22:M22" si="0">SUM(C3:C21)</f>
+        <v>90</v>
+      </c>
+      <c r="D22" s="1">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+      <c r="E22" s="1">
+        <f t="shared" si="0"/>
+        <v>2386</v>
+      </c>
+      <c r="F22" s="1">
+        <f t="shared" si="0"/>
+        <v>103</v>
+      </c>
+      <c r="G22" s="1">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+      <c r="H22" s="1">
+        <f t="shared" si="0"/>
+        <v>2368</v>
+      </c>
+      <c r="I22" s="1">
+        <f t="shared" si="0"/>
+        <v>92</v>
+      </c>
+      <c r="J22" s="1">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
+      <c r="K22" s="1">
+        <f t="shared" si="0"/>
+        <v>453</v>
+      </c>
+      <c r="L22" s="1">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="M22" s="1">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="E1:G1"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="K1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Reduced IL by 292 bytes (-14 %), from 2082 to 1790
</commit_message>
<xml_diff>
--- a/ILSIze.xlsx
+++ b/ILSIze.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87274557-5504-4948-B40A-52E010EFEB22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C965DA2D-24E0-7F4A-AC4F-14856AA9BCF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35000" yWindow="-2540" windowWidth="24960" windowHeight="15900" activeTab="6" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="24960" windowHeight="15500" activeTab="6" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
   </bookViews>
   <sheets>
     <sheet name="Chemistry.cs" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="101">
   <si>
     <t>Méthode</t>
   </si>
@@ -333,6 +333,18 @@
   </si>
   <si>
     <t>Atan2</t>
+  </si>
+  <si>
+    <t>Sqrt</t>
+  </si>
+  <si>
+    <t>ExpBySquaring</t>
+  </si>
+  <si>
+    <t>GetDecimalPlaces</t>
+  </si>
+  <si>
+    <t>Remainder</t>
   </si>
 </sst>
 </file>
@@ -342,7 +354,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -370,13 +382,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -388,9 +412,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -403,11 +428,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="2"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Pourcentage" xfId="1" builtinId="5"/>
+    <cellStyle name="Satisfaisant" xfId="2" builtinId="26"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2356,7 +2382,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2043A2D3-B79F-994A-8E5F-6CAF0A113206}">
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.5" bestFit="1" customWidth="1"/>
@@ -2369,12 +2395,9 @@
     <col min="8" max="8" width="5.5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="5.83203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.83203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="5" t="s">
         <v>77</v>
@@ -2391,13 +2414,8 @@
       </c>
       <c r="I1" s="5"/>
       <c r="J1" s="5"/>
-      <c r="K1" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>76</v>
       </c>
@@ -2428,17 +2446,8 @@
       <c r="J2" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -2469,18 +2478,9 @@
       <c r="J3">
         <v>6</v>
       </c>
-      <c r="K3">
-        <v>188</v>
-      </c>
-      <c r="L3">
-        <v>6</v>
-      </c>
-      <c r="M3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>79</v>
       </c>
       <c r="B4">
@@ -2510,18 +2510,9 @@
       <c r="J4">
         <v>3</v>
       </c>
-      <c r="K4">
-        <v>265</v>
-      </c>
-      <c r="L4">
-        <v>3</v>
-      </c>
-      <c r="M4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>81</v>
       </c>
       <c r="B5">
@@ -2551,18 +2542,9 @@
       <c r="J5">
         <v>0</v>
       </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="6" t="s">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>80</v>
       </c>
       <c r="B6">
@@ -2593,8 +2575,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>83</v>
       </c>
       <c r="B7">
@@ -2625,8 +2607,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>82</v>
       </c>
       <c r="B8">
@@ -2657,8 +2639,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="6" t="s">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>84</v>
       </c>
       <c r="B9">
@@ -2689,8 +2671,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="6" t="s">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>85</v>
       </c>
       <c r="B10">
@@ -2721,8 +2703,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="6" t="s">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>86</v>
       </c>
       <c r="B11">
@@ -2753,8 +2735,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A12" s="6" t="s">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>87</v>
       </c>
       <c r="B12">
@@ -2785,8 +2767,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A13" s="6" t="s">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>88</v>
       </c>
       <c r="B13">
@@ -2817,7 +2799,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>89</v>
       </c>
@@ -2848,18 +2830,9 @@
       <c r="J14">
         <v>0</v>
       </c>
-      <c r="K14">
-        <v>0</v>
-      </c>
-      <c r="L14">
-        <v>0</v>
-      </c>
-      <c r="M14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15" s="6" t="s">
         <v>90</v>
       </c>
       <c r="B15">
@@ -2890,8 +2863,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" s="6" t="s">
         <v>91</v>
       </c>
       <c r="B16">
@@ -2922,8 +2895,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17" s="6" t="s">
         <v>92</v>
       </c>
       <c r="B17">
@@ -2954,7 +2927,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -2986,7 +2959,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>94</v>
       </c>
@@ -3018,7 +2991,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>95</v>
       </c>
@@ -3050,7 +3023,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>96</v>
       </c>
@@ -3082,13 +3055,13 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B22" s="1">
         <f>SUM(B3:B21)</f>
         <v>2871</v>
       </c>
       <c r="C22" s="1">
-        <f t="shared" ref="C22:M22" si="0">SUM(C3:C21)</f>
+        <f t="shared" ref="C22:J22" si="0">SUM(C3:C21)</f>
         <v>90</v>
       </c>
       <c r="D22" s="1">
@@ -3119,25 +3092,257 @@
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
-      <c r="K22" s="1">
-        <f t="shared" si="0"/>
-        <v>453</v>
-      </c>
-      <c r="L22" s="1">
-        <f t="shared" si="0"/>
-        <v>9</v>
-      </c>
-      <c r="M22" s="1">
-        <f t="shared" si="0"/>
-        <v>9</v>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A24" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B24">
+        <v>347</v>
+      </c>
+      <c r="C24">
+        <v>5</v>
+      </c>
+      <c r="D24">
+        <v>4</v>
+      </c>
+      <c r="E24">
+        <v>323</v>
+      </c>
+      <c r="F24">
+        <v>5</v>
+      </c>
+      <c r="G24">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A25" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B25">
+        <v>263</v>
+      </c>
+      <c r="C25">
+        <v>6</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>194</v>
+      </c>
+      <c r="F25">
+        <v>6</v>
+      </c>
+      <c r="G25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B26">
+        <v>285</v>
+      </c>
+      <c r="C26">
+        <v>6</v>
+      </c>
+      <c r="D26">
+        <v>4</v>
+      </c>
+      <c r="E26">
+        <v>254</v>
+      </c>
+      <c r="F26">
+        <v>6</v>
+      </c>
+      <c r="G26">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>78</v>
+      </c>
+      <c r="B27">
+        <v>285</v>
+      </c>
+      <c r="C27">
+        <v>6</v>
+      </c>
+      <c r="D27">
+        <v>5</v>
+      </c>
+      <c r="E27">
+        <v>244</v>
+      </c>
+      <c r="F27">
+        <v>6</v>
+      </c>
+      <c r="G27">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B28">
+        <v>281</v>
+      </c>
+      <c r="C28">
+        <v>6</v>
+      </c>
+      <c r="D28">
+        <v>4</v>
+      </c>
+      <c r="E28">
+        <v>250</v>
+      </c>
+      <c r="F28">
+        <v>6</v>
+      </c>
+      <c r="G28">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A29" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B29">
+        <v>160</v>
+      </c>
+      <c r="C29">
+        <v>6</v>
+      </c>
+      <c r="D29">
+        <v>4</v>
+      </c>
+      <c r="E29">
+        <v>160</v>
+      </c>
+      <c r="F29">
+        <v>6</v>
+      </c>
+      <c r="G29">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>98</v>
+      </c>
+      <c r="B30">
+        <v>176</v>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+      <c r="D30">
+        <v>2</v>
+      </c>
+      <c r="E30">
+        <v>77</v>
+      </c>
+      <c r="F30">
+        <v>3</v>
+      </c>
+      <c r="G30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>99</v>
+      </c>
+      <c r="B31">
+        <v>99</v>
+      </c>
+      <c r="C31">
+        <v>4</v>
+      </c>
+      <c r="D31">
+        <v>3</v>
+      </c>
+      <c r="E31">
+        <v>99</v>
+      </c>
+      <c r="F31">
+        <v>4</v>
+      </c>
+      <c r="G31">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>100</v>
+      </c>
+      <c r="B32">
+        <v>186</v>
+      </c>
+      <c r="C32">
+        <v>5</v>
+      </c>
+      <c r="D32">
+        <v>5</v>
+      </c>
+      <c r="E32">
+        <v>189</v>
+      </c>
+      <c r="F32">
+        <v>5</v>
+      </c>
+      <c r="G32">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B33" s="1">
+        <f>SUM(B24:B32)</f>
+        <v>2082</v>
+      </c>
+      <c r="C33">
+        <f t="shared" ref="C33:G33" si="1">SUM(C24:C32)</f>
+        <v>47</v>
+      </c>
+      <c r="D33">
+        <f t="shared" si="1"/>
+        <v>32</v>
+      </c>
+      <c r="E33" s="1">
+        <f t="shared" si="1"/>
+        <v>1790</v>
+      </c>
+      <c r="F33">
+        <f t="shared" si="1"/>
+        <v>47</v>
+      </c>
+      <c r="G33">
+        <f t="shared" si="1"/>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="E34">
+        <f>E33-B33</f>
+        <v>-292</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="E35" s="3">
+        <f>E34/B33</f>
+        <v>-0.14024975984630164</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="E1:G1"/>
     <mergeCell ref="H1:J1"/>
-    <mergeCell ref="K1:M1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Single-pass linear regression computation
Not sure the added IList<PointD|PointM> overload provides better performance over IEnumerable<PointD|PointM>. It does not look so on .NET Framework 4.0 64 bits on Windows Server 2019 running on a first generation Ryzen
</commit_message>
<xml_diff>
--- a/ILSIze.xlsx
+++ b/ILSIze.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\Administrator\source\repos\repzilon\Repzilon.Libraries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C965DA2D-24E0-7F4A-AC4F-14856AA9BCF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68BA31DB-9DEC-4F54-BC1F-6F90BA2489A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="24960" windowHeight="15500" activeTab="6" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
+    <workbookView xWindow="0" yWindow="7335" windowWidth="28800" windowHeight="10065" activeTab="3" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
   </bookViews>
   <sheets>
     <sheet name="Chemistry.cs" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="115">
   <si>
     <t>Méthode</t>
   </si>
@@ -345,20 +345,59 @@
   </si>
   <si>
     <t>Remainder</t>
+  </si>
+  <si>
+    <t>Itération 6</t>
+  </si>
+  <si>
+    <t>PointD[]</t>
+  </si>
+  <si>
+    <t>I*List&lt;PointD&gt;</t>
+  </si>
+  <si>
+    <t>Aggregate</t>
+  </si>
+  <si>
+    <t>FinishCompute</t>
+  </si>
+  <si>
+    <t>PointM[]</t>
+  </si>
+  <si>
+    <t>I*List&lt;PointM&gt;</t>
+  </si>
+  <si>
+    <t>📚</t>
+  </si>
+  <si>
+    <t>📟</t>
+  </si>
+  <si>
+    <t>Itération 7</t>
+  </si>
+  <si>
+    <t>T is Decimal</t>
+  </si>
+  <si>
+    <t>T is Double</t>
+  </si>
+  <si>
+    <t>Itération 8</t>
+  </si>
+  <si>
+    <t>Itération 9</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-  </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Franklin Gothic Book"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -366,27 +405,33 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Franklin Gothic Book"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Franklin Gothic Book"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="Aptos Narrow"/>
+      <name val="Franklin Gothic Book"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF006100"/>
-      <name val="Aptos Narrow"/>
+      <name val="Franklin Gothic Book"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Franklin Gothic Book"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -417,18 +462,24 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -449,9 +500,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -459,100 +510,48 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Franklin Gothic">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Franklin Gothic Medium" panose="020B0603020102020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Jpan" typeface="HG創英角ｺﾞｼｯｸUB"/>
+        <a:font script="Hang" typeface="돋움"/>
+        <a:font script="Hans" typeface="隶书"/>
+        <a:font script="Hant" typeface="微軟正黑體"/>
+        <a:font script="Arab" typeface="Tahoma"/>
+        <a:font script="Hebr" typeface="Aharoni"/>
+        <a:font script="Thai" typeface="LilyUPC"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -576,26 +575,44 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Franklin Gothic Book" panose="020B0503020102020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="HGｺﾞｼｯｸE"/>
+        <a:font script="Hang" typeface="돋움"/>
+        <a:font script="Hans" typeface="华文楷体"/>
+        <a:font script="Hant" typeface="微軟正黑體"/>
+        <a:font script="Arab" typeface="Tahoma"/>
+        <a:font script="Hebr" typeface="Aharoni"/>
+        <a:font script="Thai" typeface="LilyUPC"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Tahoma"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -654,6 +671,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -662,13 +686,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -733,31 +750,11 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -766,30 +763,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E085EFD-832C-3644-BF11-30C65FA80A90}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.77734375" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" customWidth="1"/>
+    <col min="4" max="4" width="6.109375" customWidth="1"/>
+    <col min="5" max="5" width="5" customWidth="1"/>
+    <col min="6" max="6" width="5.6640625" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -812,7 +809,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -835,7 +832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -858,7 +855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -881,7 +878,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -904,7 +901,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -927,7 +924,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -951,7 +948,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -974,7 +971,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -997,7 +994,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -1020,7 +1017,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B12" s="1">
         <f t="shared" ref="B12:G12" si="0">SUM(B3:B11)</f>
         <v>975</v>
@@ -1046,7 +1043,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E13">
         <f>E12-B12</f>
         <v>-38</v>
@@ -1064,14 +1061,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB670503-4F5B-E64E-832A-2C886DE2735D}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" customWidth="1"/>
+    <col min="3" max="3" width="5.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -1082,7 +1079,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1093,7 +1090,7 @@
         <v>-14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1105,7 +1102,7 @@
         <v>-54</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -1117,7 +1114,7 @@
         <v>-84</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1129,7 +1126,7 @@
         <v>-20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1149,16 +1146,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE08D056-9034-D44D-B934-446C62FAF677}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.5546875" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" customWidth="1"/>
+    <col min="3" max="4" width="4.33203125" customWidth="1"/>
+    <col min="5" max="5" width="5.33203125" customWidth="1"/>
+    <col min="6" max="6" width="4.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1178,7 +1175,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -1198,7 +1195,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -1218,7 +1215,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -1232,7 +1229,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>32</v>
       </c>
@@ -1246,7 +1243,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -1257,7 +1254,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>38</v>
       </c>
@@ -1274,7 +1271,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C8" s="1">
         <f>SUM(C$2:C6)</f>
         <v>163</v>
@@ -1292,7 +1289,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C9" s="1">
         <f>SUM(C$2:C7)</f>
         <v>163</v>
@@ -1318,117 +1315,184 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14CFDCA3-71A5-DD4D-9D0E-D63068092BC8}">
-  <dimension ref="A1:R9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:AD17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="3.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="3.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="3.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="3.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="3.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="3.5546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="3.33203125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="3.5546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="3.33203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="3.5546875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="3.109375" customWidth="1"/>
+    <col min="27" max="27" width="4.109375" customWidth="1"/>
+    <col min="28" max="28" width="4" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="3.33203125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="3.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4" t="s">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4" t="s">
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4" t="s">
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4" t="s">
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="T1" s="6"/>
+      <c r="U1" s="6"/>
+      <c r="V1" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="W1" s="6"/>
+      <c r="X1" s="6"/>
+      <c r="Y1" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="Z1" s="6"/>
+      <c r="AA1" s="6"/>
+      <c r="AB1" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="AC1" s="6"/>
+      <c r="AD1" s="6"/>
+    </row>
+    <row r="2" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H2" t="s">
-        <v>2</v>
-      </c>
-      <c r="I2" t="s">
-        <v>3</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="H2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K2" t="s">
-        <v>2</v>
-      </c>
-      <c r="L2" t="s">
-        <v>3</v>
-      </c>
-      <c r="M2" t="s">
+      <c r="K2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="N2" t="s">
-        <v>2</v>
-      </c>
-      <c r="O2" t="s">
-        <v>3</v>
-      </c>
-      <c r="P2" t="s">
+      <c r="N2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="P2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="Q2" t="s">
-        <v>2</v>
-      </c>
-      <c r="R2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="Q2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="8" t="s">
         <v>41</v>
       </c>
       <c r="C3" t="s">
@@ -1479,14 +1543,46 @@
       <c r="R3">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B4" t="s">
-        <v>41</v>
-      </c>
+      <c r="S3">
+        <v>241</v>
+      </c>
+      <c r="T3">
+        <v>4</v>
+      </c>
+      <c r="U3">
+        <v>10</v>
+      </c>
+      <c r="V3">
+        <v>241</v>
+      </c>
+      <c r="W3">
+        <v>4</v>
+      </c>
+      <c r="X3">
+        <v>10</v>
+      </c>
+      <c r="Y3">
+        <v>241</v>
+      </c>
+      <c r="Z3">
+        <v>4</v>
+      </c>
+      <c r="AA3">
+        <v>10</v>
+      </c>
+      <c r="AB3">
+        <v>241</v>
+      </c>
+      <c r="AC3">
+        <v>4</v>
+      </c>
+      <c r="AD3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A4" s="7"/>
+      <c r="B4" s="8"/>
       <c r="C4" t="s">
         <v>43</v>
       </c>
@@ -1535,232 +1631,617 @@
       <c r="R4">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="S4">
+        <v>263</v>
+      </c>
+      <c r="T4">
+        <v>4</v>
+      </c>
+      <c r="U4">
+        <v>10</v>
+      </c>
+      <c r="V4">
+        <v>263</v>
+      </c>
+      <c r="W4">
+        <v>4</v>
+      </c>
+      <c r="X4">
+        <v>10</v>
+      </c>
+      <c r="Y4">
+        <v>263</v>
+      </c>
+      <c r="Z4">
+        <v>4</v>
+      </c>
+      <c r="AA4">
+        <v>10</v>
+      </c>
+      <c r="AB4">
+        <v>263</v>
+      </c>
+      <c r="AC4">
+        <v>4</v>
+      </c>
+      <c r="AD4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="S5">
+        <v>7</v>
+      </c>
+      <c r="T5">
+        <v>8</v>
+      </c>
+      <c r="U5">
+        <v>0</v>
+      </c>
+      <c r="V5">
+        <v>7</v>
+      </c>
+      <c r="W5">
+        <v>8</v>
+      </c>
+      <c r="X5">
+        <v>0</v>
+      </c>
+      <c r="Y5">
+        <v>7</v>
+      </c>
+      <c r="Z5">
+        <v>8</v>
+      </c>
+      <c r="AA5">
+        <v>0</v>
+      </c>
+      <c r="AB5">
+        <v>7</v>
+      </c>
+      <c r="AC5">
+        <v>8</v>
+      </c>
+      <c r="AD5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A6" s="7"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="V6">
+        <v>267</v>
+      </c>
+      <c r="W6">
+        <v>10</v>
+      </c>
+      <c r="X6">
+        <v>15</v>
+      </c>
+      <c r="Y6">
+        <v>215</v>
+      </c>
+      <c r="Z6">
+        <v>10</v>
+      </c>
+      <c r="AA6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A7" s="7"/>
+      <c r="B7" s="8"/>
+      <c r="C7" t="s">
         <v>42</v>
       </c>
-      <c r="D5">
+      <c r="D7">
         <v>493</v>
       </c>
-      <c r="E5">
+      <c r="E7">
         <v>12</v>
       </c>
-      <c r="F5">
+      <c r="F7">
         <v>19</v>
       </c>
-      <c r="G5">
+      <c r="G7">
         <v>471</v>
       </c>
-      <c r="H5">
+      <c r="H7">
         <v>12</v>
       </c>
-      <c r="I5">
+      <c r="I7">
         <v>21</v>
       </c>
-      <c r="J5">
+      <c r="J7">
         <v>461</v>
       </c>
-      <c r="K5">
+      <c r="K7">
         <v>12</v>
       </c>
-      <c r="L5">
+      <c r="L7">
         <v>19</v>
       </c>
-      <c r="M5">
+      <c r="M7">
         <v>453</v>
       </c>
-      <c r="N5">
+      <c r="N7">
         <v>12</v>
       </c>
-      <c r="O5">
+      <c r="O7">
         <v>16</v>
       </c>
-      <c r="P5">
+      <c r="P7">
         <v>447</v>
       </c>
-      <c r="Q5">
+      <c r="Q7">
         <v>12</v>
       </c>
-      <c r="R5">
+      <c r="R7">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="S7">
+        <v>447</v>
+      </c>
+      <c r="T7">
+        <v>12</v>
+      </c>
+      <c r="U7">
+        <v>16</v>
+      </c>
+      <c r="V7">
+        <v>253</v>
+      </c>
+      <c r="W7">
+        <v>10</v>
+      </c>
+      <c r="X7">
+        <v>14</v>
+      </c>
+      <c r="Y7">
+        <v>201</v>
+      </c>
+      <c r="Z7">
+        <v>10</v>
+      </c>
+      <c r="AA7">
+        <v>14</v>
+      </c>
+      <c r="AB7">
+        <v>199</v>
+      </c>
+      <c r="AC7">
+        <v>10</v>
+      </c>
+      <c r="AD7">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A8" s="7"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="S8">
+        <v>7</v>
+      </c>
+      <c r="T8">
+        <v>8</v>
+      </c>
+      <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <v>7</v>
+      </c>
+      <c r="W8">
+        <v>8</v>
+      </c>
+      <c r="X8">
+        <v>0</v>
+      </c>
+      <c r="Y8">
+        <v>7</v>
+      </c>
+      <c r="Z8">
+        <v>8</v>
+      </c>
+      <c r="AA8">
+        <v>0</v>
+      </c>
+      <c r="AB8">
+        <v>7</v>
+      </c>
+      <c r="AC8">
+        <v>8</v>
+      </c>
+      <c r="AD8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A9" s="7"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="V9">
+        <v>257</v>
+      </c>
+      <c r="W9">
+        <v>10</v>
+      </c>
+      <c r="X9">
+        <v>15</v>
+      </c>
+      <c r="Y9">
+        <v>220</v>
+      </c>
+      <c r="Z9">
+        <v>10</v>
+      </c>
+      <c r="AA9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A10" s="7"/>
+      <c r="B10" s="8"/>
+      <c r="C10" t="s">
         <v>43</v>
       </c>
-      <c r="D6">
+      <c r="D10">
         <v>596</v>
       </c>
-      <c r="E6">
+      <c r="E10">
         <v>12</v>
       </c>
-      <c r="F6">
+      <c r="F10">
         <v>19</v>
       </c>
-      <c r="G6">
+      <c r="G10">
         <v>568</v>
       </c>
-      <c r="H6">
+      <c r="H10">
         <v>12</v>
       </c>
-      <c r="I6">
+      <c r="I10">
         <v>21</v>
       </c>
-      <c r="J6">
+      <c r="J10">
         <v>558</v>
       </c>
-      <c r="K6">
+      <c r="K10">
         <v>12</v>
       </c>
-      <c r="L6">
+      <c r="L10">
         <v>19</v>
       </c>
-      <c r="M6">
+      <c r="M10">
         <v>550</v>
       </c>
-      <c r="N6">
+      <c r="N10">
         <v>12</v>
       </c>
-      <c r="O6">
+      <c r="O10">
         <v>16</v>
       </c>
-      <c r="P6">
+      <c r="P10">
         <v>543</v>
       </c>
-      <c r="Q6">
+      <c r="Q10">
         <v>12</v>
       </c>
-      <c r="R6">
+      <c r="R10">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D7" s="1">
-        <f>SUM(D3:D6)</f>
+      <c r="S10">
+        <v>543</v>
+      </c>
+      <c r="T10">
+        <v>12</v>
+      </c>
+      <c r="U10">
+        <v>16</v>
+      </c>
+      <c r="V10">
+        <v>253</v>
+      </c>
+      <c r="W10">
+        <v>10</v>
+      </c>
+      <c r="X10">
+        <v>14</v>
+      </c>
+      <c r="Y10">
+        <v>215</v>
+      </c>
+      <c r="Z10">
+        <v>10</v>
+      </c>
+      <c r="AA10">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A11" s="7"/>
+      <c r="B11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C11" t="s">
+        <v>112</v>
+      </c>
+      <c r="V11">
+        <v>52</v>
+      </c>
+      <c r="W11">
+        <v>4</v>
+      </c>
+      <c r="X11">
+        <v>2</v>
+      </c>
+      <c r="Y11">
+        <v>51</v>
+      </c>
+      <c r="Z11">
+        <v>4</v>
+      </c>
+      <c r="AA11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A12" s="7"/>
+      <c r="B12" t="s">
+        <v>104</v>
+      </c>
+      <c r="C12" t="s">
+        <v>111</v>
+      </c>
+      <c r="V12">
+        <v>120</v>
+      </c>
+      <c r="W12">
+        <v>4</v>
+      </c>
+      <c r="X12">
+        <v>2</v>
+      </c>
+      <c r="Y12">
+        <v>119</v>
+      </c>
+      <c r="Z12">
+        <v>4</v>
+      </c>
+      <c r="AA12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A13" s="7"/>
+      <c r="B13" t="s">
+        <v>105</v>
+      </c>
+      <c r="C13" t="s">
+        <v>112</v>
+      </c>
+      <c r="V13">
+        <v>98</v>
+      </c>
+      <c r="W13">
+        <v>12</v>
+      </c>
+      <c r="X13">
+        <v>1</v>
+      </c>
+      <c r="Y13">
+        <v>98</v>
+      </c>
+      <c r="Z13">
+        <v>12</v>
+      </c>
+      <c r="AA13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A14" s="7"/>
+      <c r="B14" t="s">
+        <v>105</v>
+      </c>
+      <c r="C14" t="s">
+        <v>111</v>
+      </c>
+      <c r="V14">
+        <v>147</v>
+      </c>
+      <c r="W14">
+        <v>12</v>
+      </c>
+      <c r="X14">
+        <v>1</v>
+      </c>
+      <c r="Y14">
+        <v>147</v>
+      </c>
+      <c r="Z14">
+        <v>12</v>
+      </c>
+      <c r="AA14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="D15" s="1">
+        <f>SUM(D3:D14)</f>
         <v>1661</v>
       </c>
-      <c r="E7" s="1">
-        <f t="shared" ref="E7:O7" si="0">SUM(E3:E6)</f>
+      <c r="E15" s="1">
+        <f t="shared" ref="E15:X15" si="0">SUM(E3:E14)</f>
         <v>34</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F15" s="1">
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G15" s="1">
         <f t="shared" si="0"/>
         <v>1588</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H15" s="1">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I15" s="1">
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J15" s="1">
         <f t="shared" si="0"/>
         <v>1561</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K15" s="1">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="L7" s="1">
-        <f>SUM(L3:L6)</f>
+      <c r="L15" s="1">
+        <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="M7" s="1">
+      <c r="M15" s="1">
         <f t="shared" si="0"/>
         <v>1507</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N15" s="1">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O15" s="1">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
-      <c r="P7" s="1">
-        <f t="shared" ref="P7" si="1">SUM(P3:P6)</f>
+      <c r="P15" s="1">
+        <f t="shared" si="0"/>
         <v>1494</v>
       </c>
-      <c r="Q7" s="1">
-        <f t="shared" ref="Q7" si="2">SUM(Q3:Q6)</f>
+      <c r="Q15" s="1">
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="R7" s="1">
-        <f t="shared" ref="R7" si="3">SUM(R3:R6)</f>
+      <c r="R15" s="1">
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="P8">
-        <f>P7-D7</f>
+      <c r="S15" s="1">
+        <f t="shared" si="0"/>
+        <v>1508</v>
+      </c>
+      <c r="T15" s="1">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="U15" s="1">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+      <c r="V15" s="1">
+        <f t="shared" si="0"/>
+        <v>1965</v>
+      </c>
+      <c r="W15" s="1">
+        <f t="shared" si="0"/>
+        <v>96</v>
+      </c>
+      <c r="X15" s="1">
+        <f t="shared" si="0"/>
+        <v>84</v>
+      </c>
+      <c r="Y15" s="1">
+        <f t="shared" ref="Y15" si="1">SUM(Y3:Y14)</f>
+        <v>1784</v>
+      </c>
+      <c r="Z15" s="1">
+        <f t="shared" ref="Z15" si="2">SUM(Z3:Z14)</f>
+        <v>96</v>
+      </c>
+      <c r="AA15" s="1">
+        <f t="shared" ref="AA15" si="3">SUM(AA3:AA14)</f>
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="P16">
+        <f>P15-D15</f>
         <v>-167</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="P9" s="2">
-        <f>P8/D7</f>
+    <row r="17" spans="16:16" x14ac:dyDescent="0.3">
+      <c r="P17" s="2">
+        <f>P16/D15</f>
         <v>-0.10054184226369657</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="13">
+    <mergeCell ref="AB1:AD1"/>
+    <mergeCell ref="Y1:AA1"/>
+    <mergeCell ref="A5:A14"/>
+    <mergeCell ref="B5:B10"/>
+    <mergeCell ref="V1:X1"/>
+    <mergeCell ref="S1:U1"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="G1:I1"/>
     <mergeCell ref="J1:L1"/>
     <mergeCell ref="M1:O1"/>
     <mergeCell ref="P1:R1"/>
   </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02857098-9EF4-7A43-8BB2-8228CE41206A}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.33203125" customWidth="1"/>
+    <col min="2" max="2" width="5.33203125" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" customWidth="1"/>
+    <col min="4" max="4" width="6.109375" customWidth="1"/>
+    <col min="5" max="5" width="5.5546875" customWidth="1"/>
+    <col min="6" max="6" width="5.6640625" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1783,7 +2264,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>50</v>
       </c>
@@ -1797,7 +2278,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>52</v>
       </c>
@@ -1811,7 +2292,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>51</v>
       </c>
@@ -1825,7 +2306,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>53</v>
       </c>
@@ -1839,7 +2320,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>54</v>
       </c>
@@ -1862,7 +2343,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>55</v>
       </c>
@@ -1876,7 +2357,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>56</v>
       </c>
@@ -1890,7 +2371,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>57</v>
       </c>
@@ -1913,7 +2394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>58</v>
       </c>
@@ -1936,7 +2417,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -1950,7 +2431,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>60</v>
       </c>
@@ -1964,7 +2445,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>61</v>
       </c>
@@ -1987,7 +2468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>62</v>
       </c>
@@ -2010,7 +2491,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>63</v>
       </c>
@@ -2033,7 +2514,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>64</v>
       </c>
@@ -2047,7 +2528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B18" s="1">
         <f>SUM(B3:B17)</f>
         <v>1588</v>
@@ -2073,14 +2554,14 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E19">
         <f>E18-B18</f>
         <v>-752</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E20" s="3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E20" s="2">
         <f>E19/B18</f>
         <v>-0.47355163727959698</v>
       </c>
@@ -2097,54 +2578,54 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3446A6D4-E7A1-DE4F-AF79-3C1286851385}">
   <dimension ref="A1:P7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.6640625" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" customWidth="1"/>
+    <col min="3" max="3" width="5.77734375" customWidth="1"/>
+    <col min="4" max="4" width="6.5546875" customWidth="1"/>
+    <col min="5" max="5" width="5.6640625" customWidth="1"/>
+    <col min="6" max="6" width="5.77734375" customWidth="1"/>
+    <col min="7" max="7" width="6.5546875" customWidth="1"/>
+    <col min="8" max="8" width="5.6640625" customWidth="1"/>
+    <col min="9" max="9" width="5.77734375" customWidth="1"/>
+    <col min="10" max="10" width="6.5546875" customWidth="1"/>
+    <col min="11" max="11" width="5.6640625" customWidth="1"/>
+    <col min="12" max="12" width="5.77734375" customWidth="1"/>
+    <col min="13" max="13" width="6.5546875" customWidth="1"/>
+    <col min="14" max="14" width="5.6640625" customWidth="1"/>
+    <col min="15" max="15" width="5.77734375" customWidth="1"/>
+    <col min="16" max="16" width="6.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="B1" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4" t="s">
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4" t="s">
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -2194,7 +2675,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>70</v>
       </c>
@@ -2244,7 +2725,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>71</v>
       </c>
@@ -2294,7 +2775,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B5" s="1">
         <f t="shared" ref="B5:G5" si="0">SUM(B3:B4)</f>
         <v>991</v>
@@ -2356,14 +2837,14 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="N6">
         <f>N5-B5</f>
         <v>-127</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="N7" s="3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="N7" s="2">
         <f>N6/B5</f>
         <v>-0.12815338042381433</v>
       </c>
@@ -2383,39 +2864,39 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2043A2D3-B79F-994A-8E5F-6CAF0A113206}">
   <dimension ref="A1:J35"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" customWidth="1"/>
+    <col min="3" max="3" width="6" customWidth="1"/>
+    <col min="4" max="4" width="6.77734375" customWidth="1"/>
+    <col min="5" max="5" width="5.6640625" customWidth="1"/>
+    <col min="6" max="6" width="6" customWidth="1"/>
+    <col min="7" max="7" width="6.77734375" customWidth="1"/>
+    <col min="8" max="8" width="5.6640625" customWidth="1"/>
+    <col min="9" max="9" width="6" customWidth="1"/>
+    <col min="10" max="10" width="6.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5" t="s">
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5" t="s">
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>76</v>
       </c>
@@ -2447,7 +2928,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -2479,7 +2960,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -2511,7 +2992,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>81</v>
       </c>
@@ -2543,7 +3024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>80</v>
       </c>
@@ -2575,7 +3056,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>83</v>
       </c>
@@ -2607,7 +3088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>82</v>
       </c>
@@ -2639,7 +3120,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>84</v>
       </c>
@@ -2671,7 +3152,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>85</v>
       </c>
@@ -2703,7 +3184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>86</v>
       </c>
@@ -2735,7 +3216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>87</v>
       </c>
@@ -2767,7 +3248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>88</v>
       </c>
@@ -2799,7 +3280,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>89</v>
       </c>
@@ -2831,8 +3312,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="6" t="s">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
         <v>90</v>
       </c>
       <c r="B15">
@@ -2863,8 +3344,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="6" t="s">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
         <v>91</v>
       </c>
       <c r="B16">
@@ -2895,8 +3376,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="6" t="s">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
         <v>92</v>
       </c>
       <c r="B17">
@@ -2927,7 +3408,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -2959,7 +3440,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>94</v>
       </c>
@@ -2991,7 +3472,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>95</v>
       </c>
@@ -3023,7 +3504,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>96</v>
       </c>
@@ -3055,7 +3536,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B22" s="1">
         <f>SUM(B3:B21)</f>
         <v>2871</v>
@@ -3093,8 +3574,8 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="6" t="s">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
         <v>94</v>
       </c>
       <c r="B24">
@@ -3116,8 +3597,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" s="6" t="s">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
         <v>96</v>
       </c>
       <c r="B25">
@@ -3139,8 +3620,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="6" t="s">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
         <v>84</v>
       </c>
       <c r="B26">
@@ -3162,7 +3643,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -3185,8 +3666,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" s="6" t="s">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
         <v>87</v>
       </c>
       <c r="B28">
@@ -3208,8 +3689,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" s="6" t="s">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" s="3" t="s">
         <v>97</v>
       </c>
       <c r="B29">
@@ -3231,7 +3712,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>98</v>
       </c>
@@ -3254,7 +3735,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>99</v>
       </c>
@@ -3277,7 +3758,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>100</v>
       </c>
@@ -3300,7 +3781,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B33" s="1">
         <f>SUM(B24:B32)</f>
         <v>2082</v>
@@ -3326,14 +3807,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:7" x14ac:dyDescent="0.3">
       <c r="E34">
         <f>E33-B33</f>
         <v>-292</v>
       </c>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="E35" s="3">
+    <row r="35" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="E35" s="2">
         <f>E34/B33</f>
         <v>-0.14024975984630164</v>
       </c>

</xml_diff>

<commit_message>
Added IList<PointM|PointD> overloads to RegressionModel.Compute
Although the global IL size increased, it seems they are at least slightly faster than the IEnumerable overloads.
</commit_message>
<xml_diff>
--- a/ILSIze.xlsx
+++ b/ILSIze.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\Administrator\source\repos\repzilon\Repzilon.Libraries\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68BA31DB-9DEC-4F54-BC1F-6F90BA2489A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2625EDCF-AC70-BC48-99D1-CD90CBADC23B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="7335" windowWidth="28800" windowHeight="10065" activeTab="3" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
+    <workbookView xWindow="25600" yWindow="-7500" windowWidth="38400" windowHeight="23500" activeTab="3" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
   </bookViews>
   <sheets>
     <sheet name="Chemistry.cs" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="119">
   <si>
     <t>Méthode</t>
   </si>
@@ -350,9 +350,6 @@
     <t>Itération 6</t>
   </si>
   <si>
-    <t>PointD[]</t>
-  </si>
-  <si>
     <t>I*List&lt;PointD&gt;</t>
   </si>
   <si>
@@ -362,9 +359,6 @@
     <t>FinishCompute</t>
   </si>
   <si>
-    <t>PointM[]</t>
-  </si>
-  <si>
     <t>I*List&lt;PointM&gt;</t>
   </si>
   <si>
@@ -387,6 +381,24 @@
   </si>
   <si>
     <t>Itération 9</t>
+  </si>
+  <si>
+    <t>IList&lt;PointD&gt;</t>
+  </si>
+  <si>
+    <t>IList&lt;PointM&gt;</t>
+  </si>
+  <si>
+    <t>InitLists&lt;T&gt;</t>
+  </si>
+  <si>
+    <t>AddDataPoint</t>
+  </si>
+  <si>
+    <t>PointD</t>
+  </si>
+  <si>
+    <t>PointM</t>
   </si>
 </sst>
 </file>
@@ -462,7 +474,7 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -479,6 +491,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -763,18 +778,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E085EFD-832C-3644-BF11-30C65FA80A90}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28.77734375" customWidth="1"/>
-    <col min="2" max="2" width="4.33203125" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" customWidth="1"/>
-    <col min="4" max="4" width="6.109375" customWidth="1"/>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.28515625" customWidth="1"/>
+    <col min="3" max="3" width="5.7109375" customWidth="1"/>
+    <col min="4" max="4" width="6.140625" customWidth="1"/>
     <col min="5" max="5" width="5" customWidth="1"/>
-    <col min="6" max="6" width="5.6640625" customWidth="1"/>
-    <col min="7" max="7" width="6.109375" customWidth="1"/>
+    <col min="6" max="6" width="5.7109375" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B1" s="5" t="s">
         <v>6</v>
       </c>
@@ -786,7 +801,7 @@
       <c r="F1" s="5"/>
       <c r="G1" s="5"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -809,7 +824,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -832,7 +847,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -855,7 +870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -878,7 +893,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -901,7 +916,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -924,7 +939,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -948,7 +963,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -971,7 +986,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -994,7 +1009,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -1017,7 +1032,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B12" s="1">
         <f t="shared" ref="B12:G12" si="0">SUM(B3:B11)</f>
         <v>975</v>
@@ -1043,7 +1058,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="E13">
         <f>E12-B12</f>
         <v>-38</v>
@@ -1061,14 +1076,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB670503-4F5B-E64E-832A-2C886DE2735D}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" customWidth="1"/>
-    <col min="3" max="3" width="5.77734375" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" customWidth="1"/>
+    <col min="3" max="3" width="5.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -1079,7 +1094,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1090,7 +1105,7 @@
         <v>-14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1102,7 +1117,7 @@
         <v>-54</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -1114,7 +1129,7 @@
         <v>-84</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1126,7 +1141,7 @@
         <v>-20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1146,16 +1161,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE08D056-9034-D44D-B934-446C62FAF677}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.5546875" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" customWidth="1"/>
-    <col min="3" max="4" width="4.33203125" customWidth="1"/>
-    <col min="5" max="5" width="5.33203125" customWidth="1"/>
-    <col min="6" max="6" width="4.33203125" customWidth="1"/>
+    <col min="1" max="1" width="29.5703125" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" customWidth="1"/>
+    <col min="3" max="4" width="4.28515625" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" customWidth="1"/>
+    <col min="6" max="6" width="4.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1175,7 +1190,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -1195,7 +1210,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -1215,7 +1230,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -1229,7 +1244,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>32</v>
       </c>
@@ -1243,7 +1258,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -1254,7 +1269,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>38</v>
       </c>
@@ -1271,7 +1286,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C8" s="1">
         <f>SUM(C$2:C6)</f>
         <v>163</v>
@@ -1289,7 +1304,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C9" s="1">
         <f>SUM(C$2:C7)</f>
         <v>163</v>
@@ -1315,41 +1330,34 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14CFDCA3-71A5-DD4D-9D0E-D63068092BC8}">
-  <dimension ref="A1:AD17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AD22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="3.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="3.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="3.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="3.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="3.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="3.5546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="3.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="3.5546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="3.33203125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="3.5546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="3.33203125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="3.5546875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="3.109375" customWidth="1"/>
-    <col min="27" max="27" width="4.109375" customWidth="1"/>
-    <col min="28" max="28" width="4" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="3.33203125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="3.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="5" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="5" bestFit="1" customWidth="1"/>
+    <col min="26" max="27" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="4" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="3.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="D1" s="6" t="s">
         <v>6</v>
       </c>
@@ -1381,22 +1389,22 @@
       <c r="T1" s="6"/>
       <c r="U1" s="6"/>
       <c r="V1" s="6" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="W1" s="6"/>
       <c r="X1" s="6"/>
       <c r="Y1" s="6" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="Z1" s="6"/>
       <c r="AA1" s="6"/>
       <c r="AB1" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="AC1" s="6"/>
       <c r="AD1" s="6"/>
     </row>
-    <row r="2" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>39</v>
       </c>
@@ -1419,76 +1427,76 @@
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="S2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="V2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="W2" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="X2" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="Y2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z2" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="AB2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AC2" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="AD2" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>40</v>
       </c>
@@ -1571,643 +1579,747 @@
         <v>10</v>
       </c>
       <c r="AB3">
-        <v>241</v>
+        <v>48</v>
       </c>
       <c r="AC3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AD3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A4" s="7"/>
       <c r="B4" s="8"/>
       <c r="C4" t="s">
+        <v>113</v>
+      </c>
+      <c r="AB4">
+        <v>41</v>
+      </c>
+      <c r="AC4">
+        <v>3</v>
+      </c>
+      <c r="AD4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A5" s="7"/>
+      <c r="B5" s="8"/>
+      <c r="C5" t="s">
         <v>43</v>
       </c>
-      <c r="D4">
+      <c r="D5">
         <v>297</v>
       </c>
-      <c r="E4">
+      <c r="E5">
         <v>5</v>
       </c>
-      <c r="F4">
+      <c r="F5">
         <v>8</v>
       </c>
-      <c r="G4">
+      <c r="G5">
         <v>287</v>
       </c>
-      <c r="H4">
-        <v>4</v>
-      </c>
-      <c r="I4">
+      <c r="H5">
+        <v>4</v>
+      </c>
+      <c r="I5">
         <v>9</v>
       </c>
-      <c r="J4">
+      <c r="J5">
         <v>282</v>
       </c>
-      <c r="K4">
-        <v>4</v>
-      </c>
-      <c r="L4">
+      <c r="K5">
+        <v>4</v>
+      </c>
+      <c r="L5">
         <v>11</v>
       </c>
-      <c r="M4">
+      <c r="M5">
         <v>263</v>
       </c>
-      <c r="N4">
-        <v>4</v>
-      </c>
-      <c r="O4">
+      <c r="N5">
+        <v>4</v>
+      </c>
+      <c r="O5">
         <v>10</v>
       </c>
-      <c r="P4">
+      <c r="P5">
         <v>263</v>
       </c>
-      <c r="Q4">
-        <v>4</v>
-      </c>
-      <c r="R4">
+      <c r="Q5">
+        <v>4</v>
+      </c>
+      <c r="R5">
         <v>10</v>
       </c>
-      <c r="S4">
+      <c r="S5">
         <v>263</v>
       </c>
-      <c r="T4">
-        <v>4</v>
-      </c>
-      <c r="U4">
+      <c r="T5">
+        <v>4</v>
+      </c>
+      <c r="U5">
         <v>10</v>
       </c>
-      <c r="V4">
+      <c r="V5">
         <v>263</v>
       </c>
-      <c r="W4">
-        <v>4</v>
-      </c>
-      <c r="X4">
+      <c r="W5">
+        <v>4</v>
+      </c>
+      <c r="X5">
         <v>10</v>
       </c>
-      <c r="Y4">
+      <c r="Y5">
         <v>263</v>
       </c>
-      <c r="Z4">
-        <v>4</v>
-      </c>
-      <c r="AA4">
+      <c r="Z5">
+        <v>4</v>
+      </c>
+      <c r="AA5">
         <v>10</v>
       </c>
-      <c r="AB4">
-        <v>263</v>
-      </c>
-      <c r="AC4">
-        <v>4</v>
-      </c>
-      <c r="AD4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="S5">
-        <v>7</v>
-      </c>
-      <c r="T5">
-        <v>8</v>
-      </c>
-      <c r="U5">
-        <v>0</v>
-      </c>
-      <c r="V5">
-        <v>7</v>
-      </c>
-      <c r="W5">
-        <v>8</v>
-      </c>
-      <c r="X5">
-        <v>0</v>
-      </c>
-      <c r="Y5">
-        <v>7</v>
-      </c>
-      <c r="Z5">
-        <v>8</v>
-      </c>
-      <c r="AA5">
-        <v>0</v>
-      </c>
       <c r="AB5">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="AC5">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="AD5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A6" s="7"/>
       <c r="B6" s="8"/>
-      <c r="C6" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="V6">
-        <v>267</v>
-      </c>
-      <c r="W6">
-        <v>10</v>
-      </c>
-      <c r="X6">
-        <v>15</v>
-      </c>
-      <c r="Y6">
-        <v>215</v>
-      </c>
-      <c r="Z6">
-        <v>10</v>
-      </c>
-      <c r="AA6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB6">
+        <v>41</v>
+      </c>
+      <c r="AC6">
+        <v>3</v>
+      </c>
+      <c r="AD6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A7" s="7"/>
-      <c r="B7" s="8"/>
-      <c r="C7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D7">
-        <v>493</v>
-      </c>
-      <c r="E7">
-        <v>12</v>
-      </c>
-      <c r="F7">
-        <v>19</v>
-      </c>
-      <c r="G7">
-        <v>471</v>
-      </c>
-      <c r="H7">
-        <v>12</v>
-      </c>
-      <c r="I7">
-        <v>21</v>
-      </c>
-      <c r="J7">
-        <v>461</v>
-      </c>
-      <c r="K7">
-        <v>12</v>
-      </c>
-      <c r="L7">
-        <v>19</v>
-      </c>
-      <c r="M7">
-        <v>453</v>
-      </c>
-      <c r="N7">
-        <v>12</v>
-      </c>
-      <c r="O7">
-        <v>16</v>
-      </c>
-      <c r="P7">
-        <v>447</v>
-      </c>
-      <c r="Q7">
-        <v>12</v>
-      </c>
-      <c r="R7">
-        <v>16</v>
-      </c>
-      <c r="S7">
-        <v>447</v>
-      </c>
-      <c r="T7">
-        <v>12</v>
-      </c>
-      <c r="U7">
-        <v>16</v>
-      </c>
-      <c r="V7">
-        <v>253</v>
-      </c>
-      <c r="W7">
-        <v>10</v>
-      </c>
-      <c r="X7">
-        <v>14</v>
-      </c>
-      <c r="Y7">
-        <v>201</v>
-      </c>
-      <c r="Z7">
-        <v>10</v>
-      </c>
-      <c r="AA7">
-        <v>14</v>
+      <c r="B7" s="9" t="s">
+        <v>115</v>
       </c>
       <c r="AB7">
-        <v>199</v>
+        <v>57</v>
       </c>
       <c r="AC7">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="AD7">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A8" s="7"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="S8">
-        <v>7</v>
-      </c>
-      <c r="T8">
-        <v>8</v>
-      </c>
-      <c r="U8">
-        <v>0</v>
-      </c>
-      <c r="V8">
-        <v>7</v>
-      </c>
-      <c r="W8">
-        <v>8</v>
-      </c>
-      <c r="X8">
-        <v>0</v>
-      </c>
-      <c r="Y8">
-        <v>7</v>
-      </c>
-      <c r="Z8">
-        <v>8</v>
-      </c>
-      <c r="AA8">
-        <v>0</v>
+      <c r="B8" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" t="s">
+        <v>117</v>
       </c>
       <c r="AB8">
-        <v>7</v>
+        <v>76</v>
       </c>
       <c r="AC8">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="AD8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="8"/>
-      <c r="C9" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="V9">
+      <c r="C9" t="s">
+        <v>118</v>
+      </c>
+      <c r="AB9">
+        <v>98</v>
+      </c>
+      <c r="AC9">
+        <v>3</v>
+      </c>
+      <c r="AD9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A10" s="7"/>
+      <c r="B10" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C10" t="s">
+        <v>113</v>
+      </c>
+      <c r="AB10">
+        <v>70</v>
+      </c>
+      <c r="AC10">
+        <v>4</v>
+      </c>
+      <c r="AD10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A11" s="7"/>
+      <c r="B11" s="8"/>
+      <c r="C11" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB11">
+        <v>70</v>
+      </c>
+      <c r="AC11">
+        <v>4</v>
+      </c>
+      <c r="AD11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A12" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="V12">
+        <v>267</v>
+      </c>
+      <c r="W12">
+        <v>10</v>
+      </c>
+      <c r="X12">
+        <v>15</v>
+      </c>
+      <c r="Y12">
+        <v>215</v>
+      </c>
+      <c r="Z12">
+        <v>10</v>
+      </c>
+      <c r="AA12">
+        <v>15</v>
+      </c>
+      <c r="AB12">
+        <v>215</v>
+      </c>
+      <c r="AC12">
+        <v>10</v>
+      </c>
+      <c r="AD12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A13" s="7"/>
+      <c r="B13" s="8"/>
+      <c r="C13" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13">
+        <v>493</v>
+      </c>
+      <c r="E13">
+        <v>12</v>
+      </c>
+      <c r="F13">
+        <v>19</v>
+      </c>
+      <c r="G13">
+        <v>471</v>
+      </c>
+      <c r="H13">
+        <v>12</v>
+      </c>
+      <c r="I13">
+        <v>21</v>
+      </c>
+      <c r="J13">
+        <v>461</v>
+      </c>
+      <c r="K13">
+        <v>12</v>
+      </c>
+      <c r="L13">
+        <v>19</v>
+      </c>
+      <c r="M13">
+        <v>453</v>
+      </c>
+      <c r="N13">
+        <v>12</v>
+      </c>
+      <c r="O13">
+        <v>16</v>
+      </c>
+      <c r="P13">
+        <v>447</v>
+      </c>
+      <c r="Q13">
+        <v>12</v>
+      </c>
+      <c r="R13">
+        <v>16</v>
+      </c>
+      <c r="S13">
+        <v>447</v>
+      </c>
+      <c r="T13">
+        <v>12</v>
+      </c>
+      <c r="U13">
+        <v>16</v>
+      </c>
+      <c r="V13">
+        <v>253</v>
+      </c>
+      <c r="W13">
+        <v>10</v>
+      </c>
+      <c r="X13">
+        <v>14</v>
+      </c>
+      <c r="Y13">
+        <v>199</v>
+      </c>
+      <c r="Z13">
+        <v>10</v>
+      </c>
+      <c r="AA13">
+        <v>14</v>
+      </c>
+      <c r="AB13">
+        <v>199</v>
+      </c>
+      <c r="AC13">
+        <v>10</v>
+      </c>
+      <c r="AD13">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A14" s="7"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="V14">
         <v>257</v>
       </c>
-      <c r="W9">
+      <c r="W14">
         <v>10</v>
       </c>
-      <c r="X9">
+      <c r="X14">
         <v>15</v>
       </c>
-      <c r="Y9">
+      <c r="Y14">
         <v>220</v>
       </c>
-      <c r="Z9">
+      <c r="Z14">
         <v>10</v>
       </c>
-      <c r="AA9">
+      <c r="AA14">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
-      <c r="B10" s="8"/>
-      <c r="C10" t="s">
+      <c r="AB14">
+        <v>220</v>
+      </c>
+      <c r="AC14">
+        <v>10</v>
+      </c>
+      <c r="AD14">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A15" s="7"/>
+      <c r="B15" s="8"/>
+      <c r="C15" t="s">
         <v>43</v>
       </c>
-      <c r="D10">
+      <c r="D15">
         <v>596</v>
       </c>
-      <c r="E10">
+      <c r="E15">
         <v>12</v>
       </c>
-      <c r="F10">
+      <c r="F15">
         <v>19</v>
       </c>
-      <c r="G10">
+      <c r="G15">
         <v>568</v>
       </c>
-      <c r="H10">
+      <c r="H15">
         <v>12</v>
       </c>
-      <c r="I10">
+      <c r="I15">
         <v>21</v>
       </c>
-      <c r="J10">
+      <c r="J15">
         <v>558</v>
       </c>
-      <c r="K10">
+      <c r="K15">
         <v>12</v>
       </c>
-      <c r="L10">
+      <c r="L15">
         <v>19</v>
       </c>
-      <c r="M10">
+      <c r="M15">
         <v>550</v>
       </c>
-      <c r="N10">
+      <c r="N15">
         <v>12</v>
       </c>
-      <c r="O10">
+      <c r="O15">
         <v>16</v>
       </c>
-      <c r="P10">
+      <c r="P15">
         <v>543</v>
       </c>
-      <c r="Q10">
+      <c r="Q15">
         <v>12</v>
       </c>
-      <c r="R10">
+      <c r="R15">
         <v>16</v>
       </c>
-      <c r="S10">
+      <c r="S15">
         <v>543</v>
       </c>
-      <c r="T10">
+      <c r="T15">
         <v>12</v>
       </c>
-      <c r="U10">
+      <c r="U15">
         <v>16</v>
       </c>
-      <c r="V10">
+      <c r="V15">
         <v>253</v>
       </c>
-      <c r="W10">
+      <c r="W15">
         <v>10</v>
       </c>
-      <c r="X10">
+      <c r="X15">
         <v>14</v>
       </c>
-      <c r="Y10">
+      <c r="Y15">
         <v>215</v>
       </c>
-      <c r="Z10">
+      <c r="Z15">
         <v>10</v>
       </c>
-      <c r="AA10">
+      <c r="AA15">
         <v>14</v>
       </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A11" s="7"/>
-      <c r="B11" t="s">
+      <c r="AB15">
+        <v>215</v>
+      </c>
+      <c r="AC15">
+        <v>10</v>
+      </c>
+      <c r="AD15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A16" s="7"/>
+      <c r="B16" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="C16" t="s">
+        <v>110</v>
+      </c>
+      <c r="V16">
+        <v>52</v>
+      </c>
+      <c r="W16">
+        <v>4</v>
+      </c>
+      <c r="X16">
+        <v>2</v>
+      </c>
+      <c r="Y16">
+        <v>51</v>
+      </c>
+      <c r="Z16">
+        <v>4</v>
+      </c>
+      <c r="AA16">
+        <v>2</v>
+      </c>
+      <c r="AB16">
+        <v>51</v>
+      </c>
+      <c r="AC16">
+        <v>4</v>
+      </c>
+      <c r="AD16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A17" s="7"/>
+      <c r="B17" s="8"/>
+      <c r="C17" t="s">
+        <v>109</v>
+      </c>
+      <c r="V17">
+        <v>120</v>
+      </c>
+      <c r="W17">
+        <v>4</v>
+      </c>
+      <c r="X17">
+        <v>2</v>
+      </c>
+      <c r="Y17">
+        <v>119</v>
+      </c>
+      <c r="Z17">
+        <v>4</v>
+      </c>
+      <c r="AA17">
+        <v>2</v>
+      </c>
+      <c r="AB17">
+        <v>119</v>
+      </c>
+      <c r="AC17">
+        <v>4</v>
+      </c>
+      <c r="AD17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A18" s="7"/>
+      <c r="B18" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="C11" t="s">
-        <v>112</v>
-      </c>
-      <c r="V11">
+      <c r="C18" t="s">
+        <v>110</v>
+      </c>
+      <c r="V18">
+        <v>98</v>
+      </c>
+      <c r="W18">
+        <v>12</v>
+      </c>
+      <c r="X18">
+        <v>1</v>
+      </c>
+      <c r="Y18">
+        <v>98</v>
+      </c>
+      <c r="Z18">
+        <v>12</v>
+      </c>
+      <c r="AA18">
+        <v>1</v>
+      </c>
+      <c r="AB18">
+        <v>98</v>
+      </c>
+      <c r="AC18">
+        <v>12</v>
+      </c>
+      <c r="AD18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="A19" s="7"/>
+      <c r="B19" s="8"/>
+      <c r="C19" t="s">
+        <v>109</v>
+      </c>
+      <c r="V19">
+        <v>147</v>
+      </c>
+      <c r="W19">
+        <v>12</v>
+      </c>
+      <c r="X19">
+        <v>1</v>
+      </c>
+      <c r="Y19">
+        <v>147</v>
+      </c>
+      <c r="Z19">
+        <v>12</v>
+      </c>
+      <c r="AA19">
+        <v>1</v>
+      </c>
+      <c r="AB19">
+        <v>147</v>
+      </c>
+      <c r="AC19">
+        <v>12</v>
+      </c>
+      <c r="AD19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="D20" s="1">
+        <f>SUM(D3:D19)</f>
+        <v>1661</v>
+      </c>
+      <c r="E20" s="1">
+        <f>SUM(E3:E19)</f>
+        <v>34</v>
+      </c>
+      <c r="F20" s="1">
+        <f>SUM(F3:F19)</f>
+        <v>54</v>
+      </c>
+      <c r="G20" s="1">
+        <f>SUM(G3:G19)</f>
+        <v>1588</v>
+      </c>
+      <c r="H20" s="1">
+        <f>SUM(H3:H19)</f>
+        <v>32</v>
+      </c>
+      <c r="I20" s="1">
+        <f>SUM(I3:I19)</f>
+        <v>60</v>
+      </c>
+      <c r="J20" s="1">
+        <f>SUM(J3:J19)</f>
+        <v>1561</v>
+      </c>
+      <c r="K20" s="1">
+        <f>SUM(K3:K19)</f>
+        <v>32</v>
+      </c>
+      <c r="L20" s="1">
+        <f>SUM(L3:L19)</f>
+        <v>60</v>
+      </c>
+      <c r="M20" s="1">
+        <f>SUM(M3:M19)</f>
+        <v>1507</v>
+      </c>
+      <c r="N20" s="1">
+        <f>SUM(N3:N19)</f>
+        <v>32</v>
+      </c>
+      <c r="O20" s="1">
+        <f>SUM(O3:O19)</f>
         <v>52</v>
       </c>
-      <c r="W11">
-        <v>4</v>
-      </c>
-      <c r="X11">
-        <v>2</v>
-      </c>
-      <c r="Y11">
-        <v>51</v>
-      </c>
-      <c r="Z11">
-        <v>4</v>
-      </c>
-      <c r="AA11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
-      <c r="B12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C12" t="s">
-        <v>111</v>
-      </c>
-      <c r="V12">
-        <v>120</v>
-      </c>
-      <c r="W12">
-        <v>4</v>
-      </c>
-      <c r="X12">
-        <v>2</v>
-      </c>
-      <c r="Y12">
-        <v>119</v>
-      </c>
-      <c r="Z12">
-        <v>4</v>
-      </c>
-      <c r="AA12">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A13" s="7"/>
-      <c r="B13" t="s">
-        <v>105</v>
-      </c>
-      <c r="C13" t="s">
-        <v>112</v>
-      </c>
-      <c r="V13">
-        <v>98</v>
-      </c>
-      <c r="W13">
-        <v>12</v>
-      </c>
-      <c r="X13">
-        <v>1</v>
-      </c>
-      <c r="Y13">
-        <v>98</v>
-      </c>
-      <c r="Z13">
-        <v>12</v>
-      </c>
-      <c r="AA13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A14" s="7"/>
-      <c r="B14" t="s">
-        <v>105</v>
-      </c>
-      <c r="C14" t="s">
-        <v>111</v>
-      </c>
-      <c r="V14">
-        <v>147</v>
-      </c>
-      <c r="W14">
-        <v>12</v>
-      </c>
-      <c r="X14">
-        <v>1</v>
-      </c>
-      <c r="Y14">
-        <v>147</v>
-      </c>
-      <c r="Z14">
-        <v>12</v>
-      </c>
-      <c r="AA14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="D15" s="1">
-        <f>SUM(D3:D14)</f>
-        <v>1661</v>
-      </c>
-      <c r="E15" s="1">
-        <f t="shared" ref="E15:X15" si="0">SUM(E3:E14)</f>
-        <v>34</v>
-      </c>
-      <c r="F15" s="1">
-        <f t="shared" si="0"/>
-        <v>54</v>
-      </c>
-      <c r="G15" s="1">
-        <f t="shared" si="0"/>
-        <v>1588</v>
-      </c>
-      <c r="H15" s="1">
-        <f t="shared" si="0"/>
+      <c r="P20" s="1">
+        <f>SUM(P3:P19)</f>
+        <v>1494</v>
+      </c>
+      <c r="Q20" s="1">
+        <f>SUM(Q3:Q19)</f>
         <v>32</v>
       </c>
-      <c r="I15" s="1">
-        <f t="shared" si="0"/>
-        <v>60</v>
-      </c>
-      <c r="J15" s="1">
-        <f t="shared" si="0"/>
-        <v>1561</v>
-      </c>
-      <c r="K15" s="1">
-        <f t="shared" si="0"/>
+      <c r="R20" s="1">
+        <f>SUM(R3:R19)</f>
+        <v>52</v>
+      </c>
+      <c r="S20" s="1">
+        <f>SUM(S3:S19)</f>
+        <v>1494</v>
+      </c>
+      <c r="T20" s="1">
+        <f>SUM(T3:T19)</f>
         <v>32</v>
       </c>
-      <c r="L15" s="1">
-        <f t="shared" si="0"/>
-        <v>60</v>
-      </c>
-      <c r="M15" s="1">
-        <f t="shared" si="0"/>
-        <v>1507</v>
-      </c>
-      <c r="N15" s="1">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-      <c r="O15" s="1">
-        <f t="shared" si="0"/>
+      <c r="U20" s="1">
+        <f>SUM(U3:U19)</f>
         <v>52</v>
       </c>
-      <c r="P15" s="1">
-        <f t="shared" si="0"/>
-        <v>1494</v>
-      </c>
-      <c r="Q15" s="1">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-      <c r="R15" s="1">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-      <c r="S15" s="1">
-        <f t="shared" si="0"/>
-        <v>1508</v>
-      </c>
-      <c r="T15" s="1">
-        <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-      <c r="U15" s="1">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-      <c r="V15" s="1">
-        <f t="shared" si="0"/>
-        <v>1965</v>
-      </c>
-      <c r="W15" s="1">
-        <f t="shared" si="0"/>
-        <v>96</v>
-      </c>
-      <c r="X15" s="1">
-        <f t="shared" si="0"/>
+      <c r="V20" s="1">
+        <f>SUM(V3:V19)</f>
+        <v>1951</v>
+      </c>
+      <c r="W20" s="1">
+        <f>SUM(W3:W19)</f>
+        <v>80</v>
+      </c>
+      <c r="X20" s="1">
+        <f>SUM(X3:X19)</f>
         <v>84</v>
       </c>
-      <c r="Y15" s="1">
-        <f t="shared" ref="Y15" si="1">SUM(Y3:Y14)</f>
-        <v>1784</v>
-      </c>
-      <c r="Z15" s="1">
-        <f t="shared" ref="Z15" si="2">SUM(Z3:Z14)</f>
-        <v>96</v>
-      </c>
-      <c r="AA15" s="1">
-        <f t="shared" ref="AA15" si="3">SUM(AA3:AA14)</f>
+      <c r="Y20" s="1">
+        <f>SUM(Y3:Y19)</f>
+        <v>1768</v>
+      </c>
+      <c r="Z20" s="1">
+        <f>SUM(Z3:Z19)</f>
+        <v>80</v>
+      </c>
+      <c r="AA20" s="1">
+        <f t="shared" ref="AA20" si="0">SUM(AA3:AA19)</f>
         <v>84</v>
       </c>
-    </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="P16">
-        <f>P15-D15</f>
+      <c r="AB20" s="1">
+        <f>SUM(AB3:AB19)</f>
+        <v>1813</v>
+      </c>
+      <c r="AC20" s="1">
+        <f>SUM(AC3:AC19)</f>
+        <v>101</v>
+      </c>
+      <c r="AD20" s="1">
+        <f>SUM(AD3:AD19)</f>
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="P21">
+        <f>P20-D20</f>
         <v>-167</v>
       </c>
     </row>
-    <row r="17" spans="16:16" x14ac:dyDescent="0.3">
-      <c r="P17" s="2">
-        <f>P16/D15</f>
+    <row r="22" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="P22" s="2">
+        <f>P21/D20</f>
         <v>-0.10054184226369657</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="17">
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B10:B11"/>
     <mergeCell ref="AB1:AD1"/>
     <mergeCell ref="Y1:AA1"/>
-    <mergeCell ref="A5:A14"/>
-    <mergeCell ref="B5:B10"/>
+    <mergeCell ref="A12:A19"/>
+    <mergeCell ref="B12:B15"/>
     <mergeCell ref="V1:X1"/>
     <mergeCell ref="S1:U1"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="A3:A11"/>
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="G1:I1"/>
     <mergeCell ref="J1:L1"/>
     <mergeCell ref="M1:O1"/>
     <mergeCell ref="P1:R1"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="B3:B6"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2218,18 +2330,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02857098-9EF4-7A43-8BB2-8228CE41206A}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.33203125" customWidth="1"/>
-    <col min="2" max="2" width="5.33203125" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" customWidth="1"/>
-    <col min="4" max="4" width="6.109375" customWidth="1"/>
-    <col min="5" max="5" width="5.5546875" customWidth="1"/>
-    <col min="6" max="6" width="5.6640625" customWidth="1"/>
-    <col min="7" max="7" width="6.109375" customWidth="1"/>
+    <col min="1" max="1" width="22.28515625" customWidth="1"/>
+    <col min="2" max="2" width="5.28515625" customWidth="1"/>
+    <col min="3" max="3" width="5.7109375" customWidth="1"/>
+    <col min="4" max="4" width="6.140625" customWidth="1"/>
+    <col min="5" max="5" width="5.5703125" customWidth="1"/>
+    <col min="6" max="6" width="5.7109375" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B1" s="5" t="s">
         <v>48</v>
       </c>
@@ -2241,7 +2353,7 @@
       <c r="F1" s="5"/>
       <c r="G1" s="5"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2264,7 +2376,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>50</v>
       </c>
@@ -2278,7 +2390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>52</v>
       </c>
@@ -2292,7 +2404,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>51</v>
       </c>
@@ -2306,7 +2418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>53</v>
       </c>
@@ -2320,7 +2432,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>54</v>
       </c>
@@ -2343,7 +2455,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>55</v>
       </c>
@@ -2357,7 +2469,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>56</v>
       </c>
@@ -2371,7 +2483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>57</v>
       </c>
@@ -2394,7 +2506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>58</v>
       </c>
@@ -2417,7 +2529,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -2431,7 +2543,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>60</v>
       </c>
@@ -2445,7 +2557,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>61</v>
       </c>
@@ -2468,7 +2580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>62</v>
       </c>
@@ -2491,7 +2603,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>63</v>
       </c>
@@ -2514,7 +2626,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>64</v>
       </c>
@@ -2528,7 +2640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B18" s="1">
         <f>SUM(B3:B17)</f>
         <v>1588</v>
@@ -2554,13 +2666,13 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="E19">
         <f>E18-B18</f>
         <v>-752</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="E20" s="2">
         <f>E19/B18</f>
         <v>-0.47355163727959698</v>
@@ -2578,27 +2690,22 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3446A6D4-E7A1-DE4F-AF79-3C1286851385}">
   <dimension ref="A1:P7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="5.6640625" customWidth="1"/>
-    <col min="3" max="3" width="5.77734375" customWidth="1"/>
-    <col min="4" max="4" width="6.5546875" customWidth="1"/>
-    <col min="5" max="5" width="5.6640625" customWidth="1"/>
-    <col min="6" max="6" width="5.77734375" customWidth="1"/>
-    <col min="7" max="7" width="6.5546875" customWidth="1"/>
-    <col min="8" max="8" width="5.6640625" customWidth="1"/>
-    <col min="9" max="9" width="5.77734375" customWidth="1"/>
-    <col min="10" max="10" width="6.5546875" customWidth="1"/>
-    <col min="11" max="11" width="5.6640625" customWidth="1"/>
-    <col min="12" max="12" width="5.77734375" customWidth="1"/>
-    <col min="13" max="13" width="6.5546875" customWidth="1"/>
-    <col min="14" max="14" width="5.6640625" customWidth="1"/>
-    <col min="15" max="15" width="5.77734375" customWidth="1"/>
-    <col min="16" max="16" width="6.5546875" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="3" width="5.7109375" customWidth="1"/>
+    <col min="4" max="4" width="6.5703125" customWidth="1"/>
+    <col min="5" max="6" width="5.7109375" customWidth="1"/>
+    <col min="7" max="7" width="6.5703125" customWidth="1"/>
+    <col min="8" max="9" width="5.7109375" customWidth="1"/>
+    <col min="10" max="10" width="6.5703125" customWidth="1"/>
+    <col min="11" max="12" width="5.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.5703125" customWidth="1"/>
+    <col min="14" max="15" width="5.7109375" customWidth="1"/>
+    <col min="16" max="16" width="6.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B1" s="5" t="s">
         <v>69</v>
       </c>
@@ -2625,7 +2732,7 @@
       <c r="O1" s="5"/>
       <c r="P1" s="5"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -2675,7 +2782,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>70</v>
       </c>
@@ -2725,7 +2832,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>71</v>
       </c>
@@ -2775,7 +2882,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B5" s="1">
         <f t="shared" ref="B5:G5" si="0">SUM(B3:B4)</f>
         <v>991</v>
@@ -2837,13 +2944,13 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="N6">
         <f>N5-B5</f>
         <v>-127</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="N7" s="2">
         <f>N6/B5</f>
         <v>-0.12815338042381433</v>
@@ -2864,21 +2971,21 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2043A2D3-B79F-994A-8E5F-6CAF0A113206}">
   <dimension ref="A1:J35"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="2" max="2" width="5.6640625" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="5.7109375" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="6.77734375" customWidth="1"/>
-    <col min="5" max="5" width="5.6640625" customWidth="1"/>
+    <col min="4" max="4" width="6.7109375" customWidth="1"/>
+    <col min="5" max="5" width="5.7109375" customWidth="1"/>
     <col min="6" max="6" width="6" customWidth="1"/>
-    <col min="7" max="7" width="6.77734375" customWidth="1"/>
-    <col min="8" max="8" width="5.6640625" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" customWidth="1"/>
+    <col min="8" max="8" width="5.7109375" customWidth="1"/>
     <col min="9" max="9" width="6" customWidth="1"/>
-    <col min="10" max="10" width="6.77734375" customWidth="1"/>
+    <col min="10" max="10" width="6.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="6" t="s">
         <v>77</v>
@@ -2896,7 +3003,7 @@
       <c r="I1" s="6"/>
       <c r="J1" s="6"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>76</v>
       </c>
@@ -2928,7 +3035,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -2960,7 +3067,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -2992,7 +3099,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>81</v>
       </c>
@@ -3024,7 +3131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>80</v>
       </c>
@@ -3056,7 +3163,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>83</v>
       </c>
@@ -3088,7 +3195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>82</v>
       </c>
@@ -3120,7 +3227,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>84</v>
       </c>
@@ -3152,7 +3259,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>85</v>
       </c>
@@ -3184,7 +3291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>86</v>
       </c>
@@ -3216,7 +3323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>87</v>
       </c>
@@ -3248,7 +3355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>88</v>
       </c>
@@ -3280,7 +3387,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>89</v>
       </c>
@@ -3312,7 +3419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>90</v>
       </c>
@@ -3344,7 +3451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>91</v>
       </c>
@@ -3376,7 +3483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>92</v>
       </c>
@@ -3408,7 +3515,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -3440,7 +3547,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>94</v>
       </c>
@@ -3472,7 +3579,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>95</v>
       </c>
@@ -3504,7 +3611,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>96</v>
       </c>
@@ -3536,7 +3643,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B22" s="1">
         <f>SUM(B3:B21)</f>
         <v>2871</v>
@@ -3574,7 +3681,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>94</v>
       </c>
@@ -3597,7 +3704,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
         <v>96</v>
       </c>
@@ -3620,7 +3727,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>84</v>
       </c>
@@ -3643,7 +3750,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -3666,7 +3773,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
         <v>87</v>
       </c>
@@ -3689,7 +3796,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
         <v>97</v>
       </c>
@@ -3712,7 +3819,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>98</v>
       </c>
@@ -3735,7 +3842,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>99</v>
       </c>
@@ -3758,7 +3865,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>100</v>
       </c>
@@ -3781,7 +3888,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B33" s="1">
         <f>SUM(B24:B32)</f>
         <v>2082</v>
@@ -3807,13 +3914,13 @@
         <v>44</v>
       </c>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
       <c r="E34">
         <f>E33-B33</f>
         <v>-292</v>
       </c>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="E35" s="2">
         <f>E34/B33</f>
         <v>-0.14024975984630164</v>

</xml_diff>

<commit_message>
Saved 33 IL bytes by optimizing argument passing in OutputLinearRegression2
</commit_message>
<xml_diff>
--- a/ILSIze.xlsx
+++ b/ILSIze.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2625EDCF-AC70-BC48-99D1-CD90CBADC23B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A783A36-9A09-6242-8FD2-271EA593A5D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25600" yWindow="-7500" windowWidth="38400" windowHeight="23500" activeTab="3" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14400" firstSheet="1" activeTab="7" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
   </bookViews>
   <sheets>
     <sheet name="Chemistry.cs" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Student" sheetId="5" r:id="rId5"/>
     <sheet name="Matrix.cs" sheetId="6" r:id="rId6"/>
     <sheet name="ExtraMath_decimal.cs" sheetId="7" r:id="rId7"/>
+    <sheet name="void OutputLinearRegression2" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="127">
   <si>
     <t>Méthode</t>
   </si>
@@ -399,13 +400,40 @@
   </si>
   <si>
     <t>PointM</t>
+  </si>
+  <si>
+    <t>Overload</t>
+  </si>
+  <si>
+    <t>OutputLinearRegression2</t>
+  </si>
+  <si>
+    <t>Args</t>
+  </si>
+  <si>
+    <t>OutputParameterMargin</t>
+  </si>
+  <si>
+    <t>OutputXExtrapolation</t>
+  </si>
+  <si>
+    <t>OutputYExtrapolation</t>
+  </si>
+  <si>
+    <t>TRegression lrp, string numberFormat, bool checkBiases, TStorage? xForYExtrapolation, TStorage? yForXExtrapolation</t>
+  </si>
+  <si>
+    <t>TRegression lrp, string numberFormat, bool checkBiases, CultureInfo ciCu, TStorage b, TStorage sr, TStorage studentLawValue</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -418,6 +446,7 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Franklin Gothic Book"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -444,7 +473,13 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Franklin Gothic Book"/>
+      <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Avenir Next Condensed Regular"/>
     </font>
   </fonts>
   <fills count="3">
@@ -474,14 +509,17 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -489,11 +527,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -778,7 +814,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E085EFD-832C-3644-BF11-30C65FA80A90}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.28515625" customWidth="1"/>
@@ -789,42 +825,43 @@
     <col min="7" max="7" width="6.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5" t="s">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1"/>
+      <c r="B1" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -847,7 +884,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -870,7 +907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -893,7 +930,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -916,7 +953,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -939,7 +976,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -963,7 +1000,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -986,7 +1023,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1009,7 +1046,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -1032,7 +1069,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7">
       <c r="B12" s="1">
         <f t="shared" ref="B12:G12" si="0">SUM(B3:B11)</f>
         <v>975</v>
@@ -1058,7 +1095,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7">
       <c r="E13">
         <f>E12-B12</f>
         <v>-38</v>
@@ -1076,25 +1113,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB670503-4F5B-E64E-832A-2C886DE2735D}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="12.5703125" customWidth="1"/>
     <col min="3" max="3" width="5.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1105,7 +1142,7 @@
         <v>-14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1117,7 +1154,7 @@
         <v>-54</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -1129,7 +1166,7 @@
         <v>-84</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1141,7 +1178,7 @@
         <v>-20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1161,36 +1198,36 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE08D056-9034-D44D-B934-446C62FAF677}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="29.5703125" customWidth="1"/>
     <col min="2" max="2" width="16.140625" customWidth="1"/>
     <col min="3" max="4" width="4.28515625" customWidth="1"/>
-    <col min="5" max="5" width="5.28515625" customWidth="1"/>
+    <col min="5" max="5" width="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="4.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -1210,7 +1247,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -1230,7 +1267,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -1244,7 +1281,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>32</v>
       </c>
@@ -1258,7 +1295,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -1269,7 +1306,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>38</v>
       </c>
@@ -1286,7 +1323,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="C8" s="1">
         <f>SUM(C$2:C6)</f>
         <v>163</v>
@@ -1304,7 +1341,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="C9" s="1">
         <f>SUM(C$2:C7)</f>
         <v>163</v>
@@ -1331,7 +1368,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14CFDCA3-71A5-DD4D-9D0E-D63068092BC8}">
   <dimension ref="A1:AD22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -1357,54 +1394,54 @@
     <col min="30" max="30" width="3.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="D1" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6" t="s">
+    <row r="1" spans="1:30" s="1" customFormat="1">
+      <c r="D1" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6" t="s">
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6" t="s">
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6" t="s">
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="Q1" s="6"/>
-      <c r="R1" s="6"/>
-      <c r="S1" s="6" t="s">
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="T1" s="6"/>
-      <c r="U1" s="6"/>
-      <c r="V1" s="6" t="s">
+      <c r="T1" s="7"/>
+      <c r="U1" s="7"/>
+      <c r="V1" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="W1" s="6"/>
-      <c r="X1" s="6"/>
-      <c r="Y1" s="6" t="s">
+      <c r="W1" s="7"/>
+      <c r="X1" s="7"/>
+      <c r="Y1" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="Z1" s="6"/>
-      <c r="AA1" s="6"/>
-      <c r="AB1" s="6" t="s">
+      <c r="Z1" s="7"/>
+      <c r="AA1" s="7"/>
+      <c r="AB1" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="AC1" s="6"/>
-      <c r="AD1" s="6"/>
-    </row>
-    <row r="2" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="AC1" s="7"/>
+      <c r="AD1" s="7"/>
+    </row>
+    <row r="2" spans="1:30" s="1" customFormat="1">
       <c r="A2" s="1" t="s">
         <v>39</v>
       </c>
@@ -1496,11 +1533,11 @@
         <v>107</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:30">
+      <c r="A3" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="6" t="s">
         <v>41</v>
       </c>
       <c r="C3" t="s">
@@ -1588,9 +1625,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A4" s="7"/>
-      <c r="B4" s="8"/>
+    <row r="4" spans="1:30">
+      <c r="A4" s="8"/>
+      <c r="B4" s="6"/>
       <c r="C4" t="s">
         <v>113</v>
       </c>
@@ -1604,9 +1641,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A5" s="7"/>
-      <c r="B5" s="8"/>
+    <row r="5" spans="1:30">
+      <c r="A5" s="8"/>
+      <c r="B5" s="6"/>
       <c r="C5" t="s">
         <v>43</v>
       </c>
@@ -1692,9 +1729,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A6" s="7"/>
-      <c r="B6" s="8"/>
+    <row r="6" spans="1:30">
+      <c r="A6" s="8"/>
+      <c r="B6" s="6"/>
       <c r="C6" t="s">
         <v>114</v>
       </c>
@@ -1708,9 +1745,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A7" s="7"/>
-      <c r="B7" s="9" t="s">
+    <row r="7" spans="1:30">
+      <c r="A7" s="8"/>
+      <c r="B7" s="5" t="s">
         <v>115</v>
       </c>
       <c r="AB7">
@@ -1723,9 +1760,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A8" s="7"/>
-      <c r="B8" s="8" t="s">
+    <row r="8" spans="1:30">
+      <c r="A8" s="8"/>
+      <c r="B8" s="6" t="s">
         <v>116</v>
       </c>
       <c r="C8" t="s">
@@ -1741,9 +1778,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A9" s="7"/>
-      <c r="B9" s="8"/>
+    <row r="9" spans="1:30">
+      <c r="A9" s="8"/>
+      <c r="B9" s="6"/>
       <c r="C9" t="s">
         <v>118</v>
       </c>
@@ -1757,9 +1794,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A10" s="7"/>
-      <c r="B10" s="8" t="s">
+    <row r="10" spans="1:30">
+      <c r="A10" s="8"/>
+      <c r="B10" s="6" t="s">
         <v>104</v>
       </c>
       <c r="C10" t="s">
@@ -1775,9 +1812,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A11" s="7"/>
-      <c r="B11" s="8"/>
+    <row r="11" spans="1:30">
+      <c r="A11" s="8"/>
+      <c r="B11" s="6"/>
       <c r="C11" t="s">
         <v>114</v>
       </c>
@@ -1791,11 +1828,11 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A12" s="7" t="s">
+    <row r="12" spans="1:30">
+      <c r="A12" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="6" t="s">
         <v>41</v>
       </c>
       <c r="C12" s="4" t="s">
@@ -1829,9 +1866,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A13" s="7"/>
-      <c r="B13" s="8"/>
+    <row r="13" spans="1:30">
+      <c r="A13" s="8"/>
+      <c r="B13" s="6"/>
       <c r="C13" t="s">
         <v>42</v>
       </c>
@@ -1917,9 +1954,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A14" s="7"/>
-      <c r="B14" s="8"/>
+    <row r="14" spans="1:30">
+      <c r="A14" s="8"/>
+      <c r="B14" s="6"/>
       <c r="C14" s="4" t="s">
         <v>105</v>
       </c>
@@ -1951,9 +1988,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A15" s="7"/>
-      <c r="B15" s="8"/>
+    <row r="15" spans="1:30">
+      <c r="A15" s="8"/>
+      <c r="B15" s="6"/>
       <c r="C15" t="s">
         <v>43</v>
       </c>
@@ -2039,9 +2076,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A16" s="7"/>
-      <c r="B16" s="8" t="s">
+    <row r="16" spans="1:30">
+      <c r="A16" s="8"/>
+      <c r="B16" s="6" t="s">
         <v>103</v>
       </c>
       <c r="C16" t="s">
@@ -2075,9 +2112,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A17" s="7"/>
-      <c r="B17" s="8"/>
+    <row r="17" spans="1:30">
+      <c r="A17" s="8"/>
+      <c r="B17" s="6"/>
       <c r="C17" t="s">
         <v>109</v>
       </c>
@@ -2109,9 +2146,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A18" s="7"/>
-      <c r="B18" s="8" t="s">
+    <row r="18" spans="1:30">
+      <c r="A18" s="8"/>
+      <c r="B18" s="6" t="s">
         <v>104</v>
       </c>
       <c r="C18" t="s">
@@ -2145,9 +2182,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A19" s="7"/>
-      <c r="B19" s="8"/>
+    <row r="19" spans="1:30">
+      <c r="A19" s="8"/>
+      <c r="B19" s="6"/>
       <c r="C19" t="s">
         <v>109</v>
       </c>
@@ -2179,101 +2216,101 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:30">
       <c r="D20" s="1">
-        <f>SUM(D3:D19)</f>
+        <f t="shared" ref="D20:Z20" si="0">SUM(D3:D19)</f>
         <v>1661</v>
       </c>
       <c r="E20" s="1">
-        <f>SUM(E3:E19)</f>
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="F20" s="1">
-        <f>SUM(F3:F19)</f>
+        <f t="shared" si="0"/>
         <v>54</v>
       </c>
       <c r="G20" s="1">
-        <f>SUM(G3:G19)</f>
+        <f t="shared" si="0"/>
         <v>1588</v>
       </c>
       <c r="H20" s="1">
-        <f>SUM(H3:H19)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="I20" s="1">
-        <f>SUM(I3:I19)</f>
+        <f t="shared" si="0"/>
         <v>60</v>
       </c>
       <c r="J20" s="1">
-        <f>SUM(J3:J19)</f>
+        <f t="shared" si="0"/>
         <v>1561</v>
       </c>
       <c r="K20" s="1">
-        <f>SUM(K3:K19)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="L20" s="1">
-        <f>SUM(L3:L19)</f>
+        <f t="shared" si="0"/>
         <v>60</v>
       </c>
       <c r="M20" s="1">
-        <f>SUM(M3:M19)</f>
+        <f t="shared" si="0"/>
         <v>1507</v>
       </c>
       <c r="N20" s="1">
-        <f>SUM(N3:N19)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="O20" s="1">
-        <f>SUM(O3:O19)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
       <c r="P20" s="1">
-        <f>SUM(P3:P19)</f>
+        <f t="shared" si="0"/>
         <v>1494</v>
       </c>
       <c r="Q20" s="1">
-        <f>SUM(Q3:Q19)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="R20" s="1">
-        <f>SUM(R3:R19)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
       <c r="S20" s="1">
-        <f>SUM(S3:S19)</f>
+        <f t="shared" si="0"/>
         <v>1494</v>
       </c>
       <c r="T20" s="1">
-        <f>SUM(T3:T19)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="U20" s="1">
-        <f>SUM(U3:U19)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
       <c r="V20" s="1">
-        <f>SUM(V3:V19)</f>
+        <f t="shared" si="0"/>
         <v>1951</v>
       </c>
       <c r="W20" s="1">
-        <f>SUM(W3:W19)</f>
+        <f t="shared" si="0"/>
         <v>80</v>
       </c>
       <c r="X20" s="1">
-        <f>SUM(X3:X19)</f>
+        <f t="shared" si="0"/>
         <v>84</v>
       </c>
       <c r="Y20" s="1">
-        <f>SUM(Y3:Y19)</f>
+        <f t="shared" si="0"/>
         <v>1768</v>
       </c>
       <c r="Z20" s="1">
-        <f>SUM(Z3:Z19)</f>
+        <f t="shared" si="0"/>
         <v>80</v>
       </c>
       <c r="AA20" s="1">
-        <f t="shared" ref="AA20" si="0">SUM(AA3:AA19)</f>
+        <f t="shared" ref="AA20" si="1">SUM(AA3:AA19)</f>
         <v>84</v>
       </c>
       <c r="AB20" s="1">
@@ -2289,13 +2326,13 @@
         <v>92</v>
       </c>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:30">
       <c r="P21">
         <f>P20-D20</f>
         <v>-167</v>
       </c>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:30">
       <c r="P22" s="2">
         <f>P21/D20</f>
         <v>-0.10054184226369657</v>
@@ -2303,6 +2340,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B3:B6"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="AB1:AD1"/>
@@ -2319,7 +2357,6 @@
     <mergeCell ref="P1:R1"/>
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="B18:B19"/>
-    <mergeCell ref="B3:B6"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2330,7 +2367,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02857098-9EF4-7A43-8BB2-8228CE41206A}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.28515625" customWidth="1"/>
     <col min="2" max="2" width="5.28515625" customWidth="1"/>
@@ -2341,42 +2378,43 @@
     <col min="7" max="7" width="6.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B1" s="5" t="s">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1"/>
+      <c r="B1" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5" t="s">
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>50</v>
       </c>
@@ -2390,7 +2428,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>52</v>
       </c>
@@ -2404,7 +2442,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>51</v>
       </c>
@@ -2418,7 +2456,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>53</v>
       </c>
@@ -2432,7 +2470,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>54</v>
       </c>
@@ -2455,7 +2493,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>55</v>
       </c>
@@ -2469,7 +2507,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
         <v>56</v>
       </c>
@@ -2483,7 +2521,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
         <v>57</v>
       </c>
@@ -2506,7 +2544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
         <v>58</v>
       </c>
@@ -2529,7 +2567,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -2543,7 +2581,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
         <v>60</v>
       </c>
@@ -2557,7 +2595,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
         <v>61</v>
       </c>
@@ -2580,7 +2618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7">
       <c r="A15" t="s">
         <v>62</v>
       </c>
@@ -2603,7 +2641,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
         <v>63</v>
       </c>
@@ -2626,7 +2664,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7">
       <c r="A17" t="s">
         <v>64</v>
       </c>
@@ -2640,7 +2678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7">
       <c r="B18" s="1">
         <f>SUM(B3:B17)</f>
         <v>1588</v>
@@ -2666,13 +2704,13 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7">
       <c r="E19">
         <f>E18-B18</f>
         <v>-752</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7">
       <c r="E20" s="2">
         <f>E19/B18</f>
         <v>-0.47355163727959698</v>
@@ -2690,7 +2728,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3446A6D4-E7A1-DE4F-AF79-3C1286851385}">
   <dimension ref="A1:P7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
     <col min="2" max="3" width="5.7109375" customWidth="1"/>
@@ -2705,84 +2743,85 @@
     <col min="16" max="16" width="6.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B1" s="5" t="s">
+    <row r="1" spans="1:16">
+      <c r="A1" s="1"/>
+      <c r="B1" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5" t="s">
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5" t="s">
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5" t="s">
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5" t="s">
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+    </row>
+    <row r="2" spans="1:16">
+      <c r="A2" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16">
       <c r="A3" t="s">
         <v>70</v>
       </c>
@@ -2832,7 +2871,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16">
       <c r="A4" t="s">
         <v>71</v>
       </c>
@@ -2882,7 +2921,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16">
       <c r="B5" s="1">
         <f t="shared" ref="B5:G5" si="0">SUM(B3:B4)</f>
         <v>991</v>
@@ -2944,13 +2983,13 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16">
       <c r="N6">
         <f>N5-B5</f>
         <v>-127</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16">
       <c r="N7" s="2">
         <f>N6/B5</f>
         <v>-0.12815338042381433</v>
@@ -2971,7 +3010,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2043A2D3-B79F-994A-8E5F-6CAF0A113206}">
   <dimension ref="A1:J35"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
     <col min="2" max="2" width="5.7109375" customWidth="1"/>
@@ -2985,25 +3024,25 @@
     <col min="10" max="10" width="6.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10">
       <c r="A1" s="1"/>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6" t="s">
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6" t="s">
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
         <v>76</v>
       </c>
@@ -3035,7 +3074,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -3067,7 +3106,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -3099,7 +3138,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="A5" t="s">
         <v>81</v>
       </c>
@@ -3131,7 +3170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="A6" t="s">
         <v>80</v>
       </c>
@@ -3163,7 +3202,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10">
       <c r="A7" t="s">
         <v>83</v>
       </c>
@@ -3195,7 +3234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10">
       <c r="A8" t="s">
         <v>82</v>
       </c>
@@ -3227,7 +3266,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10">
       <c r="A9" t="s">
         <v>84</v>
       </c>
@@ -3259,7 +3298,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10">
       <c r="A10" t="s">
         <v>85</v>
       </c>
@@ -3291,7 +3330,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10">
       <c r="A11" t="s">
         <v>86</v>
       </c>
@@ -3323,7 +3362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10">
       <c r="A12" t="s">
         <v>87</v>
       </c>
@@ -3355,7 +3394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10">
       <c r="A13" t="s">
         <v>88</v>
       </c>
@@ -3387,7 +3426,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10">
       <c r="A14" t="s">
         <v>89</v>
       </c>
@@ -3419,7 +3458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10">
       <c r="A15" s="3" t="s">
         <v>90</v>
       </c>
@@ -3451,7 +3490,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10">
       <c r="A16" s="3" t="s">
         <v>91</v>
       </c>
@@ -3483,7 +3522,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10">
       <c r="A17" s="3" t="s">
         <v>92</v>
       </c>
@@ -3515,7 +3554,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -3547,7 +3586,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10">
       <c r="A19" t="s">
         <v>94</v>
       </c>
@@ -3579,7 +3618,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10">
       <c r="A20" t="s">
         <v>95</v>
       </c>
@@ -3611,7 +3650,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10">
       <c r="A21" t="s">
         <v>96</v>
       </c>
@@ -3643,7 +3682,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10">
       <c r="B22" s="1">
         <f>SUM(B3:B21)</f>
         <v>2871</v>
@@ -3681,7 +3720,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10">
       <c r="A24" s="3" t="s">
         <v>94</v>
       </c>
@@ -3704,7 +3743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10">
       <c r="A25" s="3" t="s">
         <v>96</v>
       </c>
@@ -3727,7 +3766,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10">
       <c r="A26" s="3" t="s">
         <v>84</v>
       </c>
@@ -3750,7 +3789,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -3773,7 +3812,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10">
       <c r="A28" s="3" t="s">
         <v>87</v>
       </c>
@@ -3796,7 +3835,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10">
       <c r="A29" s="3" t="s">
         <v>97</v>
       </c>
@@ -3819,7 +3858,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10">
       <c r="A30" t="s">
         <v>98</v>
       </c>
@@ -3842,7 +3881,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10">
       <c r="A31" t="s">
         <v>99</v>
       </c>
@@ -3865,7 +3904,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10">
       <c r="A32" t="s">
         <v>100</v>
       </c>
@@ -3888,7 +3927,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:7">
       <c r="B33" s="1">
         <f>SUM(B24:B32)</f>
         <v>2082</v>
@@ -3914,13 +3953,13 @@
         <v>44</v>
       </c>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:7">
       <c r="E34">
         <f>E33-B33</f>
         <v>-292</v>
       </c>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:7">
       <c r="E35" s="2">
         <f>E34/B33</f>
         <v>-0.14024975984630164</v>
@@ -3934,4 +3973,444 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D0323DF-4A97-4C48-B3D4-92F5ADBE433C}">
+  <dimension ref="A1:R9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="5.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" s="1" customFormat="1">
+      <c r="C1" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+    </row>
+    <row r="2" spans="1:18" s="1" customFormat="1">
+      <c r="A2" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="36">
+      <c r="A3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>664</v>
+      </c>
+      <c r="E3">
+        <v>7</v>
+      </c>
+      <c r="F3">
+        <v>7</v>
+      </c>
+      <c r="G3">
+        <v>5</v>
+      </c>
+      <c r="H3">
+        <v>663</v>
+      </c>
+      <c r="I3">
+        <v>7</v>
+      </c>
+      <c r="J3">
+        <v>7</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
+      </c>
+      <c r="L3">
+        <v>231</v>
+      </c>
+      <c r="M3">
+        <v>7</v>
+      </c>
+      <c r="N3">
+        <v>5</v>
+      </c>
+      <c r="O3">
+        <v>5</v>
+      </c>
+      <c r="P3">
+        <v>231</v>
+      </c>
+      <c r="Q3">
+        <v>7</v>
+      </c>
+      <c r="R3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="36">
+      <c r="B4" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="K4">
+        <v>7</v>
+      </c>
+      <c r="L4">
+        <v>399</v>
+      </c>
+      <c r="M4">
+        <v>6</v>
+      </c>
+      <c r="N4">
+        <v>1</v>
+      </c>
+      <c r="O4">
+        <v>7</v>
+      </c>
+      <c r="P4">
+        <v>396</v>
+      </c>
+      <c r="Q4">
+        <v>6</v>
+      </c>
+      <c r="R4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18">
+      <c r="A5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="D5">
+        <v>62</v>
+      </c>
+      <c r="E5">
+        <v>6</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>6</v>
+      </c>
+      <c r="H5">
+        <v>62</v>
+      </c>
+      <c r="I5">
+        <v>6</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <v>6</v>
+      </c>
+      <c r="L5">
+        <v>62</v>
+      </c>
+      <c r="M5">
+        <v>6</v>
+      </c>
+      <c r="N5">
+        <v>2</v>
+      </c>
+      <c r="O5">
+        <v>6</v>
+      </c>
+      <c r="P5">
+        <v>60</v>
+      </c>
+      <c r="Q5">
+        <v>6</v>
+      </c>
+      <c r="R5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18">
+      <c r="A6" t="s">
+        <v>123</v>
+      </c>
+      <c r="C6">
+        <v>7</v>
+      </c>
+      <c r="D6">
+        <v>86</v>
+      </c>
+      <c r="E6">
+        <v>8</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>6</v>
+      </c>
+      <c r="H6">
+        <v>94</v>
+      </c>
+      <c r="I6">
+        <v>8</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="K6">
+        <v>6</v>
+      </c>
+      <c r="L6">
+        <v>94</v>
+      </c>
+      <c r="M6">
+        <v>8</v>
+      </c>
+      <c r="N6">
+        <v>2</v>
+      </c>
+      <c r="O6">
+        <v>6</v>
+      </c>
+      <c r="P6">
+        <v>93</v>
+      </c>
+      <c r="Q6">
+        <v>8</v>
+      </c>
+      <c r="R6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18">
+      <c r="A7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7">
+        <v>7</v>
+      </c>
+      <c r="D7">
+        <v>97</v>
+      </c>
+      <c r="E7">
+        <v>9</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>7</v>
+      </c>
+      <c r="H7">
+        <v>97</v>
+      </c>
+      <c r="I7">
+        <v>9</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7">
+        <v>7</v>
+      </c>
+      <c r="L7">
+        <v>97</v>
+      </c>
+      <c r="M7">
+        <v>9</v>
+      </c>
+      <c r="N7">
+        <v>1</v>
+      </c>
+      <c r="O7">
+        <v>7</v>
+      </c>
+      <c r="P7">
+        <v>96</v>
+      </c>
+      <c r="Q7">
+        <v>9</v>
+      </c>
+      <c r="R7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18">
+      <c r="C8" s="1">
+        <f>SUM(C3:C7)</f>
+        <v>25</v>
+      </c>
+      <c r="D8" s="1">
+        <f t="shared" ref="D8:F8" si="0">SUM(D3:D7)</f>
+        <v>909</v>
+      </c>
+      <c r="E8" s="1">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="F8" s="1">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="G8" s="1">
+        <f>SUM(G3:G7)</f>
+        <v>24</v>
+      </c>
+      <c r="H8" s="1">
+        <f>SUM(H3:H7)</f>
+        <v>916</v>
+      </c>
+      <c r="I8" s="1">
+        <f>SUM(I3:I7)</f>
+        <v>30</v>
+      </c>
+      <c r="J8" s="1">
+        <f>SUM(J3:J7)</f>
+        <v>12</v>
+      </c>
+      <c r="K8" s="1">
+        <f>SUM(K3:K7)</f>
+        <v>31</v>
+      </c>
+      <c r="L8" s="1">
+        <f>SUM(L3:L7)</f>
+        <v>883</v>
+      </c>
+      <c r="M8" s="1">
+        <f>SUM(M3:M7)</f>
+        <v>36</v>
+      </c>
+      <c r="N8" s="1">
+        <f>SUM(N3:N7)</f>
+        <v>11</v>
+      </c>
+      <c r="O8" s="1">
+        <f t="shared" ref="O8:R8" si="1">SUM(O3:O7)</f>
+        <v>31</v>
+      </c>
+      <c r="P8" s="1">
+        <f t="shared" si="1"/>
+        <v>876</v>
+      </c>
+      <c r="Q8" s="1">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="R8" s="1">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18">
+      <c r="H9" s="9">
+        <f>(H8-D8)/D8</f>
+        <v>7.7007700770077006E-3</v>
+      </c>
+      <c r="L9" s="9">
+        <f>(L8-D8)/D8</f>
+        <v>-2.8602860286028604E-2</v>
+      </c>
+      <c r="P9" s="9">
+        <f>(P8-D8)/D8</f>
+        <v>-3.6303630363036306E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="C1:F1"/>
+    <mergeCell ref="G1:J1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="O1:R1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added a mixed formatting console output method
</commit_message>
<xml_diff>
--- a/ILSIze.xlsx
+++ b/ILSIze.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A783A36-9A09-6242-8FD2-271EA593A5D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CF386F-7C6D-4F40-BF95-BF158D918346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14400" firstSheet="1" activeTab="7" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
+    <workbookView xWindow="0" yWindow="6260" windowWidth="25600" windowHeight="8620" firstSheet="1" activeTab="7" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
   </bookViews>
   <sheets>
     <sheet name="Chemistry.cs" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="131">
   <si>
     <t>Méthode</t>
   </si>
@@ -424,6 +424,18 @@
   </si>
   <si>
     <t>TRegression lrp, string numberFormat, bool checkBiases, CultureInfo ciCu, TStorage b, TStorage sr, TStorage studentLawValue</t>
+  </si>
+  <si>
+    <t>Iteration 6</t>
+  </si>
+  <si>
+    <t>Iteration 7</t>
+  </si>
+  <si>
+    <t>Iteration 8</t>
+  </si>
+  <si>
+    <t>Format / OutputLine</t>
   </si>
 </sst>
 </file>
@@ -518,18 +530,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -827,16 +839,16 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1"/>
-      <c r="B1" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7" t="s">
+      <c r="B1" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
@@ -1395,51 +1407,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" s="1" customFormat="1">
-      <c r="D1" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7" t="s">
+      <c r="D1" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7" t="s">
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7" t="s">
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7" t="s">
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-      <c r="S1" s="7" t="s">
+      <c r="Q1" s="8"/>
+      <c r="R1" s="8"/>
+      <c r="S1" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="T1" s="7"/>
-      <c r="U1" s="7"/>
-      <c r="V1" s="7" t="s">
+      <c r="T1" s="8"/>
+      <c r="U1" s="8"/>
+      <c r="V1" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="W1" s="7"/>
-      <c r="X1" s="7"/>
-      <c r="Y1" s="7" t="s">
+      <c r="W1" s="8"/>
+      <c r="X1" s="8"/>
+      <c r="Y1" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="Z1" s="7"/>
-      <c r="AA1" s="7"/>
-      <c r="AB1" s="7" t="s">
+      <c r="Z1" s="8"/>
+      <c r="AA1" s="8"/>
+      <c r="AB1" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="AC1" s="7"/>
-      <c r="AD1" s="7"/>
+      <c r="AC1" s="8"/>
+      <c r="AD1" s="8"/>
     </row>
     <row r="2" spans="1:30" s="1" customFormat="1">
       <c r="A2" s="1" t="s">
@@ -1534,10 +1546,10 @@
       </c>
     </row>
     <row r="3" spans="1:30">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="9" t="s">
         <v>41</v>
       </c>
       <c r="C3" t="s">
@@ -1626,8 +1638,8 @@
       </c>
     </row>
     <row r="4" spans="1:30">
-      <c r="A4" s="8"/>
-      <c r="B4" s="6"/>
+      <c r="A4" s="10"/>
+      <c r="B4" s="9"/>
       <c r="C4" t="s">
         <v>113</v>
       </c>
@@ -1642,8 +1654,8 @@
       </c>
     </row>
     <row r="5" spans="1:30">
-      <c r="A5" s="8"/>
-      <c r="B5" s="6"/>
+      <c r="A5" s="10"/>
+      <c r="B5" s="9"/>
       <c r="C5" t="s">
         <v>43</v>
       </c>
@@ -1730,8 +1742,8 @@
       </c>
     </row>
     <row r="6" spans="1:30">
-      <c r="A6" s="8"/>
-      <c r="B6" s="6"/>
+      <c r="A6" s="10"/>
+      <c r="B6" s="9"/>
       <c r="C6" t="s">
         <v>114</v>
       </c>
@@ -1746,7 +1758,7 @@
       </c>
     </row>
     <row r="7" spans="1:30">
-      <c r="A7" s="8"/>
+      <c r="A7" s="10"/>
       <c r="B7" s="5" t="s">
         <v>115</v>
       </c>
@@ -1761,8 +1773,8 @@
       </c>
     </row>
     <row r="8" spans="1:30">
-      <c r="A8" s="8"/>
-      <c r="B8" s="6" t="s">
+      <c r="A8" s="10"/>
+      <c r="B8" s="9" t="s">
         <v>116</v>
       </c>
       <c r="C8" t="s">
@@ -1779,8 +1791,8 @@
       </c>
     </row>
     <row r="9" spans="1:30">
-      <c r="A9" s="8"/>
-      <c r="B9" s="6"/>
+      <c r="A9" s="10"/>
+      <c r="B9" s="9"/>
       <c r="C9" t="s">
         <v>118</v>
       </c>
@@ -1795,8 +1807,8 @@
       </c>
     </row>
     <row r="10" spans="1:30">
-      <c r="A10" s="8"/>
-      <c r="B10" s="6" t="s">
+      <c r="A10" s="10"/>
+      <c r="B10" s="9" t="s">
         <v>104</v>
       </c>
       <c r="C10" t="s">
@@ -1813,8 +1825,8 @@
       </c>
     </row>
     <row r="11" spans="1:30">
-      <c r="A11" s="8"/>
-      <c r="B11" s="6"/>
+      <c r="A11" s="10"/>
+      <c r="B11" s="9"/>
       <c r="C11" t="s">
         <v>114</v>
       </c>
@@ -1829,10 +1841,10 @@
       </c>
     </row>
     <row r="12" spans="1:30">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="9" t="s">
         <v>41</v>
       </c>
       <c r="C12" s="4" t="s">
@@ -1867,8 +1879,8 @@
       </c>
     </row>
     <row r="13" spans="1:30">
-      <c r="A13" s="8"/>
-      <c r="B13" s="6"/>
+      <c r="A13" s="10"/>
+      <c r="B13" s="9"/>
       <c r="C13" t="s">
         <v>42</v>
       </c>
@@ -1955,8 +1967,8 @@
       </c>
     </row>
     <row r="14" spans="1:30">
-      <c r="A14" s="8"/>
-      <c r="B14" s="6"/>
+      <c r="A14" s="10"/>
+      <c r="B14" s="9"/>
       <c r="C14" s="4" t="s">
         <v>105</v>
       </c>
@@ -1989,8 +2001,8 @@
       </c>
     </row>
     <row r="15" spans="1:30">
-      <c r="A15" s="8"/>
-      <c r="B15" s="6"/>
+      <c r="A15" s="10"/>
+      <c r="B15" s="9"/>
       <c r="C15" t="s">
         <v>43</v>
       </c>
@@ -2077,8 +2089,8 @@
       </c>
     </row>
     <row r="16" spans="1:30">
-      <c r="A16" s="8"/>
-      <c r="B16" s="6" t="s">
+      <c r="A16" s="10"/>
+      <c r="B16" s="9" t="s">
         <v>103</v>
       </c>
       <c r="C16" t="s">
@@ -2113,8 +2125,8 @@
       </c>
     </row>
     <row r="17" spans="1:30">
-      <c r="A17" s="8"/>
-      <c r="B17" s="6"/>
+      <c r="A17" s="10"/>
+      <c r="B17" s="9"/>
       <c r="C17" t="s">
         <v>109</v>
       </c>
@@ -2147,8 +2159,8 @@
       </c>
     </row>
     <row r="18" spans="1:30">
-      <c r="A18" s="8"/>
-      <c r="B18" s="6" t="s">
+      <c r="A18" s="10"/>
+      <c r="B18" s="9" t="s">
         <v>104</v>
       </c>
       <c r="C18" t="s">
@@ -2183,8 +2195,8 @@
       </c>
     </row>
     <row r="19" spans="1:30">
-      <c r="A19" s="8"/>
-      <c r="B19" s="6"/>
+      <c r="A19" s="10"/>
+      <c r="B19" s="9"/>
       <c r="C19" t="s">
         <v>109</v>
       </c>
@@ -2340,11 +2352,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B3:B6"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="AB1:AD1"/>
-    <mergeCell ref="Y1:AA1"/>
     <mergeCell ref="A12:A19"/>
     <mergeCell ref="B12:B15"/>
     <mergeCell ref="V1:X1"/>
@@ -2357,6 +2364,11 @@
     <mergeCell ref="P1:R1"/>
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="B18:B19"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="AB1:AD1"/>
+    <mergeCell ref="Y1:AA1"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2380,16 +2392,16 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1"/>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7" t="s">
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
@@ -2745,31 +2757,31 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" s="1"/>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7" t="s">
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7" t="s">
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7" t="s">
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7" t="s">
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8"/>
     </row>
     <row r="2" spans="1:16">
       <c r="A2" s="1" t="s">
@@ -3026,21 +3038,21 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="1"/>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7" t="s">
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7" t="s">
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
@@ -3977,7 +3989,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D0323DF-4A97-4C48-B3D4-92F5ADBE433C}">
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:AH10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
@@ -3996,35 +4008,75 @@
     <col min="15" max="15" width="4.140625" bestFit="1" customWidth="1"/>
     <col min="16" max="17" width="5.140625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="5" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="5.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="1" customFormat="1">
-      <c r="C1" s="7" t="s">
+    <row r="1" spans="1:34" s="1" customFormat="1">
+      <c r="C1" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7" t="s">
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7" t="s">
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7" t="s">
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-    </row>
-    <row r="2" spans="1:18" s="1" customFormat="1">
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
+      <c r="R1" s="8"/>
+      <c r="S1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="T1" s="8"/>
+      <c r="U1" s="8"/>
+      <c r="V1" s="8"/>
+      <c r="W1" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="X1" s="8"/>
+      <c r="Y1" s="8"/>
+      <c r="Z1" s="8"/>
+      <c r="AA1" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB1" s="8"/>
+      <c r="AC1" s="8"/>
+      <c r="AD1" s="8"/>
+      <c r="AE1" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="AF1" s="8"/>
+      <c r="AG1" s="8"/>
+      <c r="AH1" s="8"/>
+    </row>
+    <row r="2" spans="1:34" s="1" customFormat="1">
       <c r="A2" s="1" t="s">
         <v>76</v>
       </c>
@@ -4079,12 +4131,60 @@
       <c r="R2" s="1" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="3" spans="1:18" ht="36">
+      <c r="S2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:34" ht="36">
       <c r="A3" t="s">
         <v>120</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="7" t="s">
         <v>125</v>
       </c>
       <c r="C3">
@@ -4135,9 +4235,57 @@
       <c r="R3">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" ht="36">
-      <c r="B4" s="10" t="s">
+      <c r="S3">
+        <v>5</v>
+      </c>
+      <c r="T3">
+        <v>231</v>
+      </c>
+      <c r="U3">
+        <v>7</v>
+      </c>
+      <c r="V3">
+        <v>5</v>
+      </c>
+      <c r="W3">
+        <v>5</v>
+      </c>
+      <c r="X3">
+        <v>220</v>
+      </c>
+      <c r="Y3">
+        <v>7</v>
+      </c>
+      <c r="Z3">
+        <v>5</v>
+      </c>
+      <c r="AA3">
+        <v>5</v>
+      </c>
+      <c r="AB3">
+        <v>220</v>
+      </c>
+      <c r="AC3">
+        <v>8</v>
+      </c>
+      <c r="AD3">
+        <v>4</v>
+      </c>
+      <c r="AE3">
+        <v>5</v>
+      </c>
+      <c r="AF3">
+        <v>215</v>
+      </c>
+      <c r="AG3">
+        <v>8</v>
+      </c>
+      <c r="AH3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:34" ht="36">
+      <c r="B4" s="7" t="s">
         <v>126</v>
       </c>
       <c r="K4">
@@ -4164,8 +4312,56 @@
       <c r="R4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:18">
+      <c r="S4">
+        <v>7</v>
+      </c>
+      <c r="T4">
+        <v>396</v>
+      </c>
+      <c r="U4">
+        <v>6</v>
+      </c>
+      <c r="V4">
+        <v>1</v>
+      </c>
+      <c r="W4">
+        <v>7</v>
+      </c>
+      <c r="X4">
+        <v>377</v>
+      </c>
+      <c r="Y4">
+        <v>6</v>
+      </c>
+      <c r="Z4">
+        <v>1</v>
+      </c>
+      <c r="AA4">
+        <v>7</v>
+      </c>
+      <c r="AB4">
+        <v>342</v>
+      </c>
+      <c r="AC4">
+        <v>6</v>
+      </c>
+      <c r="AD4">
+        <v>1</v>
+      </c>
+      <c r="AE4">
+        <v>7</v>
+      </c>
+      <c r="AF4">
+        <v>337</v>
+      </c>
+      <c r="AG4">
+        <v>7</v>
+      </c>
+      <c r="AH4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:34">
       <c r="A5" t="s">
         <v>122</v>
       </c>
@@ -4217,8 +4413,56 @@
       <c r="R5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:18">
+      <c r="S5">
+        <v>6</v>
+      </c>
+      <c r="T5">
+        <v>60</v>
+      </c>
+      <c r="U5">
+        <v>6</v>
+      </c>
+      <c r="V5">
+        <v>2</v>
+      </c>
+      <c r="W5">
+        <v>6</v>
+      </c>
+      <c r="X5">
+        <v>60</v>
+      </c>
+      <c r="Y5">
+        <v>6</v>
+      </c>
+      <c r="Z5">
+        <v>2</v>
+      </c>
+      <c r="AA5">
+        <v>6</v>
+      </c>
+      <c r="AB5">
+        <v>60</v>
+      </c>
+      <c r="AC5">
+        <v>6</v>
+      </c>
+      <c r="AD5">
+        <v>2</v>
+      </c>
+      <c r="AE5">
+        <v>6</v>
+      </c>
+      <c r="AF5">
+        <v>60</v>
+      </c>
+      <c r="AG5">
+        <v>6</v>
+      </c>
+      <c r="AH5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:34">
       <c r="A6" t="s">
         <v>123</v>
       </c>
@@ -4270,8 +4514,56 @@
       <c r="R6">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="1:18">
+      <c r="S6">
+        <v>6</v>
+      </c>
+      <c r="T6">
+        <v>129</v>
+      </c>
+      <c r="U6">
+        <v>8</v>
+      </c>
+      <c r="V6">
+        <v>2</v>
+      </c>
+      <c r="W6">
+        <v>6</v>
+      </c>
+      <c r="X6">
+        <v>115</v>
+      </c>
+      <c r="Y6">
+        <v>8</v>
+      </c>
+      <c r="Z6">
+        <v>2</v>
+      </c>
+      <c r="AA6">
+        <v>6</v>
+      </c>
+      <c r="AB6">
+        <v>116</v>
+      </c>
+      <c r="AC6">
+        <v>8</v>
+      </c>
+      <c r="AD6">
+        <v>2</v>
+      </c>
+      <c r="AE6">
+        <v>6</v>
+      </c>
+      <c r="AF6">
+        <v>111</v>
+      </c>
+      <c r="AG6">
+        <v>7</v>
+      </c>
+      <c r="AH6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:34">
       <c r="A7" t="s">
         <v>124</v>
       </c>
@@ -4323,93 +4615,250 @@
       <c r="R7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:18">
-      <c r="C8" s="1">
-        <f>SUM(C3:C7)</f>
+      <c r="S7">
+        <v>7</v>
+      </c>
+      <c r="T7">
+        <v>132</v>
+      </c>
+      <c r="U7">
+        <v>9</v>
+      </c>
+      <c r="V7">
+        <v>1</v>
+      </c>
+      <c r="W7">
+        <v>7</v>
+      </c>
+      <c r="X7">
+        <v>132</v>
+      </c>
+      <c r="Y7">
+        <v>9</v>
+      </c>
+      <c r="Z7">
+        <v>1</v>
+      </c>
+      <c r="AA7">
+        <v>7</v>
+      </c>
+      <c r="AB7">
+        <v>132</v>
+      </c>
+      <c r="AC7">
+        <v>9</v>
+      </c>
+      <c r="AD7">
+        <v>1</v>
+      </c>
+      <c r="AE7">
+        <v>7</v>
+      </c>
+      <c r="AF7">
+        <v>132</v>
+      </c>
+      <c r="AG7">
+        <v>9</v>
+      </c>
+      <c r="AH7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:34">
+      <c r="A8" t="s">
+        <v>130</v>
+      </c>
+      <c r="W8">
+        <v>4</v>
+      </c>
+      <c r="X8">
+        <v>76</v>
+      </c>
+      <c r="Y8">
+        <v>5</v>
+      </c>
+      <c r="Z8">
+        <v>4</v>
+      </c>
+      <c r="AA8">
+        <v>4</v>
+      </c>
+      <c r="AB8">
+        <v>89</v>
+      </c>
+      <c r="AC8">
+        <v>5</v>
+      </c>
+      <c r="AD8">
+        <v>3</v>
+      </c>
+      <c r="AE8">
+        <v>4</v>
+      </c>
+      <c r="AF8">
+        <v>94</v>
+      </c>
+      <c r="AG8">
+        <v>5</v>
+      </c>
+      <c r="AH8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:34">
+      <c r="C9" s="1">
+        <f>SUM(C3:C8)</f>
         <v>25</v>
       </c>
-      <c r="D8" s="1">
-        <f t="shared" ref="D8:F8" si="0">SUM(D3:D7)</f>
+      <c r="D9" s="1">
+        <f t="shared" ref="D9:Z9" si="0">SUM(D3:D8)</f>
         <v>909</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E9" s="1">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F9" s="1">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="G8" s="1">
-        <f>SUM(G3:G7)</f>
+      <c r="G9" s="1">
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="H8" s="1">
-        <f>SUM(H3:H7)</f>
+      <c r="H9" s="1">
+        <f t="shared" si="0"/>
         <v>916</v>
       </c>
-      <c r="I8" s="1">
-        <f>SUM(I3:I7)</f>
+      <c r="I9" s="1">
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="J8" s="1">
-        <f>SUM(J3:J7)</f>
+      <c r="J9" s="1">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="K8" s="1">
-        <f>SUM(K3:K7)</f>
+      <c r="K9" s="1">
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="L8" s="1">
-        <f>SUM(L3:L7)</f>
+      <c r="L9" s="1">
+        <f t="shared" si="0"/>
         <v>883</v>
       </c>
-      <c r="M8" s="1">
-        <f>SUM(M3:M7)</f>
+      <c r="M9" s="1">
+        <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="N8" s="1">
-        <f>SUM(N3:N7)</f>
+      <c r="N9" s="1">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="O8" s="1">
-        <f t="shared" ref="O8:R8" si="1">SUM(O3:O7)</f>
+      <c r="O9" s="1">
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="P8" s="1">
-        <f t="shared" si="1"/>
+      <c r="P9" s="1">
+        <f t="shared" si="0"/>
         <v>876</v>
       </c>
-      <c r="Q8" s="1">
-        <f t="shared" si="1"/>
+      <c r="Q9" s="1">
+        <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="R8" s="1">
-        <f t="shared" si="1"/>
+      <c r="R9" s="1">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="1:18">
-      <c r="H9" s="9">
-        <f>(H8-D8)/D8</f>
+      <c r="S9" s="1">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+      <c r="T9" s="1">
+        <f t="shared" si="0"/>
+        <v>948</v>
+      </c>
+      <c r="U9" s="1">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+      <c r="V9" s="1">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="W9" s="1">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+      <c r="X9" s="1">
+        <f t="shared" si="0"/>
+        <v>980</v>
+      </c>
+      <c r="Y9" s="1">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+      <c r="Z9" s="1">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="AA9" s="1">
+        <f t="shared" ref="AA9" si="1">SUM(AA3:AA8)</f>
+        <v>35</v>
+      </c>
+      <c r="AB9" s="1">
+        <f t="shared" ref="AB9" si="2">SUM(AB3:AB8)</f>
+        <v>959</v>
+      </c>
+      <c r="AC9" s="1">
+        <f t="shared" ref="AC9" si="3">SUM(AC3:AC8)</f>
+        <v>42</v>
+      </c>
+      <c r="AD9" s="1">
+        <f t="shared" ref="AD9" si="4">SUM(AD3:AD8)</f>
+        <v>13</v>
+      </c>
+      <c r="AE9" s="1">
+        <f t="shared" ref="AE9" si="5">SUM(AE3:AE8)</f>
+        <v>35</v>
+      </c>
+      <c r="AF9" s="1">
+        <f t="shared" ref="AF9" si="6">SUM(AF3:AF8)</f>
+        <v>949</v>
+      </c>
+      <c r="AG9" s="1">
+        <f t="shared" ref="AG9" si="7">SUM(AG3:AG8)</f>
+        <v>42</v>
+      </c>
+      <c r="AH9" s="1">
+        <f t="shared" ref="AH9" si="8">SUM(AH3:AH8)</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:34">
+      <c r="H10" s="6">
+        <f>(H9-D9)/D9</f>
         <v>7.7007700770077006E-3</v>
       </c>
-      <c r="L9" s="9">
-        <f>(L8-D8)/D8</f>
+      <c r="L10" s="6">
+        <f>(L9-D9)/D9</f>
         <v>-2.8602860286028604E-2</v>
       </c>
-      <c r="P9" s="9">
-        <f>(P8-D8)/D8</f>
+      <c r="P10" s="6">
+        <f>(P9-D9)/D9</f>
         <v>-3.6303630363036306E-2</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="8">
+    <mergeCell ref="W1:Z1"/>
+    <mergeCell ref="AA1:AD1"/>
+    <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="G1:J1"/>
     <mergeCell ref="K1:N1"/>
     <mergeCell ref="O1:R1"/>
+    <mergeCell ref="S1:V1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Saved 745 IL bytes with shorter Console.Write calls
Creating an array, such as ones for variable length arguments, is heavy on IL code
</commit_message>
<xml_diff>
--- a/ILSIze.xlsx
+++ b/ILSIze.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CF386F-7C6D-4F40-BF95-BF158D918346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE13BD5D-41AD-8B45-8516-BC1AD0D1DFDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="6260" windowWidth="25600" windowHeight="8620" firstSheet="1" activeTab="7" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14420" firstSheet="2" activeTab="8" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
   </bookViews>
   <sheets>
     <sheet name="Chemistry.cs" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="Matrix.cs" sheetId="6" r:id="rId6"/>
     <sheet name="ExtraMath_decimal.cs" sheetId="7" r:id="rId7"/>
     <sheet name="void OutputLinearRegression2" sheetId="8" r:id="rId8"/>
+    <sheet name="Console.Write" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="158">
   <si>
     <t>Méthode</t>
   </si>
@@ -436,6 +437,87 @@
   </si>
   <si>
     <t>Format / OutputLine</t>
+  </si>
+  <si>
+    <t>ChemistryTest.Run</t>
+  </si>
+  <si>
+    <t>DigitTest.Run</t>
+  </si>
+  <si>
+    <t>LinearRegressionTest.Run</t>
+  </si>
+  <si>
+    <t>LinearRegressionTest.OutputBenchResults</t>
+  </si>
+  <si>
+    <t>LinearRegressionTest.InterpolateMolecularWeight</t>
+  </si>
+  <si>
+    <t>LinearRegressionTest.OutputYExtrapolation</t>
+  </si>
+  <si>
+    <t>LinearRegressionTest.OutputRegression</t>
+  </si>
+  <si>
+    <t>MatrixTest.OutputExample89</t>
+  </si>
+  <si>
+    <t>NormalLawTest.OutputNormalIntegral(double…</t>
+  </si>
+  <si>
+    <t>NormalLawTest.OutputNormalIntegral(Decimal…</t>
+  </si>
+  <si>
+    <t>NormalLawTest.OutputNormalIntegral&lt;T&gt;</t>
+  </si>
+  <si>
+    <t>NormalLawTest.BeginOutputNormalIntegral</t>
+  </si>
+  <si>
+    <t>NormalLawTest.EndOutputNormalIntegral</t>
+  </si>
+  <si>
+    <t>NormalLawTest.FindBestIterationCountForNormalLawIntegral(…double…</t>
+  </si>
+  <si>
+    <t>Iterations</t>
+  </si>
+  <si>
+    <t>Before</t>
+  </si>
+  <si>
+    <t>After</t>
+  </si>
+  <si>
+    <t>Relative</t>
+  </si>
+  <si>
+    <t>NormalLawTest.FindBestIterationCountForNormalLawIntegral(…Decimal…</t>
+  </si>
+  <si>
+    <t>NormalLawTest.FindMacLaurinBreakpointForNormalLawIntegral</t>
+  </si>
+  <si>
+    <t>NormalLawTest.OutputProbitEstimate</t>
+  </si>
+  <si>
+    <t>NormalLawTest.LogisticModel</t>
+  </si>
+  <si>
+    <t>NormalLawTest.EvaluateLogisticModel</t>
+  </si>
+  <si>
+    <t>Program.RunSingleDemo</t>
+  </si>
+  <si>
+    <t>VectorTest.Run</t>
+  </si>
+  <si>
+    <t>VectorTest.ShowcaseExample69</t>
+  </si>
+  <si>
+    <t>VectorTest.Example69Console</t>
   </si>
 </sst>
 </file>
@@ -521,7 +603,7 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -538,11 +620,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1546,10 +1629,10 @@
       </c>
     </row>
     <row r="3" spans="1:30">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="10" t="s">
         <v>41</v>
       </c>
       <c r="C3" t="s">
@@ -1638,8 +1721,8 @@
       </c>
     </row>
     <row r="4" spans="1:30">
-      <c r="A4" s="10"/>
-      <c r="B4" s="9"/>
+      <c r="A4" s="9"/>
+      <c r="B4" s="10"/>
       <c r="C4" t="s">
         <v>113</v>
       </c>
@@ -1654,8 +1737,8 @@
       </c>
     </row>
     <row r="5" spans="1:30">
-      <c r="A5" s="10"/>
-      <c r="B5" s="9"/>
+      <c r="A5" s="9"/>
+      <c r="B5" s="10"/>
       <c r="C5" t="s">
         <v>43</v>
       </c>
@@ -1742,8 +1825,8 @@
       </c>
     </row>
     <row r="6" spans="1:30">
-      <c r="A6" s="10"/>
-      <c r="B6" s="9"/>
+      <c r="A6" s="9"/>
+      <c r="B6" s="10"/>
       <c r="C6" t="s">
         <v>114</v>
       </c>
@@ -1758,7 +1841,7 @@
       </c>
     </row>
     <row r="7" spans="1:30">
-      <c r="A7" s="10"/>
+      <c r="A7" s="9"/>
       <c r="B7" s="5" t="s">
         <v>115</v>
       </c>
@@ -1773,8 +1856,8 @@
       </c>
     </row>
     <row r="8" spans="1:30">
-      <c r="A8" s="10"/>
-      <c r="B8" s="9" t="s">
+      <c r="A8" s="9"/>
+      <c r="B8" s="10" t="s">
         <v>116</v>
       </c>
       <c r="C8" t="s">
@@ -1791,8 +1874,8 @@
       </c>
     </row>
     <row r="9" spans="1:30">
-      <c r="A9" s="10"/>
-      <c r="B9" s="9"/>
+      <c r="A9" s="9"/>
+      <c r="B9" s="10"/>
       <c r="C9" t="s">
         <v>118</v>
       </c>
@@ -1807,8 +1890,8 @@
       </c>
     </row>
     <row r="10" spans="1:30">
-      <c r="A10" s="10"/>
-      <c r="B10" s="9" t="s">
+      <c r="A10" s="9"/>
+      <c r="B10" s="10" t="s">
         <v>104</v>
       </c>
       <c r="C10" t="s">
@@ -1825,8 +1908,8 @@
       </c>
     </row>
     <row r="11" spans="1:30">
-      <c r="A11" s="10"/>
-      <c r="B11" s="9"/>
+      <c r="A11" s="9"/>
+      <c r="B11" s="10"/>
       <c r="C11" t="s">
         <v>114</v>
       </c>
@@ -1841,10 +1924,10 @@
       </c>
     </row>
     <row r="12" spans="1:30">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="10" t="s">
         <v>41</v>
       </c>
       <c r="C12" s="4" t="s">
@@ -1879,8 +1962,8 @@
       </c>
     </row>
     <row r="13" spans="1:30">
-      <c r="A13" s="10"/>
-      <c r="B13" s="9"/>
+      <c r="A13" s="9"/>
+      <c r="B13" s="10"/>
       <c r="C13" t="s">
         <v>42</v>
       </c>
@@ -1967,8 +2050,8 @@
       </c>
     </row>
     <row r="14" spans="1:30">
-      <c r="A14" s="10"/>
-      <c r="B14" s="9"/>
+      <c r="A14" s="9"/>
+      <c r="B14" s="10"/>
       <c r="C14" s="4" t="s">
         <v>105</v>
       </c>
@@ -2001,8 +2084,8 @@
       </c>
     </row>
     <row r="15" spans="1:30">
-      <c r="A15" s="10"/>
-      <c r="B15" s="9"/>
+      <c r="A15" s="9"/>
+      <c r="B15" s="10"/>
       <c r="C15" t="s">
         <v>43</v>
       </c>
@@ -2089,8 +2172,8 @@
       </c>
     </row>
     <row r="16" spans="1:30">
-      <c r="A16" s="10"/>
-      <c r="B16" s="9" t="s">
+      <c r="A16" s="9"/>
+      <c r="B16" s="10" t="s">
         <v>103</v>
       </c>
       <c r="C16" t="s">
@@ -2125,8 +2208,8 @@
       </c>
     </row>
     <row r="17" spans="1:30">
-      <c r="A17" s="10"/>
-      <c r="B17" s="9"/>
+      <c r="A17" s="9"/>
+      <c r="B17" s="10"/>
       <c r="C17" t="s">
         <v>109</v>
       </c>
@@ -2159,8 +2242,8 @@
       </c>
     </row>
     <row r="18" spans="1:30">
-      <c r="A18" s="10"/>
-      <c r="B18" s="9" t="s">
+      <c r="A18" s="9"/>
+      <c r="B18" s="10" t="s">
         <v>104</v>
       </c>
       <c r="C18" t="s">
@@ -2195,8 +2278,8 @@
       </c>
     </row>
     <row r="19" spans="1:30">
-      <c r="A19" s="10"/>
-      <c r="B19" s="9"/>
+      <c r="A19" s="9"/>
+      <c r="B19" s="10"/>
       <c r="C19" t="s">
         <v>109</v>
       </c>
@@ -2352,6 +2435,8 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="AB1:AD1"/>
+    <mergeCell ref="Y1:AA1"/>
     <mergeCell ref="A12:A19"/>
     <mergeCell ref="B12:B15"/>
     <mergeCell ref="V1:X1"/>
@@ -2367,8 +2452,6 @@
     <mergeCell ref="B3:B6"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="B10:B11"/>
-    <mergeCell ref="AB1:AD1"/>
-    <mergeCell ref="Y1:AA1"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4862,4 +4945,720 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2CB8517-AE04-3E4E-B5BB-4C5D322F3AE8}">
+  <dimension ref="A1:K24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="1" width="54" customWidth="1"/>
+    <col min="2" max="4" width="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5" customWidth="1"/>
+    <col min="8" max="9" width="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="H1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B2">
+        <v>3023</v>
+      </c>
+      <c r="C2">
+        <v>3009</v>
+      </c>
+      <c r="D2">
+        <v>2997</v>
+      </c>
+      <c r="E2">
+        <v>2949</v>
+      </c>
+      <c r="F2">
+        <v>2903</v>
+      </c>
+      <c r="H2">
+        <f>B2</f>
+        <v>3023</v>
+      </c>
+      <c r="I2">
+        <f>MIN(C2:F2)</f>
+        <v>2903</v>
+      </c>
+      <c r="J2" s="11">
+        <f>I2-H2</f>
+        <v>-120</v>
+      </c>
+      <c r="K2" s="6">
+        <f>J2/H2</f>
+        <v>-3.9695666556400923E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3">
+        <v>1413</v>
+      </c>
+      <c r="C3">
+        <v>1389</v>
+      </c>
+      <c r="D3">
+        <v>1367</v>
+      </c>
+      <c r="E3">
+        <v>1364</v>
+      </c>
+      <c r="H3">
+        <f>B3</f>
+        <v>1413</v>
+      </c>
+      <c r="I3">
+        <f t="shared" ref="I3:I9" si="0">MIN(C3:F3)</f>
+        <v>1364</v>
+      </c>
+      <c r="J3" s="11">
+        <f>I3-H3</f>
+        <v>-49</v>
+      </c>
+      <c r="K3" s="6">
+        <f t="shared" ref="K3:K4" si="1">J3/H3</f>
+        <v>-3.4677990092002828E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4">
+        <v>10094</v>
+      </c>
+      <c r="C4">
+        <v>10056</v>
+      </c>
+      <c r="D4">
+        <v>10025</v>
+      </c>
+      <c r="H4">
+        <f>B4</f>
+        <v>10094</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="0"/>
+        <v>10025</v>
+      </c>
+      <c r="J4" s="11">
+        <f>I4-H4</f>
+        <v>-69</v>
+      </c>
+      <c r="K4" s="6">
+        <f t="shared" si="1"/>
+        <v>-6.8357440063403999E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" t="s">
+        <v>134</v>
+      </c>
+      <c r="B5">
+        <v>74</v>
+      </c>
+      <c r="C5">
+        <v>69</v>
+      </c>
+      <c r="H5">
+        <f>B5</f>
+        <v>74</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="0"/>
+        <v>69</v>
+      </c>
+      <c r="J5" s="11">
+        <f>I5-H5</f>
+        <v>-5</v>
+      </c>
+      <c r="K5" s="6">
+        <f t="shared" ref="K5:K10" si="2">J5/H5</f>
+        <v>-6.7567567567567571E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B6">
+        <v>142</v>
+      </c>
+      <c r="C6">
+        <v>125</v>
+      </c>
+      <c r="H6">
+        <f>B6</f>
+        <v>142</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="0"/>
+        <v>125</v>
+      </c>
+      <c r="J6" s="11">
+        <f>I6-H6</f>
+        <v>-17</v>
+      </c>
+      <c r="K6" s="6">
+        <f t="shared" si="2"/>
+        <v>-0.11971830985915492</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B7">
+        <v>146</v>
+      </c>
+      <c r="C7">
+        <v>133</v>
+      </c>
+      <c r="H7">
+        <f>B7</f>
+        <v>146</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="0"/>
+        <v>133</v>
+      </c>
+      <c r="J7" s="11">
+        <f>I7-H7</f>
+        <v>-13</v>
+      </c>
+      <c r="K7" s="6">
+        <f t="shared" si="2"/>
+        <v>-8.9041095890410954E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B8">
+        <v>85</v>
+      </c>
+      <c r="C8">
+        <v>71</v>
+      </c>
+      <c r="H8">
+        <f>B8</f>
+        <v>85</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="0"/>
+        <v>71</v>
+      </c>
+      <c r="J8" s="11">
+        <f>I8-H8</f>
+        <v>-14</v>
+      </c>
+      <c r="K8" s="6">
+        <f t="shared" si="2"/>
+        <v>-0.16470588235294117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" t="s">
+        <v>138</v>
+      </c>
+      <c r="B9">
+        <v>106</v>
+      </c>
+      <c r="C9">
+        <v>102</v>
+      </c>
+      <c r="H9">
+        <f>B9</f>
+        <v>106</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="0"/>
+        <v>102</v>
+      </c>
+      <c r="J9" s="11">
+        <f>I9-H9</f>
+        <v>-4</v>
+      </c>
+      <c r="K9" s="6">
+        <f t="shared" si="2"/>
+        <v>-3.7735849056603772E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10">
+        <v>121</v>
+      </c>
+      <c r="C10">
+        <v>114</v>
+      </c>
+      <c r="D10">
+        <v>40</v>
+      </c>
+      <c r="E10">
+        <v>60</v>
+      </c>
+      <c r="H10">
+        <f>B10</f>
+        <v>121</v>
+      </c>
+      <c r="I10">
+        <f>E10</f>
+        <v>60</v>
+      </c>
+      <c r="J10" s="11">
+        <f>I10-H10</f>
+        <v>-61</v>
+      </c>
+      <c r="K10" s="6">
+        <f t="shared" si="2"/>
+        <v>-0.50413223140495866</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" t="s">
+        <v>140</v>
+      </c>
+      <c r="B11">
+        <v>104</v>
+      </c>
+      <c r="C11">
+        <v>97</v>
+      </c>
+      <c r="D11">
+        <v>20</v>
+      </c>
+      <c r="E11">
+        <v>38</v>
+      </c>
+      <c r="H11">
+        <f>B11</f>
+        <v>104</v>
+      </c>
+      <c r="I11">
+        <f t="shared" ref="I11:I14" si="3">E11</f>
+        <v>38</v>
+      </c>
+      <c r="J11" s="11">
+        <f t="shared" ref="J11:J14" si="4">I11-H11</f>
+        <v>-66</v>
+      </c>
+      <c r="K11" s="6">
+        <f t="shared" ref="K11:K14" si="5">J11/H11</f>
+        <v>-0.63461538461538458</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" t="s">
+        <v>141</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>125</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <f>B12</f>
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J12" s="11">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K12" s="6" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" t="s">
+        <v>142</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>54</v>
+      </c>
+      <c r="H13">
+        <f>B13</f>
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="3"/>
+        <v>54</v>
+      </c>
+      <c r="J13" s="11">
+        <f t="shared" si="4"/>
+        <v>54</v>
+      </c>
+      <c r="K13" s="6" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" t="s">
+        <v>143</v>
+      </c>
+      <c r="B14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>24</v>
+      </c>
+      <c r="H14">
+        <f>B14</f>
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="3"/>
+        <v>24</v>
+      </c>
+      <c r="J14" s="11">
+        <f t="shared" si="4"/>
+        <v>24</v>
+      </c>
+      <c r="K14" s="6" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" t="s">
+        <v>144</v>
+      </c>
+      <c r="B15">
+        <v>518</v>
+      </c>
+      <c r="C15">
+        <v>507</v>
+      </c>
+      <c r="H15">
+        <f>B15</f>
+        <v>518</v>
+      </c>
+      <c r="I15">
+        <f t="shared" ref="I15:I16" si="6">MIN(C15:F15)</f>
+        <v>507</v>
+      </c>
+      <c r="J15" s="11">
+        <f t="shared" ref="J15:J16" si="7">I15-H15</f>
+        <v>-11</v>
+      </c>
+      <c r="K15" s="6">
+        <f t="shared" ref="K15:K16" si="8">J15/H15</f>
+        <v>-2.1235521235521235E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" t="s">
+        <v>149</v>
+      </c>
+      <c r="B16">
+        <v>871</v>
+      </c>
+      <c r="C16">
+        <v>855</v>
+      </c>
+      <c r="H16">
+        <f>B16</f>
+        <v>871</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="6"/>
+        <v>855</v>
+      </c>
+      <c r="J16" s="11">
+        <f t="shared" si="7"/>
+        <v>-16</v>
+      </c>
+      <c r="K16" s="6">
+        <f t="shared" si="8"/>
+        <v>-1.8369690011481057E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17" t="s">
+        <v>150</v>
+      </c>
+      <c r="B17">
+        <v>358</v>
+      </c>
+      <c r="C17">
+        <v>344</v>
+      </c>
+      <c r="H17">
+        <f>B17</f>
+        <v>358</v>
+      </c>
+      <c r="I17">
+        <f t="shared" ref="I17" si="9">MIN(C17:F17)</f>
+        <v>344</v>
+      </c>
+      <c r="J17" s="11">
+        <f t="shared" ref="J17" si="10">I17-H17</f>
+        <v>-14</v>
+      </c>
+      <c r="K17" s="6">
+        <f t="shared" ref="K17" si="11">J17/H17</f>
+        <v>-3.9106145251396648E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" t="s">
+        <v>151</v>
+      </c>
+      <c r="B18">
+        <v>161</v>
+      </c>
+      <c r="C18">
+        <v>147</v>
+      </c>
+      <c r="H18">
+        <f>B18</f>
+        <v>161</v>
+      </c>
+      <c r="I18">
+        <f t="shared" ref="I18:I19" si="12">MIN(C18:F18)</f>
+        <v>147</v>
+      </c>
+      <c r="J18" s="11">
+        <f t="shared" ref="J18:J19" si="13">I18-H18</f>
+        <v>-14</v>
+      </c>
+      <c r="K18" s="6">
+        <f t="shared" ref="K18:K19" si="14">J18/H18</f>
+        <v>-8.6956521739130432E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19" t="s">
+        <v>152</v>
+      </c>
+      <c r="B19">
+        <v>982</v>
+      </c>
+      <c r="C19">
+        <v>977</v>
+      </c>
+      <c r="D19">
+        <v>967</v>
+      </c>
+      <c r="E19">
+        <v>951</v>
+      </c>
+      <c r="F19">
+        <v>479</v>
+      </c>
+      <c r="H19">
+        <f>B19</f>
+        <v>982</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="12"/>
+        <v>479</v>
+      </c>
+      <c r="J19" s="11">
+        <f t="shared" si="13"/>
+        <v>-503</v>
+      </c>
+      <c r="K19" s="6">
+        <f t="shared" si="14"/>
+        <v>-0.51221995926680242</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" t="s">
+        <v>153</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>235</v>
+      </c>
+      <c r="H20">
+        <f>B20</f>
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <f t="shared" ref="I20" si="15">MIN(C20:F20)</f>
+        <v>235</v>
+      </c>
+      <c r="J20" s="11">
+        <f t="shared" ref="J20" si="16">I20-H20</f>
+        <v>235</v>
+      </c>
+      <c r="K20" s="6" t="e">
+        <f t="shared" ref="K20" si="17">J20/H20</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21" t="s">
+        <v>154</v>
+      </c>
+      <c r="B21">
+        <v>245</v>
+      </c>
+      <c r="C21">
+        <v>233</v>
+      </c>
+      <c r="D21">
+        <v>224</v>
+      </c>
+      <c r="H21">
+        <f>B21</f>
+        <v>245</v>
+      </c>
+      <c r="I21">
+        <f t="shared" ref="I21" si="18">MIN(C21:F21)</f>
+        <v>224</v>
+      </c>
+      <c r="J21" s="11">
+        <f t="shared" ref="J21" si="19">I21-H21</f>
+        <v>-21</v>
+      </c>
+      <c r="K21" s="6">
+        <f t="shared" ref="K21" si="20">J21/H21</f>
+        <v>-8.5714285714285715E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
+      <c r="A22" t="s">
+        <v>155</v>
+      </c>
+      <c r="B22">
+        <v>1918</v>
+      </c>
+      <c r="C22">
+        <v>1882</v>
+      </c>
+      <c r="H22">
+        <f>B22</f>
+        <v>1918</v>
+      </c>
+      <c r="I22">
+        <f t="shared" ref="I22:I23" si="21">MIN(C22:F22)</f>
+        <v>1882</v>
+      </c>
+      <c r="J22" s="11">
+        <f t="shared" ref="J22:J23" si="22">I22-H22</f>
+        <v>-36</v>
+      </c>
+      <c r="K22" s="6">
+        <f t="shared" ref="K22:K23" si="23">J22/H22</f>
+        <v>-1.8769551616266946E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
+      <c r="A23" t="s">
+        <v>156</v>
+      </c>
+      <c r="B23">
+        <v>183</v>
+      </c>
+      <c r="C23">
+        <v>172</v>
+      </c>
+      <c r="H23">
+        <f>B23</f>
+        <v>183</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="21"/>
+        <v>172</v>
+      </c>
+      <c r="J23" s="11">
+        <f t="shared" si="22"/>
+        <v>-11</v>
+      </c>
+      <c r="K23" s="6">
+        <f t="shared" si="23"/>
+        <v>-6.0109289617486336E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
+      <c r="A24" t="s">
+        <v>157</v>
+      </c>
+      <c r="B24">
+        <v>107</v>
+      </c>
+      <c r="C24">
+        <v>94</v>
+      </c>
+      <c r="D24">
+        <v>93</v>
+      </c>
+      <c r="H24">
+        <f>B24</f>
+        <v>107</v>
+      </c>
+      <c r="I24">
+        <f t="shared" ref="I24" si="24">MIN(C24:F24)</f>
+        <v>93</v>
+      </c>
+      <c r="J24" s="11">
+        <f t="shared" ref="J24" si="25">I24-H24</f>
+        <v>-14</v>
+      </c>
+      <c r="K24" s="6">
+        <f t="shared" ref="K24" si="26">J24/H24</f>
+        <v>-0.13084112149532709</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Saved only 13 bytes by changing String.Format calls
</commit_message>
<xml_diff>
--- a/ILSIze.xlsx
+++ b/ILSIze.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE13BD5D-41AD-8B45-8516-BC1AD0D1DFDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9AE3D08-21D7-EB4E-AECB-2F3590F855BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14420" firstSheet="2" activeTab="8" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14420" firstSheet="2" activeTab="9" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
   </bookViews>
   <sheets>
     <sheet name="Chemistry.cs" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="ExtraMath_decimal.cs" sheetId="7" r:id="rId7"/>
     <sheet name="void OutputLinearRegression2" sheetId="8" r:id="rId8"/>
     <sheet name="Console.Write" sheetId="9" r:id="rId9"/>
+    <sheet name="String.Format" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="163">
   <si>
     <t>Méthode</t>
   </si>
@@ -518,6 +519,21 @@
   </si>
   <si>
     <t>VectorTest.Example69Console</t>
+  </si>
+  <si>
+    <t>Matrix.op_Addition</t>
+  </si>
+  <si>
+    <t>Matrix.op_Subtraction</t>
+  </si>
+  <si>
+    <t>Matrix.op_Multiply(Matrix&lt;T&gt;</t>
+  </si>
+  <si>
+    <t>EnzymeKinematic.ToString()</t>
+  </si>
+  <si>
+    <t>CalculusTest.TestMathAnalog(double…</t>
   </si>
 </sst>
 </file>
@@ -616,6 +632,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -625,7 +642,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -922,16 +938,16 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1"/>
-      <c r="B1" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8" t="s">
+      <c r="B1" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
@@ -1201,6 +1217,75 @@
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="E1:G1"/>
   </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B14FDF44-9379-3942-B963-F6E0C991A132}">
+  <dimension ref="A2:C6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="4" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B2">
+        <v>179</v>
+      </c>
+      <c r="C2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B3">
+        <v>179</v>
+      </c>
+      <c r="C3">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B4">
+        <v>244</v>
+      </c>
+      <c r="C4">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>161</v>
+      </c>
+      <c r="B5">
+        <v>109</v>
+      </c>
+      <c r="C5">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>162</v>
+      </c>
+      <c r="B6">
+        <v>129</v>
+      </c>
+      <c r="C6">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1490,51 +1575,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" s="1" customFormat="1">
-      <c r="D1" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8" t="s">
+      <c r="D1" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8" t="s">
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8" t="s">
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-      <c r="P1" s="8" t="s">
+      <c r="N1" s="9"/>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="Q1" s="8"/>
-      <c r="R1" s="8"/>
-      <c r="S1" s="8" t="s">
+      <c r="Q1" s="9"/>
+      <c r="R1" s="9"/>
+      <c r="S1" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="T1" s="8"/>
-      <c r="U1" s="8"/>
-      <c r="V1" s="8" t="s">
+      <c r="T1" s="9"/>
+      <c r="U1" s="9"/>
+      <c r="V1" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="W1" s="8"/>
-      <c r="X1" s="8"/>
-      <c r="Y1" s="8" t="s">
+      <c r="W1" s="9"/>
+      <c r="X1" s="9"/>
+      <c r="Y1" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="Z1" s="8"/>
-      <c r="AA1" s="8"/>
-      <c r="AB1" s="8" t="s">
+      <c r="Z1" s="9"/>
+      <c r="AA1" s="9"/>
+      <c r="AB1" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="AC1" s="8"/>
-      <c r="AD1" s="8"/>
+      <c r="AC1" s="9"/>
+      <c r="AD1" s="9"/>
     </row>
     <row r="2" spans="1:30" s="1" customFormat="1">
       <c r="A2" s="1" t="s">
@@ -1629,10 +1714,10 @@
       </c>
     </row>
     <row r="3" spans="1:30">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="11" t="s">
         <v>41</v>
       </c>
       <c r="C3" t="s">
@@ -1721,8 +1806,8 @@
       </c>
     </row>
     <row r="4" spans="1:30">
-      <c r="A4" s="9"/>
-      <c r="B4" s="10"/>
+      <c r="A4" s="10"/>
+      <c r="B4" s="11"/>
       <c r="C4" t="s">
         <v>113</v>
       </c>
@@ -1737,8 +1822,8 @@
       </c>
     </row>
     <row r="5" spans="1:30">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
+      <c r="A5" s="10"/>
+      <c r="B5" s="11"/>
       <c r="C5" t="s">
         <v>43</v>
       </c>
@@ -1825,8 +1910,8 @@
       </c>
     </row>
     <row r="6" spans="1:30">
-      <c r="A6" s="9"/>
-      <c r="B6" s="10"/>
+      <c r="A6" s="10"/>
+      <c r="B6" s="11"/>
       <c r="C6" t="s">
         <v>114</v>
       </c>
@@ -1841,7 +1926,7 @@
       </c>
     </row>
     <row r="7" spans="1:30">
-      <c r="A7" s="9"/>
+      <c r="A7" s="10"/>
       <c r="B7" s="5" t="s">
         <v>115</v>
       </c>
@@ -1856,8 +1941,8 @@
       </c>
     </row>
     <row r="8" spans="1:30">
-      <c r="A8" s="9"/>
-      <c r="B8" s="10" t="s">
+      <c r="A8" s="10"/>
+      <c r="B8" s="11" t="s">
         <v>116</v>
       </c>
       <c r="C8" t="s">
@@ -1874,8 +1959,8 @@
       </c>
     </row>
     <row r="9" spans="1:30">
-      <c r="A9" s="9"/>
-      <c r="B9" s="10"/>
+      <c r="A9" s="10"/>
+      <c r="B9" s="11"/>
       <c r="C9" t="s">
         <v>118</v>
       </c>
@@ -1890,8 +1975,8 @@
       </c>
     </row>
     <row r="10" spans="1:30">
-      <c r="A10" s="9"/>
-      <c r="B10" s="10" t="s">
+      <c r="A10" s="10"/>
+      <c r="B10" s="11" t="s">
         <v>104</v>
       </c>
       <c r="C10" t="s">
@@ -1908,8 +1993,8 @@
       </c>
     </row>
     <row r="11" spans="1:30">
-      <c r="A11" s="9"/>
-      <c r="B11" s="10"/>
+      <c r="A11" s="10"/>
+      <c r="B11" s="11"/>
       <c r="C11" t="s">
         <v>114</v>
       </c>
@@ -1924,10 +2009,10 @@
       </c>
     </row>
     <row r="12" spans="1:30">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>41</v>
       </c>
       <c r="C12" s="4" t="s">
@@ -1962,8 +2047,8 @@
       </c>
     </row>
     <row r="13" spans="1:30">
-      <c r="A13" s="9"/>
-      <c r="B13" s="10"/>
+      <c r="A13" s="10"/>
+      <c r="B13" s="11"/>
       <c r="C13" t="s">
         <v>42</v>
       </c>
@@ -2050,8 +2135,8 @@
       </c>
     </row>
     <row r="14" spans="1:30">
-      <c r="A14" s="9"/>
-      <c r="B14" s="10"/>
+      <c r="A14" s="10"/>
+      <c r="B14" s="11"/>
       <c r="C14" s="4" t="s">
         <v>105</v>
       </c>
@@ -2084,8 +2169,8 @@
       </c>
     </row>
     <row r="15" spans="1:30">
-      <c r="A15" s="9"/>
-      <c r="B15" s="10"/>
+      <c r="A15" s="10"/>
+      <c r="B15" s="11"/>
       <c r="C15" t="s">
         <v>43</v>
       </c>
@@ -2172,8 +2257,8 @@
       </c>
     </row>
     <row r="16" spans="1:30">
-      <c r="A16" s="9"/>
-      <c r="B16" s="10" t="s">
+      <c r="A16" s="10"/>
+      <c r="B16" s="11" t="s">
         <v>103</v>
       </c>
       <c r="C16" t="s">
@@ -2208,8 +2293,8 @@
       </c>
     </row>
     <row r="17" spans="1:30">
-      <c r="A17" s="9"/>
-      <c r="B17" s="10"/>
+      <c r="A17" s="10"/>
+      <c r="B17" s="11"/>
       <c r="C17" t="s">
         <v>109</v>
       </c>
@@ -2242,8 +2327,8 @@
       </c>
     </row>
     <row r="18" spans="1:30">
-      <c r="A18" s="9"/>
-      <c r="B18" s="10" t="s">
+      <c r="A18" s="10"/>
+      <c r="B18" s="11" t="s">
         <v>104</v>
       </c>
       <c r="C18" t="s">
@@ -2278,8 +2363,8 @@
       </c>
     </row>
     <row r="19" spans="1:30">
-      <c r="A19" s="9"/>
-      <c r="B19" s="10"/>
+      <c r="A19" s="10"/>
+      <c r="B19" s="11"/>
       <c r="C19" t="s">
         <v>109</v>
       </c>
@@ -2435,6 +2520,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B10:B11"/>
     <mergeCell ref="AB1:AD1"/>
     <mergeCell ref="Y1:AA1"/>
     <mergeCell ref="A12:A19"/>
@@ -2451,7 +2537,6 @@
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="B3:B6"/>
     <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B10:B11"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2475,16 +2560,16 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1"/>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8" t="s">
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
@@ -2840,31 +2925,31 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" s="1"/>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8" t="s">
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8" t="s">
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8" t="s">
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8" t="s">
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="O1" s="8"/>
-      <c r="P1" s="8"/>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9"/>
     </row>
     <row r="2" spans="1:16">
       <c r="A2" s="1" t="s">
@@ -3121,21 +3206,21 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="1"/>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8" t="s">
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8" t="s">
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
@@ -4110,54 +4195,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" s="1" customFormat="1">
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8" t="s">
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8" t="s">
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8" t="s">
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
+      <c r="O1" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="8"/>
-      <c r="R1" s="8"/>
-      <c r="S1" s="8" t="s">
+      <c r="P1" s="9"/>
+      <c r="Q1" s="9"/>
+      <c r="R1" s="9"/>
+      <c r="S1" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="T1" s="8"/>
-      <c r="U1" s="8"/>
-      <c r="V1" s="8"/>
-      <c r="W1" s="8" t="s">
+      <c r="T1" s="9"/>
+      <c r="U1" s="9"/>
+      <c r="V1" s="9"/>
+      <c r="W1" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="X1" s="8"/>
-      <c r="Y1" s="8"/>
-      <c r="Z1" s="8"/>
-      <c r="AA1" s="8" t="s">
+      <c r="X1" s="9"/>
+      <c r="Y1" s="9"/>
+      <c r="Z1" s="9"/>
+      <c r="AA1" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="AB1" s="8"/>
-      <c r="AC1" s="8"/>
-      <c r="AD1" s="8"/>
-      <c r="AE1" s="8" t="s">
+      <c r="AB1" s="9"/>
+      <c r="AC1" s="9"/>
+      <c r="AD1" s="9"/>
+      <c r="AE1" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="AF1" s="8"/>
-      <c r="AG1" s="8"/>
-      <c r="AH1" s="8"/>
+      <c r="AF1" s="9"/>
+      <c r="AG1" s="9"/>
+      <c r="AH1" s="9"/>
     </row>
     <row r="2" spans="1:34" s="1" customFormat="1">
       <c r="A2" s="1" t="s">
@@ -4965,13 +5050,13 @@
       <c r="A1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
       <c r="H1" s="1" t="s">
         <v>146</v>
       </c>
@@ -5005,15 +5090,15 @@
         <v>2903</v>
       </c>
       <c r="H2">
-        <f>B2</f>
+        <f t="shared" ref="H2:H24" si="0">B2</f>
         <v>3023</v>
       </c>
       <c r="I2">
         <f>MIN(C2:F2)</f>
         <v>2903</v>
       </c>
-      <c r="J2" s="11">
-        <f>I2-H2</f>
+      <c r="J2" s="8">
+        <f t="shared" ref="J2:J10" si="1">I2-H2</f>
         <v>-120</v>
       </c>
       <c r="K2" s="6">
@@ -5038,19 +5123,19 @@
         <v>1364</v>
       </c>
       <c r="H3">
-        <f>B3</f>
+        <f t="shared" si="0"/>
         <v>1413</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I9" si="0">MIN(C3:F3)</f>
+        <f t="shared" ref="I3:I9" si="2">MIN(C3:F3)</f>
         <v>1364</v>
       </c>
-      <c r="J3" s="11">
-        <f>I3-H3</f>
+      <c r="J3" s="8">
+        <f t="shared" si="1"/>
         <v>-49</v>
       </c>
       <c r="K3" s="6">
-        <f t="shared" ref="K3:K4" si="1">J3/H3</f>
+        <f t="shared" ref="K3:K4" si="3">J3/H3</f>
         <v>-3.4677990092002828E-2</v>
       </c>
     </row>
@@ -5068,19 +5153,19 @@
         <v>10025</v>
       </c>
       <c r="H4">
-        <f>B4</f>
+        <f t="shared" si="0"/>
         <v>10094</v>
       </c>
       <c r="I4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>10025</v>
       </c>
-      <c r="J4" s="11">
-        <f>I4-H4</f>
+      <c r="J4" s="8">
+        <f t="shared" si="1"/>
         <v>-69</v>
       </c>
       <c r="K4" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-6.8357440063403999E-3</v>
       </c>
     </row>
@@ -5095,19 +5180,19 @@
         <v>69</v>
       </c>
       <c r="H5">
-        <f>B5</f>
+        <f t="shared" si="0"/>
         <v>74</v>
       </c>
       <c r="I5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>69</v>
       </c>
-      <c r="J5" s="11">
-        <f>I5-H5</f>
+      <c r="J5" s="8">
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
       <c r="K5" s="6">
-        <f t="shared" ref="K5:K10" si="2">J5/H5</f>
+        <f t="shared" ref="K5:K10" si="4">J5/H5</f>
         <v>-6.7567567567567571E-2</v>
       </c>
     </row>
@@ -5122,19 +5207,19 @@
         <v>125</v>
       </c>
       <c r="H6">
-        <f>B6</f>
+        <f t="shared" si="0"/>
         <v>142</v>
       </c>
       <c r="I6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>125</v>
       </c>
-      <c r="J6" s="11">
-        <f>I6-H6</f>
+      <c r="J6" s="8">
+        <f t="shared" si="1"/>
         <v>-17</v>
       </c>
       <c r="K6" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.11971830985915492</v>
       </c>
     </row>
@@ -5149,19 +5234,19 @@
         <v>133</v>
       </c>
       <c r="H7">
-        <f>B7</f>
+        <f t="shared" si="0"/>
         <v>146</v>
       </c>
       <c r="I7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>133</v>
       </c>
-      <c r="J7" s="11">
-        <f>I7-H7</f>
+      <c r="J7" s="8">
+        <f t="shared" si="1"/>
         <v>-13</v>
       </c>
       <c r="K7" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-8.9041095890410954E-2</v>
       </c>
     </row>
@@ -5176,19 +5261,19 @@
         <v>71</v>
       </c>
       <c r="H8">
-        <f>B8</f>
+        <f t="shared" si="0"/>
         <v>85</v>
       </c>
       <c r="I8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>71</v>
       </c>
-      <c r="J8" s="11">
-        <f>I8-H8</f>
+      <c r="J8" s="8">
+        <f t="shared" si="1"/>
         <v>-14</v>
       </c>
       <c r="K8" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.16470588235294117</v>
       </c>
     </row>
@@ -5203,19 +5288,19 @@
         <v>102</v>
       </c>
       <c r="H9">
-        <f>B9</f>
+        <f t="shared" si="0"/>
         <v>106</v>
       </c>
       <c r="I9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>102</v>
       </c>
-      <c r="J9" s="11">
-        <f>I9-H9</f>
+      <c r="J9" s="8">
+        <f t="shared" si="1"/>
         <v>-4</v>
       </c>
       <c r="K9" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-3.7735849056603772E-2</v>
       </c>
     </row>
@@ -5236,19 +5321,19 @@
         <v>60</v>
       </c>
       <c r="H10">
-        <f>B10</f>
+        <f t="shared" si="0"/>
         <v>121</v>
       </c>
       <c r="I10">
         <f>E10</f>
         <v>60</v>
       </c>
-      <c r="J10" s="11">
-        <f>I10-H10</f>
+      <c r="J10" s="8">
+        <f t="shared" si="1"/>
         <v>-61</v>
       </c>
       <c r="K10" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>-0.50413223140495866</v>
       </c>
     </row>
@@ -5269,19 +5354,19 @@
         <v>38</v>
       </c>
       <c r="H11">
-        <f>B11</f>
+        <f t="shared" si="0"/>
         <v>104</v>
       </c>
       <c r="I11">
-        <f t="shared" ref="I11:I14" si="3">E11</f>
+        <f t="shared" ref="I11:I14" si="5">E11</f>
         <v>38</v>
       </c>
-      <c r="J11" s="11">
-        <f t="shared" ref="J11:J14" si="4">I11-H11</f>
+      <c r="J11" s="8">
+        <f t="shared" ref="J11:J14" si="6">I11-H11</f>
         <v>-66</v>
       </c>
       <c r="K11" s="6">
-        <f t="shared" ref="K11:K14" si="5">J11/H11</f>
+        <f t="shared" ref="K11:K14" si="7">J11/H11</f>
         <v>-0.63461538461538458</v>
       </c>
     </row>
@@ -5299,19 +5384,19 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <f>B12</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J12" s="11">
-        <f t="shared" si="4"/>
+      <c r="J12" s="8">
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="K12" s="6" t="e">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -5326,19 +5411,19 @@
         <v>54</v>
       </c>
       <c r="H13">
-        <f>B13</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>54</v>
       </c>
-      <c r="J13" s="11">
-        <f t="shared" si="4"/>
+      <c r="J13" s="8">
+        <f t="shared" si="6"/>
         <v>54</v>
       </c>
       <c r="K13" s="6" t="e">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -5353,19 +5438,19 @@
         <v>24</v>
       </c>
       <c r="H14">
-        <f>B14</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>24</v>
       </c>
-      <c r="J14" s="11">
-        <f t="shared" si="4"/>
+      <c r="J14" s="8">
+        <f t="shared" si="6"/>
         <v>24</v>
       </c>
       <c r="K14" s="6" t="e">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -5380,19 +5465,19 @@
         <v>507</v>
       </c>
       <c r="H15">
-        <f>B15</f>
+        <f t="shared" si="0"/>
         <v>518</v>
       </c>
       <c r="I15">
-        <f t="shared" ref="I15:I16" si="6">MIN(C15:F15)</f>
+        <f t="shared" ref="I15:I16" si="8">MIN(C15:F15)</f>
         <v>507</v>
       </c>
-      <c r="J15" s="11">
-        <f t="shared" ref="J15:J16" si="7">I15-H15</f>
+      <c r="J15" s="8">
+        <f t="shared" ref="J15:J16" si="9">I15-H15</f>
         <v>-11</v>
       </c>
       <c r="K15" s="6">
-        <f t="shared" ref="K15:K16" si="8">J15/H15</f>
+        <f t="shared" ref="K15:K16" si="10">J15/H15</f>
         <v>-2.1235521235521235E-2</v>
       </c>
     </row>
@@ -5407,19 +5492,19 @@
         <v>855</v>
       </c>
       <c r="H16">
-        <f>B16</f>
+        <f t="shared" si="0"/>
         <v>871</v>
       </c>
       <c r="I16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>855</v>
       </c>
-      <c r="J16" s="11">
-        <f t="shared" si="7"/>
+      <c r="J16" s="8">
+        <f t="shared" si="9"/>
         <v>-16</v>
       </c>
       <c r="K16" s="6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-1.8369690011481057E-2</v>
       </c>
     </row>
@@ -5434,19 +5519,19 @@
         <v>344</v>
       </c>
       <c r="H17">
-        <f>B17</f>
+        <f t="shared" si="0"/>
         <v>358</v>
       </c>
       <c r="I17">
-        <f t="shared" ref="I17" si="9">MIN(C17:F17)</f>
+        <f t="shared" ref="I17" si="11">MIN(C17:F17)</f>
         <v>344</v>
       </c>
-      <c r="J17" s="11">
-        <f t="shared" ref="J17" si="10">I17-H17</f>
+      <c r="J17" s="8">
+        <f t="shared" ref="J17" si="12">I17-H17</f>
         <v>-14</v>
       </c>
       <c r="K17" s="6">
-        <f t="shared" ref="K17" si="11">J17/H17</f>
+        <f t="shared" ref="K17" si="13">J17/H17</f>
         <v>-3.9106145251396648E-2</v>
       </c>
     </row>
@@ -5461,19 +5546,19 @@
         <v>147</v>
       </c>
       <c r="H18">
-        <f>B18</f>
+        <f t="shared" si="0"/>
         <v>161</v>
       </c>
       <c r="I18">
-        <f t="shared" ref="I18:I19" si="12">MIN(C18:F18)</f>
+        <f t="shared" ref="I18:I19" si="14">MIN(C18:F18)</f>
         <v>147</v>
       </c>
-      <c r="J18" s="11">
-        <f t="shared" ref="J18:J19" si="13">I18-H18</f>
+      <c r="J18" s="8">
+        <f t="shared" ref="J18:J19" si="15">I18-H18</f>
         <v>-14</v>
       </c>
       <c r="K18" s="6">
-        <f t="shared" ref="K18:K19" si="14">J18/H18</f>
+        <f t="shared" ref="K18:K19" si="16">J18/H18</f>
         <v>-8.6956521739130432E-2</v>
       </c>
     </row>
@@ -5497,19 +5582,19 @@
         <v>479</v>
       </c>
       <c r="H19">
-        <f>B19</f>
+        <f t="shared" si="0"/>
         <v>982</v>
       </c>
       <c r="I19">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>479</v>
       </c>
-      <c r="J19" s="11">
-        <f t="shared" si="13"/>
+      <c r="J19" s="8">
+        <f t="shared" si="15"/>
         <v>-503</v>
       </c>
       <c r="K19" s="6">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>-0.51221995926680242</v>
       </c>
     </row>
@@ -5524,19 +5609,19 @@
         <v>235</v>
       </c>
       <c r="H20">
-        <f>B20</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I20">
-        <f t="shared" ref="I20" si="15">MIN(C20:F20)</f>
+        <f t="shared" ref="I20" si="17">MIN(C20:F20)</f>
         <v>235</v>
       </c>
-      <c r="J20" s="11">
-        <f t="shared" ref="J20" si="16">I20-H20</f>
+      <c r="J20" s="8">
+        <f t="shared" ref="J20" si="18">I20-H20</f>
         <v>235</v>
       </c>
       <c r="K20" s="6" t="e">
-        <f t="shared" ref="K20" si="17">J20/H20</f>
+        <f t="shared" ref="K20" si="19">J20/H20</f>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -5554,19 +5639,19 @@
         <v>224</v>
       </c>
       <c r="H21">
-        <f>B21</f>
+        <f t="shared" si="0"/>
         <v>245</v>
       </c>
       <c r="I21">
-        <f t="shared" ref="I21" si="18">MIN(C21:F21)</f>
+        <f t="shared" ref="I21" si="20">MIN(C21:F21)</f>
         <v>224</v>
       </c>
-      <c r="J21" s="11">
-        <f t="shared" ref="J21" si="19">I21-H21</f>
+      <c r="J21" s="8">
+        <f t="shared" ref="J21" si="21">I21-H21</f>
         <v>-21</v>
       </c>
       <c r="K21" s="6">
-        <f t="shared" ref="K21" si="20">J21/H21</f>
+        <f t="shared" ref="K21" si="22">J21/H21</f>
         <v>-8.5714285714285715E-2</v>
       </c>
     </row>
@@ -5581,19 +5666,19 @@
         <v>1882</v>
       </c>
       <c r="H22">
-        <f>B22</f>
+        <f t="shared" si="0"/>
         <v>1918</v>
       </c>
       <c r="I22">
-        <f t="shared" ref="I22:I23" si="21">MIN(C22:F22)</f>
+        <f t="shared" ref="I22:I23" si="23">MIN(C22:F22)</f>
         <v>1882</v>
       </c>
-      <c r="J22" s="11">
-        <f t="shared" ref="J22:J23" si="22">I22-H22</f>
+      <c r="J22" s="8">
+        <f t="shared" ref="J22:J23" si="24">I22-H22</f>
         <v>-36</v>
       </c>
       <c r="K22" s="6">
-        <f t="shared" ref="K22:K23" si="23">J22/H22</f>
+        <f t="shared" ref="K22:K23" si="25">J22/H22</f>
         <v>-1.8769551616266946E-2</v>
       </c>
     </row>
@@ -5608,19 +5693,19 @@
         <v>172</v>
       </c>
       <c r="H23">
-        <f>B23</f>
+        <f t="shared" si="0"/>
         <v>183</v>
       </c>
       <c r="I23">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>172</v>
       </c>
-      <c r="J23" s="11">
-        <f t="shared" si="22"/>
+      <c r="J23" s="8">
+        <f t="shared" si="24"/>
         <v>-11</v>
       </c>
       <c r="K23" s="6">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>-6.0109289617486336E-2</v>
       </c>
     </row>
@@ -5638,19 +5723,19 @@
         <v>93</v>
       </c>
       <c r="H24">
-        <f>B24</f>
+        <f t="shared" si="0"/>
         <v>107</v>
       </c>
       <c r="I24">
-        <f t="shared" ref="I24" si="24">MIN(C24:F24)</f>
+        <f t="shared" ref="I24" si="26">MIN(C24:F24)</f>
         <v>93</v>
       </c>
-      <c r="J24" s="11">
-        <f t="shared" ref="J24" si="25">I24-H24</f>
+      <c r="J24" s="8">
+        <f t="shared" ref="J24" si="27">I24-H24</f>
         <v>-14</v>
       </c>
       <c r="K24" s="6">
-        <f t="shared" ref="K24" si="26">J24/H24</f>
+        <f t="shared" ref="K24" si="28">J24/H24</f>
         <v>-0.13084112149532709</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Saved 102 IL bytes with an exception factory method
</commit_message>
<xml_diff>
--- a/ILSIze.xlsx
+++ b/ILSIze.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9AE3D08-21D7-EB4E-AECB-2F3590F855BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA05290E-D578-FC48-8C2E-E0453D78EB7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14420" firstSheet="2" activeTab="9" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="164">
   <si>
     <t>Méthode</t>
   </si>
@@ -534,6 +534,9 @@
   </si>
   <si>
     <t>CalculusTest.TestMathAnalog(double…</t>
+  </si>
+  <si>
+    <t>MatrixDimensionsMismatch</t>
   </si>
 </sst>
 </file>
@@ -637,10 +640,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1223,14 +1226,14 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B14FDF44-9379-3942-B963-F6E0C991A132}">
-  <dimension ref="A2:C6"/>
+  <dimension ref="A2:D7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>158</v>
       </c>
@@ -1240,8 +1243,11 @@
       <c r="C2">
         <v>175</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="D2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>159</v>
       </c>
@@ -1251,8 +1257,11 @@
       <c r="C3">
         <v>175</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
+      <c r="D3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>160</v>
       </c>
@@ -1262,26 +1271,43 @@
       <c r="C4">
         <v>243</v>
       </c>
-    </row>
-    <row r="5" spans="1:3">
+      <c r="D4">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
+        <v>163</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
         <v>161</v>
       </c>
-      <c r="B5">
+      <c r="B6">
         <v>109</v>
       </c>
-      <c r="C5">
+      <c r="C6">
         <v>107</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
         <v>162</v>
       </c>
-      <c r="B6">
+      <c r="B7">
         <v>129</v>
       </c>
-      <c r="C6">
+      <c r="C7">
         <v>127</v>
       </c>
     </row>
@@ -1714,10 +1740,10 @@
       </c>
     </row>
     <row r="3" spans="1:30">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="10" t="s">
         <v>41</v>
       </c>
       <c r="C3" t="s">
@@ -1806,8 +1832,8 @@
       </c>
     </row>
     <row r="4" spans="1:30">
-      <c r="A4" s="10"/>
-      <c r="B4" s="11"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="10"/>
       <c r="C4" t="s">
         <v>113</v>
       </c>
@@ -1822,8 +1848,8 @@
       </c>
     </row>
     <row r="5" spans="1:30">
-      <c r="A5" s="10"/>
-      <c r="B5" s="11"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="10"/>
       <c r="C5" t="s">
         <v>43</v>
       </c>
@@ -1910,8 +1936,8 @@
       </c>
     </row>
     <row r="6" spans="1:30">
-      <c r="A6" s="10"/>
-      <c r="B6" s="11"/>
+      <c r="A6" s="11"/>
+      <c r="B6" s="10"/>
       <c r="C6" t="s">
         <v>114</v>
       </c>
@@ -1926,7 +1952,7 @@
       </c>
     </row>
     <row r="7" spans="1:30">
-      <c r="A7" s="10"/>
+      <c r="A7" s="11"/>
       <c r="B7" s="5" t="s">
         <v>115</v>
       </c>
@@ -1941,8 +1967,8 @@
       </c>
     </row>
     <row r="8" spans="1:30">
-      <c r="A8" s="10"/>
-      <c r="B8" s="11" t="s">
+      <c r="A8" s="11"/>
+      <c r="B8" s="10" t="s">
         <v>116</v>
       </c>
       <c r="C8" t="s">
@@ -1959,8 +1985,8 @@
       </c>
     </row>
     <row r="9" spans="1:30">
-      <c r="A9" s="10"/>
-      <c r="B9" s="11"/>
+      <c r="A9" s="11"/>
+      <c r="B9" s="10"/>
       <c r="C9" t="s">
         <v>118</v>
       </c>
@@ -1975,8 +2001,8 @@
       </c>
     </row>
     <row r="10" spans="1:30">
-      <c r="A10" s="10"/>
-      <c r="B10" s="11" t="s">
+      <c r="A10" s="11"/>
+      <c r="B10" s="10" t="s">
         <v>104</v>
       </c>
       <c r="C10" t="s">
@@ -1993,8 +2019,8 @@
       </c>
     </row>
     <row r="11" spans="1:30">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11"/>
+      <c r="A11" s="11"/>
+      <c r="B11" s="10"/>
       <c r="C11" t="s">
         <v>114</v>
       </c>
@@ -2009,10 +2035,10 @@
       </c>
     </row>
     <row r="12" spans="1:30">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="10" t="s">
         <v>41</v>
       </c>
       <c r="C12" s="4" t="s">
@@ -2047,8 +2073,8 @@
       </c>
     </row>
     <row r="13" spans="1:30">
-      <c r="A13" s="10"/>
-      <c r="B13" s="11"/>
+      <c r="A13" s="11"/>
+      <c r="B13" s="10"/>
       <c r="C13" t="s">
         <v>42</v>
       </c>
@@ -2135,8 +2161,8 @@
       </c>
     </row>
     <row r="14" spans="1:30">
-      <c r="A14" s="10"/>
-      <c r="B14" s="11"/>
+      <c r="A14" s="11"/>
+      <c r="B14" s="10"/>
       <c r="C14" s="4" t="s">
         <v>105</v>
       </c>
@@ -2169,8 +2195,8 @@
       </c>
     </row>
     <row r="15" spans="1:30">
-      <c r="A15" s="10"/>
-      <c r="B15" s="11"/>
+      <c r="A15" s="11"/>
+      <c r="B15" s="10"/>
       <c r="C15" t="s">
         <v>43</v>
       </c>
@@ -2257,8 +2283,8 @@
       </c>
     </row>
     <row r="16" spans="1:30">
-      <c r="A16" s="10"/>
-      <c r="B16" s="11" t="s">
+      <c r="A16" s="11"/>
+      <c r="B16" s="10" t="s">
         <v>103</v>
       </c>
       <c r="C16" t="s">
@@ -2293,8 +2319,8 @@
       </c>
     </row>
     <row r="17" spans="1:30">
-      <c r="A17" s="10"/>
-      <c r="B17" s="11"/>
+      <c r="A17" s="11"/>
+      <c r="B17" s="10"/>
       <c r="C17" t="s">
         <v>109</v>
       </c>
@@ -2327,8 +2353,8 @@
       </c>
     </row>
     <row r="18" spans="1:30">
-      <c r="A18" s="10"/>
-      <c r="B18" s="11" t="s">
+      <c r="A18" s="11"/>
+      <c r="B18" s="10" t="s">
         <v>104</v>
       </c>
       <c r="C18" t="s">
@@ -2363,8 +2389,8 @@
       </c>
     </row>
     <row r="19" spans="1:30">
-      <c r="A19" s="10"/>
-      <c r="B19" s="11"/>
+      <c r="A19" s="11"/>
+      <c r="B19" s="10"/>
       <c r="C19" t="s">
         <v>109</v>
       </c>
@@ -2520,6 +2546,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B8:B9"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="AB1:AD1"/>
     <mergeCell ref="Y1:AA1"/>
@@ -2536,7 +2563,6 @@
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="B3:B6"/>
-    <mergeCell ref="B8:B9"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Corrected most U2U1015 warnings
U2U1015: Do not index an array multiple times within a loop body. Saves 71 IL bytes too.
</commit_message>
<xml_diff>
--- a/ILSIze.xlsx
+++ b/ILSIze.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\Administrator\source\repos\repzilon\Repzilon.Libraries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA05290E-D578-FC48-8C2E-E0453D78EB7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DDE0AD6-760D-4EC0-A766-70F7B2B161B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14420" firstSheet="2" activeTab="9" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="17400" tabRatio="540" firstSheet="4" activeTab="10" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
   </bookViews>
   <sheets>
     <sheet name="Chemistry.cs" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="void OutputLinearRegression2" sheetId="8" r:id="rId8"/>
     <sheet name="Console.Write" sheetId="9" r:id="rId9"/>
     <sheet name="String.Format" sheetId="10" r:id="rId10"/>
+    <sheet name="U2U1015" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="187">
   <si>
     <t>Méthode</t>
   </si>
@@ -537,6 +538,125 @@
   </si>
   <si>
     <t>MatrixDimensionsMismatch</t>
+  </si>
+  <si>
+    <r>
+      <t>n</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <vertAlign val="superscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Franklin Gothic Book"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Franklin Gothic Book"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 0</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>n</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <vertAlign val="superscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Franklin Gothic Book"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Franklin Gothic Book"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 1</t>
+    </r>
+  </si>
+  <si>
+    <t>Repzilon.Tests.ForCoreLibrary</t>
+  </si>
+  <si>
+    <t>ChemistryTest</t>
+  </si>
+  <si>
+    <t>Run</t>
+  </si>
+  <si>
+    <t>EnzymeSpeedDecimal</t>
+  </si>
+  <si>
+    <t>LinearRegressionTest</t>
+  </si>
+  <si>
+    <t>CalibrateGelElectrophoresis</t>
+  </si>
+  <si>
+    <t>Repzilon.Libraries.Core</t>
+  </si>
+  <si>
+    <t>Enzyme</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>DirectLinearPlot</t>
+  </si>
+  <si>
+    <t>RunCommand</t>
+  </si>
+  <si>
+    <t>Matrix</t>
+  </si>
+  <si>
+    <t>Speed(string, string, PointD[])</t>
+  </si>
+  <si>
+    <t>DigitTest</t>
+  </si>
+  <si>
+    <t>TestDigitCount</t>
+  </si>
+  <si>
+    <t>InterpolateMolecularWeight</t>
+  </si>
+  <si>
+    <t>NormalLawTest</t>
+  </si>
+  <si>
+    <t>FindBestIterationCountForNormalLawIntegral(float[], double[], double)</t>
+  </si>
+  <si>
+    <t>FindBestIterationCountForNormalLawIntegral(float[], decimal[], decimal)</t>
+  </si>
+  <si>
+    <t>PeptideGuess</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
   </si>
 </sst>
 </file>
@@ -546,7 +666,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -594,6 +714,21 @@
       <color theme="1"/>
       <name val="Avenir Next Condensed Regular"/>
     </font>
+    <font>
+      <b/>
+      <vertAlign val="superscript"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Franklin Gothic Book"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Franklin Gothic Medium Cond"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -622,7 +757,7 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -644,6 +779,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -928,15 +1071,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E085EFD-832C-3644-BF11-30C65FA80A90}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="1" width="28.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.28515625" customWidth="1"/>
-    <col min="3" max="3" width="5.7109375" customWidth="1"/>
-    <col min="4" max="4" width="6.140625" customWidth="1"/>
+    <col min="1" max="1" width="28.6640625" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" customWidth="1"/>
+    <col min="4" max="4" width="6.109375" customWidth="1"/>
     <col min="5" max="5" width="5" customWidth="1"/>
-    <col min="6" max="6" width="5.7109375" customWidth="1"/>
-    <col min="7" max="7" width="6.140625" customWidth="1"/>
+    <col min="6" max="6" width="5.6640625" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1227,9 +1370,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B14FDF44-9379-3942-B963-F6E0C991A132}">
   <dimension ref="A2:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1312,6 +1455,295 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEFD4D16-60D3-41BE-AECD-07D9E215899B}">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5"/>
+  <cols>
+    <col min="1" max="1" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="6" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="19.5">
+      <c r="D1" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="1" customFormat="1">
+      <c r="A2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" s="1" customFormat="1">
+      <c r="A3" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="C3" t="s">
+        <v>178</v>
+      </c>
+      <c r="D3" s="14">
+        <v>354</v>
+      </c>
+      <c r="E3" s="14">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" s="1" customFormat="1">
+      <c r="A4" s="10"/>
+      <c r="B4" s="10"/>
+      <c r="C4" t="s">
+        <v>175</v>
+      </c>
+      <c r="D4" s="14">
+        <v>370</v>
+      </c>
+      <c r="E4" s="14">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="1" customFormat="1">
+      <c r="A5" s="10"/>
+      <c r="B5" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="C5" t="s">
+        <v>176</v>
+      </c>
+      <c r="D5" s="14">
+        <v>232</v>
+      </c>
+      <c r="E5" s="14">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="1" customFormat="1">
+      <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
+      <c r="C6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6" s="14">
+        <v>244</v>
+      </c>
+      <c r="E6" s="14">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="C7" t="s">
+        <v>168</v>
+      </c>
+      <c r="D7">
+        <v>2911</v>
+      </c>
+      <c r="E7">
+        <v>2914</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="13"/>
+      <c r="B8" s="10"/>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8">
+        <v>470</v>
+      </c>
+      <c r="E8">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="13"/>
+      <c r="B9" s="10"/>
+      <c r="C9" t="s">
+        <v>169</v>
+      </c>
+      <c r="D9">
+        <v>807</v>
+      </c>
+      <c r="E9">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="13"/>
+      <c r="B10" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="C10" t="s">
+        <v>181</v>
+      </c>
+      <c r="D10">
+        <v>125</v>
+      </c>
+      <c r="E10">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="13"/>
+      <c r="B11" s="10"/>
+      <c r="C11" t="s">
+        <v>171</v>
+      </c>
+      <c r="D11">
+        <v>295</v>
+      </c>
+      <c r="E11">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="13"/>
+      <c r="B12" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="C12" t="s">
+        <v>168</v>
+      </c>
+      <c r="D12">
+        <v>1364</v>
+      </c>
+      <c r="E12">
+        <v>1367</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="13"/>
+      <c r="B13" s="10"/>
+      <c r="C13" t="s">
+        <v>180</v>
+      </c>
+      <c r="D13">
+        <v>178</v>
+      </c>
+      <c r="E13">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="13"/>
+      <c r="B14" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="C14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D14">
+        <v>2332</v>
+      </c>
+      <c r="E14">
+        <v>2324</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="13"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="D15">
+        <v>507</v>
+      </c>
+      <c r="E15">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="13"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="D16">
+        <v>855</v>
+      </c>
+      <c r="E16">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="13"/>
+      <c r="B17" t="s">
+        <v>185</v>
+      </c>
+      <c r="C17" t="s">
+        <v>168</v>
+      </c>
+      <c r="D17">
+        <v>678</v>
+      </c>
+      <c r="E17">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="C18" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="D18">
+        <f>SUM(D3:D17)</f>
+        <v>11722</v>
+      </c>
+      <c r="E18">
+        <f>SUM(E3:E17)</f>
+        <v>11651</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="E19">
+        <f>E18-D18</f>
+        <v>-71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="E20" s="6">
+        <f>E19/D18</f>
+        <v>-6.0569868623101862E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="A7:A17"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="B12:B13"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1319,11 +1751,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB670503-4F5B-E64E-832A-2C886DE2735D}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" customWidth="1"/>
-    <col min="3" max="3" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1404,13 +1836,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE08D056-9034-D44D-B934-446C62FAF677}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="1" width="29.5703125" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" customWidth="1"/>
-    <col min="3" max="4" width="4.28515625" customWidth="1"/>
+    <col min="1" max="1" width="29.5546875" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" customWidth="1"/>
+    <col min="3" max="4" width="4.33203125" customWidth="1"/>
     <col min="5" max="5" width="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.28515625" customWidth="1"/>
+    <col min="6" max="6" width="4.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1574,30 +2006,30 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14CFDCA3-71A5-DD4D-9D0E-D63068092BC8}">
   <dimension ref="A1:AD22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="3.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="3.33203125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="3.33203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="5" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="3.33203125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="5" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="3.33203125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="5" bestFit="1" customWidth="1"/>
-    <col min="23" max="24" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="3.33203125" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="5" bestFit="1" customWidth="1"/>
-    <col min="26" max="27" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="26" max="27" width="3.33203125" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="5" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="4" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="3.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" s="1" customFormat="1">
@@ -2546,6 +2978,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B3:B6"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="AB1:AD1"/>
@@ -2562,7 +2995,6 @@
     <mergeCell ref="P1:R1"/>
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="B18:B19"/>
-    <mergeCell ref="B3:B6"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2573,15 +3005,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02857098-9EF4-7A43-8BB2-8228CE41206A}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="1" width="22.28515625" customWidth="1"/>
-    <col min="2" max="2" width="5.28515625" customWidth="1"/>
-    <col min="3" max="3" width="5.7109375" customWidth="1"/>
-    <col min="4" max="4" width="6.140625" customWidth="1"/>
-    <col min="5" max="5" width="5.5703125" customWidth="1"/>
-    <col min="6" max="6" width="5.7109375" customWidth="1"/>
-    <col min="7" max="7" width="6.140625" customWidth="1"/>
+    <col min="1" max="1" width="22.33203125" customWidth="1"/>
+    <col min="2" max="2" width="5.33203125" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" customWidth="1"/>
+    <col min="4" max="4" width="6.109375" customWidth="1"/>
+    <col min="5" max="5" width="5.5546875" customWidth="1"/>
+    <col min="6" max="6" width="5.6640625" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2934,19 +3366,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3446A6D4-E7A1-DE4F-AF79-3C1286851385}">
   <dimension ref="A1:P7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" customWidth="1"/>
-    <col min="2" max="3" width="5.7109375" customWidth="1"/>
-    <col min="4" max="4" width="6.5703125" customWidth="1"/>
-    <col min="5" max="6" width="5.7109375" customWidth="1"/>
-    <col min="7" max="7" width="6.5703125" customWidth="1"/>
-    <col min="8" max="9" width="5.7109375" customWidth="1"/>
-    <col min="10" max="10" width="6.5703125" customWidth="1"/>
-    <col min="11" max="12" width="5.7109375" customWidth="1"/>
-    <col min="13" max="13" width="6.5703125" customWidth="1"/>
-    <col min="14" max="15" width="5.7109375" customWidth="1"/>
-    <col min="16" max="16" width="6.5703125" customWidth="1"/>
+    <col min="1" max="1" width="15.6640625" customWidth="1"/>
+    <col min="2" max="3" width="5.6640625" customWidth="1"/>
+    <col min="4" max="4" width="6.5546875" customWidth="1"/>
+    <col min="5" max="6" width="5.6640625" customWidth="1"/>
+    <col min="7" max="7" width="6.5546875" customWidth="1"/>
+    <col min="8" max="9" width="5.6640625" customWidth="1"/>
+    <col min="10" max="10" width="6.5546875" customWidth="1"/>
+    <col min="11" max="12" width="5.6640625" customWidth="1"/>
+    <col min="13" max="13" width="6.5546875" customWidth="1"/>
+    <col min="14" max="15" width="5.6640625" customWidth="1"/>
+    <col min="16" max="16" width="6.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -3216,18 +3648,18 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2043A2D3-B79F-994A-8E5F-6CAF0A113206}">
   <dimension ref="A1:J35"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="5.7109375" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="6.7109375" customWidth="1"/>
-    <col min="5" max="5" width="5.7109375" customWidth="1"/>
+    <col min="4" max="4" width="6.6640625" customWidth="1"/>
+    <col min="5" max="5" width="5.6640625" customWidth="1"/>
     <col min="6" max="6" width="6" customWidth="1"/>
-    <col min="7" max="7" width="6.7109375" customWidth="1"/>
-    <col min="8" max="8" width="5.7109375" customWidth="1"/>
+    <col min="7" max="7" width="6.6640625" customWidth="1"/>
+    <col min="8" max="8" width="5.6640625" customWidth="1"/>
     <col min="9" max="9" width="6" customWidth="1"/>
-    <col min="10" max="10" width="6.7109375" customWidth="1"/>
+    <col min="10" max="10" width="6.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -4184,40 +4616,40 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D0323DF-4A97-4C48-B3D4-92F5ADBE433C}">
   <dimension ref="A1:AH10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="4.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="4.109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="4.109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="4.109375" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="5" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="4.7109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="4.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="4.109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="4.109375" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="5.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34" s="1" customFormat="1">
@@ -4374,7 +4806,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:34" ht="36">
+    <row r="3" spans="1:34" ht="46.5">
       <c r="A3" t="s">
         <v>120</v>
       </c>
@@ -4478,7 +4910,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:34" ht="36">
+    <row r="4" spans="1:34" ht="46.5">
       <c r="B4" s="7" t="s">
         <v>126</v>
       </c>
@@ -5061,15 +5493,15 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2CB8517-AE04-3E4E-B5BB-4C5D322F3AE8}">
   <dimension ref="A1:K24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="54" customWidth="1"/>
     <col min="2" max="4" width="6" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5" customWidth="1"/>
     <col min="8" max="9" width="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="1" customFormat="1">

</xml_diff>

<commit_message>
Saved 230 IL bytes by reorganizing variables
</commit_message>
<xml_diff>
--- a/ILSIze.xlsx
+++ b/ILSIze.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\Administrator\source\repos\repzilon\Repzilon.Libraries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DDE0AD6-760D-4EC0-A766-70F7B2B161B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9709800-6EEA-4464-8BC2-CE240D4629A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="17400" tabRatio="540" firstSheet="4" activeTab="10" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
+    <workbookView xWindow="600" yWindow="3555" windowWidth="17235" windowHeight="12735" tabRatio="522" firstSheet="8" activeTab="10" xr2:uid="{E50D0282-9BF7-F541-B69F-D7AC36D41BED}"/>
   </bookViews>
   <sheets>
     <sheet name="Chemistry.cs" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="188">
   <si>
     <t>Méthode</t>
   </si>
@@ -658,6 +658,44 @@
   <si>
     <t>TOTAL</t>
   </si>
+  <si>
+    <r>
+      <t>n</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <vertAlign val="superscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Franklin Gothic Book"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Franklin Gothic Book"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Franklin Gothic Book"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t/>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -666,9 +704,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Franklin Gothic Book"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Franklin Gothic Book"/>
       <family val="2"/>
@@ -754,39 +799,38 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1084,16 +1128,16 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1"/>
-      <c r="B1" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9" t="s">
+      <c r="B1" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
@@ -1461,289 +1505,343 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEFD4D16-60D3-41BE-AECD-07D9E215899B}">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="19.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="48.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" ht="19.5">
+    <row r="1" spans="1:6" s="1" customFormat="1" ht="19.5">
+      <c r="A1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>76</v>
+      </c>
       <c r="D1" s="1" t="s">
         <v>164</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" s="1" customFormat="1">
-      <c r="A2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="1" customFormat="1">
-      <c r="A3" s="10" t="s">
+      <c r="F1" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="1" customFormat="1">
+      <c r="A2" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B2" s="13" t="s">
         <v>173</v>
       </c>
+      <c r="C2" t="s">
+        <v>178</v>
+      </c>
+      <c r="D2">
+        <v>354</v>
+      </c>
+      <c r="E2">
+        <v>352</v>
+      </c>
+      <c r="F2">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="1" customFormat="1">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
       <c r="C3" t="s">
+        <v>175</v>
+      </c>
+      <c r="D3">
+        <v>370</v>
+      </c>
+      <c r="E3">
+        <v>372</v>
+      </c>
+      <c r="F3">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="1" customFormat="1">
+      <c r="A4" s="13"/>
+      <c r="B4" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="C4" t="s">
+        <v>176</v>
+      </c>
+      <c r="D4">
+        <v>232</v>
+      </c>
+      <c r="E4">
+        <v>231</v>
+      </c>
+      <c r="F4">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="1" customFormat="1">
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" t="s">
+        <v>71</v>
+      </c>
+      <c r="D5">
+        <v>244</v>
+      </c>
+      <c r="E5">
+        <v>247</v>
+      </c>
+      <c r="F5">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="C6" t="s">
+        <v>168</v>
+      </c>
+      <c r="D6">
+        <v>2911</v>
+      </c>
+      <c r="E6">
+        <v>2914</v>
+      </c>
+      <c r="F6">
+        <v>2878</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="14"/>
+      <c r="B7" s="13"/>
+      <c r="C7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7">
+        <v>470</v>
+      </c>
+      <c r="E7">
+        <v>466</v>
+      </c>
+      <c r="F7">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="14"/>
+      <c r="B8" s="13"/>
+      <c r="C8" t="s">
+        <v>169</v>
+      </c>
+      <c r="D8">
+        <v>807</v>
+      </c>
+      <c r="E8">
+        <v>787</v>
+      </c>
+      <c r="F8">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="14"/>
+      <c r="B9" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="C9" t="s">
+        <v>181</v>
+      </c>
+      <c r="D9">
+        <v>125</v>
+      </c>
+      <c r="E9">
+        <v>124</v>
+      </c>
+      <c r="F9">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="14"/>
+      <c r="B10" s="13"/>
+      <c r="C10" t="s">
+        <v>171</v>
+      </c>
+      <c r="D10">
+        <v>295</v>
+      </c>
+      <c r="E10">
+        <v>283</v>
+      </c>
+      <c r="F10">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="14"/>
+      <c r="B11" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="C11" t="s">
+        <v>168</v>
+      </c>
+      <c r="D11">
+        <v>1364</v>
+      </c>
+      <c r="E11">
+        <v>1367</v>
+      </c>
+      <c r="F11">
+        <v>1355</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="14"/>
+      <c r="B12" s="13"/>
+      <c r="C12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D12">
         <v>178</v>
       </c>
-      <c r="D3" s="14">
-        <v>354</v>
-      </c>
-      <c r="E3" s="14">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="1" customFormat="1">
-      <c r="A4" s="10"/>
-      <c r="B4" s="10"/>
-      <c r="C4" t="s">
-        <v>175</v>
-      </c>
-      <c r="D4" s="14">
-        <v>370</v>
-      </c>
-      <c r="E4" s="14">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="1" customFormat="1">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10" t="s">
-        <v>177</v>
-      </c>
-      <c r="C5" t="s">
-        <v>176</v>
-      </c>
-      <c r="D5" s="14">
-        <v>232</v>
-      </c>
-      <c r="E5" s="14">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="1" customFormat="1">
-      <c r="A6" s="10"/>
-      <c r="B6" s="10"/>
-      <c r="C6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D6" s="14">
-        <v>244</v>
-      </c>
-      <c r="E6" s="14">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="E12">
+        <v>180</v>
+      </c>
+      <c r="F12">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="14"/>
+      <c r="B13" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="C13" t="s">
         <v>168</v>
       </c>
-      <c r="D7">
-        <v>2911</v>
-      </c>
-      <c r="E7">
-        <v>2914</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="13"/>
-      <c r="B8" s="10"/>
-      <c r="C8" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8">
-        <v>470</v>
-      </c>
-      <c r="E8">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="13"/>
-      <c r="B9" s="10"/>
-      <c r="C9" t="s">
-        <v>169</v>
-      </c>
-      <c r="D9">
-        <v>807</v>
-      </c>
-      <c r="E9">
-        <v>787</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="13"/>
-      <c r="B10" s="10" t="s">
-        <v>170</v>
-      </c>
-      <c r="C10" t="s">
-        <v>181</v>
-      </c>
-      <c r="D10">
-        <v>125</v>
-      </c>
-      <c r="E10">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="13"/>
-      <c r="B11" s="10"/>
-      <c r="C11" t="s">
-        <v>171</v>
-      </c>
-      <c r="D11">
-        <v>295</v>
-      </c>
-      <c r="E11">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="13"/>
-      <c r="B12" s="10" t="s">
-        <v>179</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="D13">
+        <v>2332</v>
+      </c>
+      <c r="E13">
+        <v>2324</v>
+      </c>
+      <c r="F13">
+        <v>2259</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="14"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="D14">
+        <v>507</v>
+      </c>
+      <c r="E14">
+        <v>508</v>
+      </c>
+      <c r="F14">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="14"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="D15">
+        <v>855</v>
+      </c>
+      <c r="E15">
+        <v>829</v>
+      </c>
+      <c r="F15">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="14"/>
+      <c r="B16" t="s">
+        <v>185</v>
+      </c>
+      <c r="C16" t="s">
         <v>168</v>
       </c>
-      <c r="D12">
-        <v>1364</v>
-      </c>
-      <c r="E12">
-        <v>1367</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="13"/>
-      <c r="B13" s="10"/>
-      <c r="C13" t="s">
-        <v>180</v>
-      </c>
-      <c r="D13">
-        <v>178</v>
-      </c>
-      <c r="E13">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="13"/>
-      <c r="B14" s="10" t="s">
-        <v>182</v>
-      </c>
-      <c r="C14" t="s">
-        <v>168</v>
-      </c>
-      <c r="D14">
-        <v>2332</v>
-      </c>
-      <c r="E14">
-        <v>2324</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="13"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="12" t="s">
-        <v>183</v>
-      </c>
-      <c r="D15">
-        <v>507</v>
-      </c>
-      <c r="E15">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" s="13"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="12" t="s">
-        <v>184</v>
-      </c>
       <c r="D16">
-        <v>855</v>
+        <v>678</v>
       </c>
       <c r="E16">
-        <v>829</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="13"/>
-      <c r="B17" t="s">
-        <v>185</v>
-      </c>
-      <c r="C17" t="s">
-        <v>168</v>
+        <v>667</v>
+      </c>
+      <c r="F16">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="17" spans="3:6">
+      <c r="C17" s="10" t="s">
+        <v>186</v>
       </c>
       <c r="D17">
-        <v>678</v>
+        <f>SUM(D2:D16)</f>
+        <v>11722</v>
       </c>
       <c r="E17">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="C18" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="D18">
-        <f>SUM(D3:D17)</f>
-        <v>11722</v>
-      </c>
+        <f>SUM(E2:E16)</f>
+        <v>11651</v>
+      </c>
+      <c r="F17">
+        <f>SUM(F2:F16)</f>
+        <v>11421</v>
+      </c>
+    </row>
+    <row r="18" spans="3:6">
       <c r="E18">
-        <f>SUM(E3:E17)</f>
-        <v>11651</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="E19">
-        <f>E18-D18</f>
+        <f>E17-D17</f>
         <v>-71</v>
       </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="E20" s="6">
-        <f>E19/D18</f>
+      <c r="F18">
+        <f>F17-E17</f>
+        <v>-230</v>
+      </c>
+    </row>
+    <row r="19" spans="3:6">
+      <c r="E19" s="6">
+        <f>E18/D17</f>
         <v>-6.0569868623101862E-3</v>
+      </c>
+      <c r="F19" s="6">
+        <f>F18/E17</f>
+        <v>-1.9740794781563813E-2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A7:A17"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="A6:A16"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B11:B12"/>
   </mergeCells>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1998,7 +2096,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2033,51 +2131,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" s="1" customFormat="1">
-      <c r="D1" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9" t="s">
+      <c r="D1" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9" t="s">
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9" t="s">
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9"/>
-      <c r="P1" s="9" t="s">
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
-      <c r="S1" s="9" t="s">
+      <c r="Q1" s="11"/>
+      <c r="R1" s="11"/>
+      <c r="S1" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="T1" s="9"/>
-      <c r="U1" s="9"/>
-      <c r="V1" s="9" t="s">
+      <c r="T1" s="11"/>
+      <c r="U1" s="11"/>
+      <c r="V1" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="W1" s="9"/>
-      <c r="X1" s="9"/>
-      <c r="Y1" s="9" t="s">
+      <c r="W1" s="11"/>
+      <c r="X1" s="11"/>
+      <c r="Y1" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="Z1" s="9"/>
-      <c r="AA1" s="9"/>
-      <c r="AB1" s="9" t="s">
+      <c r="Z1" s="11"/>
+      <c r="AA1" s="11"/>
+      <c r="AB1" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="AC1" s="9"/>
-      <c r="AD1" s="9"/>
+      <c r="AC1" s="11"/>
+      <c r="AD1" s="11"/>
     </row>
     <row r="2" spans="1:30" s="1" customFormat="1">
       <c r="A2" s="1" t="s">
@@ -2172,10 +2270,10 @@
       </c>
     </row>
     <row r="3" spans="1:30">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="13" t="s">
         <v>41</v>
       </c>
       <c r="C3" t="s">
@@ -2264,8 +2362,8 @@
       </c>
     </row>
     <row r="4" spans="1:30">
-      <c r="A4" s="11"/>
-      <c r="B4" s="10"/>
+      <c r="A4" s="12"/>
+      <c r="B4" s="13"/>
       <c r="C4" t="s">
         <v>113</v>
       </c>
@@ -2280,8 +2378,8 @@
       </c>
     </row>
     <row r="5" spans="1:30">
-      <c r="A5" s="11"/>
-      <c r="B5" s="10"/>
+      <c r="A5" s="12"/>
+      <c r="B5" s="13"/>
       <c r="C5" t="s">
         <v>43</v>
       </c>
@@ -2368,8 +2466,8 @@
       </c>
     </row>
     <row r="6" spans="1:30">
-      <c r="A6" s="11"/>
-      <c r="B6" s="10"/>
+      <c r="A6" s="12"/>
+      <c r="B6" s="13"/>
       <c r="C6" t="s">
         <v>114</v>
       </c>
@@ -2384,7 +2482,7 @@
       </c>
     </row>
     <row r="7" spans="1:30">
-      <c r="A7" s="11"/>
+      <c r="A7" s="12"/>
       <c r="B7" s="5" t="s">
         <v>115</v>
       </c>
@@ -2399,8 +2497,8 @@
       </c>
     </row>
     <row r="8" spans="1:30">
-      <c r="A8" s="11"/>
-      <c r="B8" s="10" t="s">
+      <c r="A8" s="12"/>
+      <c r="B8" s="13" t="s">
         <v>116</v>
       </c>
       <c r="C8" t="s">
@@ -2417,8 +2515,8 @@
       </c>
     </row>
     <row r="9" spans="1:30">
-      <c r="A9" s="11"/>
-      <c r="B9" s="10"/>
+      <c r="A9" s="12"/>
+      <c r="B9" s="13"/>
       <c r="C9" t="s">
         <v>118</v>
       </c>
@@ -2433,8 +2531,8 @@
       </c>
     </row>
     <row r="10" spans="1:30">
-      <c r="A10" s="11"/>
-      <c r="B10" s="10" t="s">
+      <c r="A10" s="12"/>
+      <c r="B10" s="13" t="s">
         <v>104</v>
       </c>
       <c r="C10" t="s">
@@ -2451,8 +2549,8 @@
       </c>
     </row>
     <row r="11" spans="1:30">
-      <c r="A11" s="11"/>
-      <c r="B11" s="10"/>
+      <c r="A11" s="12"/>
+      <c r="B11" s="13"/>
       <c r="C11" t="s">
         <v>114</v>
       </c>
@@ -2467,10 +2565,10 @@
       </c>
     </row>
     <row r="12" spans="1:30">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="13" t="s">
         <v>41</v>
       </c>
       <c r="C12" s="4" t="s">
@@ -2505,8 +2603,8 @@
       </c>
     </row>
     <row r="13" spans="1:30">
-      <c r="A13" s="11"/>
-      <c r="B13" s="10"/>
+      <c r="A13" s="12"/>
+      <c r="B13" s="13"/>
       <c r="C13" t="s">
         <v>42</v>
       </c>
@@ -2593,8 +2691,8 @@
       </c>
     </row>
     <row r="14" spans="1:30">
-      <c r="A14" s="11"/>
-      <c r="B14" s="10"/>
+      <c r="A14" s="12"/>
+      <c r="B14" s="13"/>
       <c r="C14" s="4" t="s">
         <v>105</v>
       </c>
@@ -2627,8 +2725,8 @@
       </c>
     </row>
     <row r="15" spans="1:30">
-      <c r="A15" s="11"/>
-      <c r="B15" s="10"/>
+      <c r="A15" s="12"/>
+      <c r="B15" s="13"/>
       <c r="C15" t="s">
         <v>43</v>
       </c>
@@ -2715,8 +2813,8 @@
       </c>
     </row>
     <row r="16" spans="1:30">
-      <c r="A16" s="11"/>
-      <c r="B16" s="10" t="s">
+      <c r="A16" s="12"/>
+      <c r="B16" s="13" t="s">
         <v>103</v>
       </c>
       <c r="C16" t="s">
@@ -2751,8 +2849,8 @@
       </c>
     </row>
     <row r="17" spans="1:30">
-      <c r="A17" s="11"/>
-      <c r="B17" s="10"/>
+      <c r="A17" s="12"/>
+      <c r="B17" s="13"/>
       <c r="C17" t="s">
         <v>109</v>
       </c>
@@ -2785,8 +2883,8 @@
       </c>
     </row>
     <row r="18" spans="1:30">
-      <c r="A18" s="11"/>
-      <c r="B18" s="10" t="s">
+      <c r="A18" s="12"/>
+      <c r="B18" s="13" t="s">
         <v>104</v>
       </c>
       <c r="C18" t="s">
@@ -2821,8 +2919,8 @@
       </c>
     </row>
     <row r="19" spans="1:30">
-      <c r="A19" s="11"/>
-      <c r="B19" s="10"/>
+      <c r="A19" s="12"/>
+      <c r="B19" s="13"/>
       <c r="C19" t="s">
         <v>109</v>
       </c>
@@ -2978,9 +3076,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B3:B6"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B10:B11"/>
     <mergeCell ref="AB1:AD1"/>
     <mergeCell ref="Y1:AA1"/>
     <mergeCell ref="A12:A19"/>
@@ -2995,8 +3090,11 @@
     <mergeCell ref="P1:R1"/>
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="B18:B19"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B10:B11"/>
   </mergeCells>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
 </worksheet>
@@ -3018,16 +3116,16 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1"/>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9" t="s">
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
@@ -3383,31 +3481,31 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" s="1"/>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9" t="s">
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9" t="s">
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9" t="s">
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9" t="s">
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="O1" s="9"/>
-      <c r="P1" s="9"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11"/>
     </row>
     <row r="2" spans="1:16">
       <c r="A2" s="1" t="s">
@@ -3664,21 +3762,21 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="1"/>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9" t="s">
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9" t="s">
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
@@ -4653,54 +4751,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" s="1" customFormat="1">
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9" t="s">
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9" t="s">
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9" t="s">
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
-      <c r="S1" s="9" t="s">
+      <c r="P1" s="11"/>
+      <c r="Q1" s="11"/>
+      <c r="R1" s="11"/>
+      <c r="S1" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="T1" s="9"/>
-      <c r="U1" s="9"/>
-      <c r="V1" s="9"/>
-      <c r="W1" s="9" t="s">
+      <c r="T1" s="11"/>
+      <c r="U1" s="11"/>
+      <c r="V1" s="11"/>
+      <c r="W1" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="X1" s="9"/>
-      <c r="Y1" s="9"/>
-      <c r="Z1" s="9"/>
-      <c r="AA1" s="9" t="s">
+      <c r="X1" s="11"/>
+      <c r="Y1" s="11"/>
+      <c r="Z1" s="11"/>
+      <c r="AA1" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="AB1" s="9"/>
-      <c r="AC1" s="9"/>
-      <c r="AD1" s="9"/>
-      <c r="AE1" s="9" t="s">
+      <c r="AB1" s="11"/>
+      <c r="AC1" s="11"/>
+      <c r="AD1" s="11"/>
+      <c r="AE1" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="AF1" s="9"/>
-      <c r="AG1" s="9"/>
-      <c r="AH1" s="9"/>
+      <c r="AF1" s="11"/>
+      <c r="AG1" s="11"/>
+      <c r="AH1" s="11"/>
     </row>
     <row r="2" spans="1:34" s="1" customFormat="1">
       <c r="A2" s="1" t="s">
@@ -5508,13 +5606,13 @@
       <c r="A1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
       <c r="H1" s="1" t="s">
         <v>146</v>
       </c>

</xml_diff>